<commit_message>
refactor: 单轨化批6——API 收编+管线加固:/api/v1/v2→/api/v1(57 路由零冲突);条件解析器收敛(后端 3→1:运行期 condition_matches 补 list 分支成唯一实现、生成物改 import;前端 unknown-op 改 console.error+false、解析失败兜底两端统一为条件不成立);docs/standard/condition-cases.json 16 例跨语言 fixture(pytest+vitest 双端同源断言);check_field_source 补四护栏(condition.field 可解析/op 白名单/in 必 list/下拉词表非空,现有 YAML 零违例);VISIBILITY_GATED_KEYS 编入 YAML ui.visibility_gated×3+生成器透传+前端数据驱动(Codex gpt-5.6-sol 初稿+Fable 验收)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/standard/字段草案-v3.xlsx
+++ b/docs/standard/字段草案-v3.xlsx
@@ -36,14 +36,25 @@
     <font>
       <b val="1"/>
       <color rgb="001F4E79"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00C00000"/>
     </font>
     <font>
+      <color rgb="00C00000"/>
+    </font>
+    <font>
+      <color rgb="00806000"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00B26B00"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
     </font>
     <font>
       <b val="1"/>
@@ -56,17 +67,6 @@
     <font>
       <color rgb="00666666"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001F4E79"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <color rgb="00C00000"/>
-    </font>
-    <font>
-      <color rgb="00806000"/>
     </font>
   </fonts>
   <fills count="9">
@@ -83,7 +83,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FCE4E4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF7DA"/>
       </patternFill>
     </fill>
     <fill>
@@ -93,22 +103,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF7DA"/>
+        <fgColor rgb="00E4ECF7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E4ECF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D6E4F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -143,49 +143,49 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>

</xml_diff>

<commit_message>
feat: add run search audit and exports
</commit_message>
<xml_diff>
--- a/docs/standard/字段草案-v3.xlsx
+++ b/docs/standard/字段草案-v3.xlsx
@@ -836,7 +836,7 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>样品/实验编号</t>
+          <t>炉次编号</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
@@ -866,7 +866,7 @@
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>CVD-20260620-03</t>
+          <t>CVD-2026-0003</t>
         </is>
       </c>
       <c r="I7" s="11" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>组成明细(components)</t>
+          <t>组成明细</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="F19" s="11" t="inlineStr">
         <is>
-          <t>视性能</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G19" s="14" t="inlineStr">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="F41" s="11" t="inlineStr">
         <is>
-          <t>见展开</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G41" s="15" t="inlineStr">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="F51" s="11" t="inlineStr">
         <is>
-          <t>见展开</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G51" s="15" t="inlineStr">
@@ -4040,7 +4040,7 @@
       </c>
       <c r="F75" s="11" t="inlineStr">
         <is>
-          <t>视仪器</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G75" s="15" t="inlineStr">
@@ -7001,7 +7001,7 @@
       </c>
       <c r="F50" s="11" t="inlineStr">
         <is>
-          <t>视仪器</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G50" s="14" t="inlineStr">

</xml_diff>

<commit_message>
feat: refine target product entry
</commit_message>
<xml_diff>
--- a/docs/standard/字段草案-v3.xlsx
+++ b/docs/standard/字段草案-v3.xlsx
@@ -1121,7 +1121,7 @@
       </c>
       <c r="J12" s="13" t="inlineStr">
         <is>
-          <t>★R0；复合体系权威在『组成明细』；录入使用普通数字；允许常见圆括号、组成分组与结晶水点号</t>
+          <t>★R0；复合体系权威在『组成明细』；系统静默归一化粘贴的下标数字；允许常见圆括号、组成分组与结晶水点号</t>
         </is>
       </c>
       <c r="K12" s="11" t="inlineStr"/>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>按结构类型记录主体与掺杂元素、合金混合位点，或异质结构的材料层与区域</t>
+          <t>按结构类型记录掺杂元素、合金混合位点，或异质结构的材料层与区域；掺杂主体直接取上方主体材料化学式</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>每条:化学式/角色(主体材料·掺杂剂·合金组分·材料层·上层·下层·横向域)/名义含量或占位比例(%)/层序(整数)/体相空间群(1-230)</t>
+          <t>掺杂=掺杂元素+名义含量；合金=混合占位元素+占位比例；垂直异质结=材料层+层序+体相空间群；横向异质结=材料区域+体相空间群；其他=组成材料+适用属性；机器角色(主体材料·掺杂剂·合金组分·材料层·上层·下层·横向域)</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="J14" s="11" t="inlineStr">
         <is>
-          <t>掺杂记录一条主体材料和一个或多个掺杂元素；合金组分只表示混合占位元素及比例；垂直结构按从衬底向上顺序记录材料层，横向结构逐区域记录；上层/下层只用于历史兼容</t>
+          <t>掺杂界面只填一个或多个掺杂元素，保存时由主体材料化学式自动加入主体记录；合金组分只表示混合占位元素及比例；垂直结构按从衬底向上顺序记录材料层，横向结构逐区域记录；上层/下层只用于历史兼容</t>
         </is>
       </c>
       <c r="K14" s="11" t="inlineStr"/>
@@ -1240,12 +1240,12 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>目标层数</t>
+          <t>目标原子层数</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>期望层数</t>
+          <t>单一材料体系期望的原子层数；异质结构按材料层或区域记录，不显示本全局字段</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>体相空间群</t>
+          <t>目标体相空间群</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
@@ -1320,9 +1320,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G16" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>推荐</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="J16" s="11" t="inlineStr">
         <is>
-          <t>本征、掺杂、合金和其他结构可选；垂直或横向异质结构在组成明细逐层或逐区域填写</t>
+          <t>本征、掺杂、合金和其他结构推荐填写；垂直或横向异质结构在组成明细逐层或逐区域填写；常见体相候选仅作快速录入，不自动判定物相</t>
         </is>
       </c>
       <c r="K16" s="11" t="inlineStr"/>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>样品形态</t>
+          <t>目标形态</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
@@ -8202,7 +8202,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -9394,28 +9394,50 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="11" t="inlineStr"/>
-      <c r="B58" s="11" t="inlineStr"/>
-      <c r="C58" s="11" t="inlineStr"/>
-      <c r="D58" s="11" t="inlineStr"/>
+      <c r="A58" s="11" t="inlineStr">
+        <is>
+          <t>v3.13</t>
+        </is>
+      </c>
+      <c r="B58" s="11" t="inlineStr">
+        <is>
+          <t>§1b</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>目标产物复核：化学式示例按结构类型变化；删除“普通数字”用户文案；掺杂区只显示掺杂元素；空间群按化学式给出经核对的常见体相候选并保留230项搜索；异质结构逐层或逐区域填写空间群</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-28用户逐项复核</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="11" t="inlineStr">
+      <c r="A59" s="11" t="inlineStr"/>
+      <c r="B59" s="11" t="inlineStr"/>
+      <c r="C59" s="11" t="inlineStr"/>
+      <c r="D59" s="11" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
         <is>
           <t>R0</t>
         </is>
       </c>
-      <c r="B59" s="11" t="inlineStr">
+      <c r="B60" s="11" t="inlineStr">
         <is>
           <t>硬必填核心(30项，含条件必填)</t>
         </is>
       </c>
-      <c r="C59" s="11" t="inlineStr">
+      <c r="C60" s="11" t="inlineStr">
         <is>
           <t>v3.7新增环境温湿度、预检、目标形态、Setup测温传感器、前驱体与衬底批次、衬底化学式/晶向/粗糙度/尺寸放置、预处理操作；过程R0改为结构化温度程序、逐气体供气、绝对压力及反应时长</t>
         </is>
       </c>
-      <c r="D59" s="11" t="inlineStr">
+      <c r="D60" s="11" t="inlineStr">
         <is>
           <t>必填集</t>
         </is>

</xml_diff>

<commit_message>
[frontend] refine target product entry (#6)
* feat: refine target product entry

* test: keep target product checks focused
</commit_message>
<xml_diff>
--- a/docs/standard/字段草案-v3.xlsx
+++ b/docs/standard/字段草案-v3.xlsx
@@ -1121,7 +1121,7 @@
       </c>
       <c r="J12" s="13" t="inlineStr">
         <is>
-          <t>★R0；复合体系权威在『组成明细』；录入使用普通数字；允许常见圆括号、组成分组与结晶水点号</t>
+          <t>★R0；复合体系权威在『组成明细』；系统静默归一化粘贴的下标数字；允许常见圆括号、组成分组与结晶水点号</t>
         </is>
       </c>
       <c r="K12" s="11" t="inlineStr"/>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>按结构类型记录主体与掺杂元素、合金混合位点，或异质结构的材料层与区域</t>
+          <t>按结构类型记录掺杂元素、合金混合位点，或异质结构的材料层与区域；掺杂主体直接取上方主体材料化学式</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>每条:化学式/角色(主体材料·掺杂剂·合金组分·材料层·上层·下层·横向域)/名义含量或占位比例(%)/层序(整数)/体相空间群(1-230)</t>
+          <t>掺杂=掺杂元素+名义含量；合金=混合占位元素+占位比例；垂直异质结=材料层+层序+体相空间群；横向异质结=材料区域+体相空间群；其他=组成材料+适用属性；机器角色(主体材料·掺杂剂·合金组分·材料层·上层·下层·横向域)</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="J14" s="11" t="inlineStr">
         <is>
-          <t>掺杂记录一条主体材料和一个或多个掺杂元素；合金组分只表示混合占位元素及比例；垂直结构按从衬底向上顺序记录材料层，横向结构逐区域记录；上层/下层只用于历史兼容</t>
+          <t>掺杂界面只填一个或多个掺杂元素，保存时由主体材料化学式自动加入主体记录；合金组分只表示混合占位元素及比例；垂直结构按从衬底向上顺序记录材料层，横向结构逐区域记录；上层/下层只用于历史兼容</t>
         </is>
       </c>
       <c r="K14" s="11" t="inlineStr"/>
@@ -1240,12 +1240,12 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>目标层数</t>
+          <t>目标原子层数</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>期望层数</t>
+          <t>单一材料体系期望的原子层数；异质结构按材料层或区域记录，不显示本全局字段</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>体相空间群</t>
+          <t>目标体相空间群</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
@@ -1320,9 +1320,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G16" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>推荐</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="J16" s="11" t="inlineStr">
         <is>
-          <t>本征、掺杂、合金和其他结构可选；垂直或横向异质结构在组成明细逐层或逐区域填写</t>
+          <t>本征、掺杂、合金和其他结构推荐填写；垂直或横向异质结构在组成明细逐层或逐区域填写；常见体相候选仅作快速录入，不自动判定物相</t>
         </is>
       </c>
       <c r="K16" s="11" t="inlineStr"/>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>样品形态</t>
+          <t>目标形态</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
@@ -8202,7 +8202,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -9394,28 +9394,50 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="11" t="inlineStr"/>
-      <c r="B58" s="11" t="inlineStr"/>
-      <c r="C58" s="11" t="inlineStr"/>
-      <c r="D58" s="11" t="inlineStr"/>
+      <c r="A58" s="11" t="inlineStr">
+        <is>
+          <t>v3.13</t>
+        </is>
+      </c>
+      <c r="B58" s="11" t="inlineStr">
+        <is>
+          <t>§1b</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>目标产物复核：化学式示例按结构类型变化；删除“普通数字”用户文案；掺杂区只显示掺杂元素；空间群按化学式给出经核对的常见体相候选并保留230项搜索；异质结构逐层或逐区域填写空间群</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-28用户逐项复核</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="11" t="inlineStr">
+      <c r="A59" s="11" t="inlineStr"/>
+      <c r="B59" s="11" t="inlineStr"/>
+      <c r="C59" s="11" t="inlineStr"/>
+      <c r="D59" s="11" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
         <is>
           <t>R0</t>
         </is>
       </c>
-      <c r="B59" s="11" t="inlineStr">
+      <c r="B60" s="11" t="inlineStr">
         <is>
           <t>硬必填核心(30项，含条件必填)</t>
         </is>
       </c>
-      <c r="C59" s="11" t="inlineStr">
+      <c r="C60" s="11" t="inlineStr">
         <is>
           <t>v3.7新增环境温湿度、预检、目标形态、Setup测温传感器、前驱体与衬底批次、衬底化学式/晶向/粗糙度/尺寸放置、预处理操作；过程R0改为结构化温度程序、逐气体供气、绝对压力及反应时长</t>
         </is>
       </c>
-      <c r="D59" s="11" t="inlineStr">
+      <c r="D60" s="11" t="inlineStr">
         <is>
           <t>必填集</t>
         </is>

</xml_diff>

<commit_message>
fix: align experimental setup workflow
</commit_message>
<xml_diff>
--- a/docs/standard/字段草案-v3.xlsx
+++ b/docs/standard/字段草案-v3.xlsx
@@ -1522,7 +1522,7 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>装置（引用）</t>
+          <t>实验装置</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
@@ -2090,7 +2090,7 @@
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>当前炉管的累计重置次数，以及本次实验是最近一次重置后的第几次使用</t>
+          <t>当前炉管的累计清洗或更换次数，以及本次实验是最近一次清洗或更换后的第几次使用</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="J32" s="11" t="inlineStr">
         <is>
-          <t>每炉手填；清洗或更换炉管后重置次数加1，本次使用序号从1重新累计</t>
+          <t>每炉手填；清洗或更换炉管后累计次数加1，本次使用序号从1重新累计</t>
         </is>
       </c>
       <c r="K32" s="11" t="inlineStr"/>
@@ -7166,12 +7166,12 @@
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>下拉+其他</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>受控+其他</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F33" s="11" t="inlineStr">
@@ -7258,46 +7258,50 @@
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>壁型</t>
+          <t>温区数</t>
         </is>
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>热壁/冷壁</t>
+          <t>独立控温区数</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>下拉</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="E35" s="11" t="inlineStr">
         <is>
-          <t>热壁/冷壁</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F35" s="11" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G35" s="15" t="inlineStr">
-        <is>
-          <t>推荐</t>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
         </is>
       </c>
       <c r="H35" s="11" t="inlineStr">
         <is>
-          <t>热壁</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I35" s="11" t="inlineStr">
         <is>
-          <t>复审</t>
+          <t>会议</t>
         </is>
       </c>
       <c r="J35" s="11" t="inlineStr"/>
-      <c r="K35" s="11" t="inlineStr"/>
+      <c r="K35" s="11" t="inlineStr">
+        <is>
+          <t>{"ge":1,"type":"integer"}</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
@@ -7307,27 +7311,27 @@
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>温区数</t>
+          <t>各温区温度传感器</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>独立控温区数</t>
+          <t>装置每个温区的传感器类型和用户可直接理解的温度测量误差</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>温度传感器数组</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>{sensor_type: k_thermocouple|s_thermocouple|r_thermocouple|b_thermocouple|infrared_pyrometer|other, sensor_type_other?, zone_index, uncertainty_C；旧记录可含sensor_name与uncertainty_source}</t>
         </is>
       </c>
       <c r="F36" s="11" t="inlineStr">
         <is>
-          <t>个</t>
+          <t>℃</t>
         </is>
       </c>
       <c r="G36" s="12" t="inlineStr">
@@ -7337,20 +7341,20 @@
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>[{sensor_type: K型热电偶, zone_index: 1, uncertainty_C: 1}]</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>会议</t>
-        </is>
-      </c>
-      <c r="J36" s="11" t="inlineStr"/>
-      <c r="K36" s="11" t="inlineStr">
-        <is>
-          <t>{"ge":1,"type":"integer"}</t>
-        </is>
-      </c>
+          <t>2026-07-24导师走查·2026-07-27终版整改</t>
+        </is>
+      </c>
+      <c r="J36" s="11" t="inlineStr">
+        <is>
+          <t>温区数决定卡片数量；不让用户另起传感器名称，不要求填写难以理解的误差来源；旧字段只读兼容</t>
+        </is>
+      </c>
+      <c r="K36" s="11" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
@@ -7360,27 +7364,27 @@
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>各温区温度传感器</t>
+          <t>炉体方向</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>装置每个温区的传感器类型和用户可直接理解的温度测量误差</t>
+          <t>水平/垂直</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>温度传感器数组</t>
+          <t>下拉</t>
         </is>
       </c>
       <c r="E37" s="11" t="inlineStr">
         <is>
-          <t>{sensor_type, zone_index, uncertainty_C；旧记录可含sensor_name与uncertainty_source}</t>
+          <t>水平/垂直</t>
         </is>
       </c>
       <c r="F37" s="11" t="inlineStr">
         <is>
-          <t>℃</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G37" s="12" t="inlineStr">
@@ -7390,19 +7394,15 @@
       </c>
       <c r="H37" s="11" t="inlineStr">
         <is>
-          <t>[{sensor_type: K型热电偶, zone_index: 1, uncertainty_C: 1}]</t>
+          <t>水平</t>
         </is>
       </c>
       <c r="I37" s="11" t="inlineStr">
         <is>
-          <t>2026-07-24导师走查·2026-07-27终版整改</t>
-        </is>
-      </c>
-      <c r="J37" s="11" t="inlineStr">
-        <is>
-          <t>温区数决定卡片数量；不让用户另起传感器名称，不要求填写难以理解的误差来源；旧字段只读兼容</t>
-        </is>
-      </c>
+          <t>会议</t>
+        </is>
+      </c>
+      <c r="J37" s="11" t="inlineStr"/>
       <c r="K37" s="11" t="inlineStr"/>
     </row>
     <row r="38">
@@ -7413,22 +7413,22 @@
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>炉体方向</t>
+          <t>炉管材质与截面</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>水平/垂直</t>
+          <t>炉管材料与截面</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>下拉</t>
+          <t>管材质形状对象</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>水平/垂直</t>
+          <t>{material: 石英|刚玉|其他, material_other?, shape: 圆形|方形|矩形|其他, shape_other?}</t>
         </is>
       </c>
       <c r="F38" s="11" t="inlineStr">
@@ -7443,15 +7443,19 @@
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>水平</t>
+          <t>{material: 石英, shape: 圆形}</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>会议</t>
-        </is>
-      </c>
-      <c r="J38" s="11" t="inlineStr"/>
+          <t>2026-07-24导师走查</t>
+        </is>
+      </c>
+      <c r="J38" s="11" t="inlineStr">
+        <is>
+          <t>材质与截面形状独立保存，禁止把“刚玉；圆”当作一个选项</t>
+        </is>
+      </c>
       <c r="K38" s="11" t="inlineStr"/>
     </row>
     <row r="39">
@@ -7462,47 +7466,47 @@
       </c>
       <c r="B39" s="11" t="inlineStr">
         <is>
-          <t>炉管材质与截面</t>
+          <t>炉管尺寸</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>炉管材料与截面</t>
+          <t>按截面形状记录外部尺寸和壁厚</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>管材质形状对象</t>
+          <t>炉管尺寸对象</t>
         </is>
       </c>
       <c r="E39" s="11" t="inlineStr">
         <is>
-          <t>{material: 石英|刚玉|其他, material_other?, shape: 圆形|方形|矩形|其他, shape_other?}</t>
+          <t>{圆形: outer_diameter_mm+wall_thickness_mm; 方形: outer_side_mm+wall_thickness_mm; 矩形: outer_width_mm+outer_height_mm+wall_thickness_mm; 其他: dimension_description}</t>
         </is>
       </c>
       <c r="F39" s="11" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G39" s="15" t="inlineStr">
-        <is>
-          <t>推荐</t>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="G39" s="12" t="inlineStr">
+        <is>
+          <t>必填；按炉管截面填写</t>
         </is>
       </c>
       <c r="H39" s="11" t="inlineStr">
         <is>
-          <t>{material: 石英, shape: 圆形}</t>
+          <t>{outer_width_mm: 50, outer_height_mm: 30, wall_thickness_mm: 2}</t>
         </is>
       </c>
       <c r="I39" s="11" t="inlineStr">
         <is>
-          <t>2026-07-24导师走查</t>
+          <t>会议·用户复核2026-07-24</t>
         </is>
       </c>
       <c r="J39" s="11" t="inlineStr">
         <is>
-          <t>材质与截面形状独立保存，禁止把“刚玉；圆”当作一个选项</t>
+          <t>选择材质与截面后必须按形状完整填写；圆形填外径+壁厚，方形填外边长+壁厚，矩形填外宽+外高+壁厚，其他截面填写具名尺寸说明</t>
         </is>
       </c>
       <c r="K39" s="11" t="inlineStr"/>
@@ -7515,47 +7519,47 @@
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>炉管尺寸</t>
+          <t>壁型</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>按截面形状记录外部尺寸和壁厚</t>
+          <t>热壁/冷壁</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>炉管尺寸对象</t>
+          <t>下拉</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
         <is>
-          <t>{圆形: outer_diameter_mm+wall_thickness_mm; 方形: outer_side_mm+wall_thickness_mm; 矩形: outer_width_mm+outer_height_mm+wall_thickness_mm; 其他: dimension_description}</t>
+          <t>热壁/冷壁</t>
         </is>
       </c>
       <c r="F40" s="11" t="inlineStr">
         <is>
-          <t>mm</t>
-        </is>
-      </c>
-      <c r="G40" s="16" t="inlineStr">
-        <is>
-          <t>选择炉管材质与截面后必填</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G40" s="15" t="inlineStr">
+        <is>
+          <t>推荐</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>{outer_width_mm: 50, outer_height_mm: 30, wall_thickness_mm: 2}</t>
+          <t>热壁</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>会议·用户复核2026-07-24</t>
+          <t>复审</t>
         </is>
       </c>
       <c r="J40" s="11" t="inlineStr">
         <is>
-          <t>选择材质与截面后必须按形状完整填写；圆形填外径+壁厚，方形填外边长+壁厚，矩形填外宽+外高+壁厚，其他截面填写具名尺寸说明</t>
+          <t>放在装置身份、温区与炉管结构之后，避免打断由粗到细的登记顺序</t>
         </is>
       </c>
       <c r="K40" s="11" t="inlineStr"/>
@@ -7644,9 +7648,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G42" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
+      <c r="G42" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">

</xml_diff>

<commit_message>
feat: implement scientific v4 audit remediation
</commit_message>
<xml_diff>
--- a/docs/standard/字段草案-v3.xlsx
+++ b/docs/standard/字段草案-v3.xlsx
@@ -757,7 +757,7 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>CVD/APCVD/LPCVD/PECVD/MOCVD/盐辅助CVD/PVD-磁控溅射/PVD-热蒸发/PLD</t>
+          <t>CVD</t>
         </is>
       </c>
       <c r="F5" s="11" t="inlineStr">
@@ -782,7 +782,7 @@
       </c>
       <c r="J5" s="11" t="inlineStr">
         <is>
-          <t>新记录固定为CVD；历史APCVD/LPCVD/PECVD/MOCVD/盐辅助CVD值继续兼容读取</t>
+          <t>新记录固定为CVD；压力、等离子体、金属有机源和盐辅助均在正交事实字段中表达；PVD未发布</t>
         </is>
       </c>
       <c r="K5" s="11" t="inlineStr"/>
@@ -4867,7 +4867,7 @@
     <row r="87" ht="20" customHeight="1">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>§7 产物表征 + 实测产物（★独立表，用编号与实验记录关联；只记事实，不判好坏）</t>
+          <t>§7 旧扁平结果字段（未发布；由 MeasurementRun → AnalysisRun → PropertyValue / MaterialAssertion 替代）</t>
         </is>
       </c>
       <c r="B87" s="8" t="n"/>
@@ -4912,9 +4912,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G88" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
+      <c r="G88" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H88" s="11" t="inlineStr">
@@ -4965,9 +4965,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G89" s="15" t="inlineStr">
-        <is>
-          <t>推荐</t>
+      <c r="G89" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H89" s="11" t="inlineStr">
@@ -5018,9 +5018,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G90" s="15" t="inlineStr">
-        <is>
-          <t>推荐</t>
+      <c r="G90" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H90" s="11" t="inlineStr">
@@ -5069,7 +5069,7 @@
       </c>
       <c r="G91" s="16" t="inlineStr">
         <is>
-          <t>选填</t>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H91" s="11" t="inlineStr">
@@ -5122,7 +5122,7 @@
       </c>
       <c r="G92" s="16" t="inlineStr">
         <is>
-          <t>选填</t>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H92" s="11" t="inlineStr">
@@ -5175,7 +5175,7 @@
       </c>
       <c r="G93" s="16" t="inlineStr">
         <is>
-          <t>选填</t>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H93" s="11" t="inlineStr">
@@ -5232,7 +5232,7 @@
       </c>
       <c r="G94" s="16" t="inlineStr">
         <is>
-          <t>选填</t>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H94" s="11" t="inlineStr">
@@ -5289,7 +5289,7 @@
       </c>
       <c r="G95" s="16" t="inlineStr">
         <is>
-          <t>选填</t>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H95" s="11" t="inlineStr">
@@ -5342,7 +5342,7 @@
       </c>
       <c r="G96" s="16" t="inlineStr">
         <is>
-          <t>选填</t>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H96" s="11" t="inlineStr">
@@ -5395,7 +5395,7 @@
       </c>
       <c r="G97" s="16" t="inlineStr">
         <is>
-          <t>选填</t>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H97" s="11" t="inlineStr">
@@ -5467,9 +5467,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G99" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(PVD)</t>
+      <c r="G99" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H99" s="11" t="inlineStr">
@@ -5516,9 +5516,9 @@
           <t>mm</t>
         </is>
       </c>
-      <c r="G100" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(PVD)</t>
+      <c r="G100" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H100" s="11" t="inlineStr">
@@ -5569,9 +5569,9 @@
           <t>W·V</t>
         </is>
       </c>
-      <c r="G101" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(PVD)</t>
+      <c r="G101" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H101" s="11" t="inlineStr">
@@ -5618,9 +5618,9 @@
           <t>Pa</t>
         </is>
       </c>
-      <c r="G102" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(PVD)</t>
+      <c r="G102" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H102" s="11" t="inlineStr">
@@ -5671,9 +5671,9 @@
           <t>min·s</t>
         </is>
       </c>
-      <c r="G103" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(PVD)</t>
+      <c r="G103" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H103" s="11" t="inlineStr">
@@ -5724,9 +5724,9 @@
           <t>nm/s</t>
         </is>
       </c>
-      <c r="G104" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(PVD)</t>
+      <c r="G104" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H104" s="11" t="inlineStr">
@@ -5768,7 +5768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K58"/>
+  <dimension ref="A1:K71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6140,22 +6140,22 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>供应商</t>
+          <t>物质同义名</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>商业批次：厂商</t>
+          <t>用于检索的稳定同义名，不替代标签名称</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>下拉+其他(可扩展)</t>
+          <t>文本数组</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>受控+其他</t>
+          <t>JSON字符串数组</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
@@ -6163,22 +6163,26 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G9" s="15" t="inlineStr">
-        <is>
-          <t>推荐</t>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>阿拉丁</t>
+          <t>["Molybdenum trioxide"]</t>
         </is>
       </c>
       <c r="I9" s="11" t="inlineStr">
         <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="J9" s="11" t="inlineStr"/>
+          <t>2026-07-28深度审查</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>归一化到Substance实体</t>
+        </is>
+      </c>
       <c r="K9" s="11" t="inlineStr"/>
     </row>
     <row r="10">
@@ -6189,22 +6193,22 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>供应商货号</t>
+          <t>物质标识符</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>商业批次：产品号</t>
+          <t>CAS、InChIKey等标识符及其类型</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>JSON数组</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>[{type,value}]</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
@@ -6219,17 +6223,17 @@
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>M112056</t>
+          <t>[{"type":"CAS","value":"1313-27-5"}]</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>2026-07-28深度审查</t>
         </is>
       </c>
       <c r="J10" s="11" t="inlineStr">
         <is>
-          <t>供应商产品规格编号，标签上常写作 Cat. No.；同一货号可有多个生产批号</t>
+          <t>归一化到Substance实体</t>
         </is>
       </c>
       <c r="K10" s="11" t="inlineStr"/>
@@ -6242,22 +6246,22 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>生产批号</t>
+          <t>供应商</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>商业批次：生产批号（同名不同批的区分键）</t>
+          <t>商业批次：厂商</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>下拉+其他(可扩展)</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>受控+其他</t>
         </is>
       </c>
       <c r="F11" s="11" t="inlineStr">
@@ -6265,14 +6269,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G11" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>推荐</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>B202405</t>
+          <t>阿拉丁</t>
         </is>
       </c>
       <c r="I11" s="11" t="inlineStr">
@@ -6280,11 +6284,7 @@
           <t>review</t>
         </is>
       </c>
-      <c r="J11" s="11" t="inlineStr">
-        <is>
-          <t>GMP法定术语『批号』；标签上常写作 Lot No. 或 Batch No.</t>
-        </is>
-      </c>
+      <c r="J11" s="11" t="inlineStr"/>
       <c r="K11" s="11" t="inlineStr"/>
     </row>
     <row r="12">
@@ -6295,37 +6295,37 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>纯度</t>
+          <t>供应商货号</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>仅存质量百分数；N值由质量百分数派生显示，不作为独立存储值</t>
+          <t>商业批次：产品号</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>质量百分数（N值仅派生显示）</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(化学品或气瓶)</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G12" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>99.995（派生显示4N5）</t>
+          <t>M112056</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
@@ -6335,14 +6335,10 @@
       </c>
       <c r="J12" s="11" t="inlineStr">
         <is>
-          <t>原始证书中的N值或其他纯度表述保留在CoA/附件说明中</t>
-        </is>
-      </c>
-      <c r="K12" s="11" t="inlineStr">
-        <is>
-          <t>{"gt":0,"le":100}</t>
-        </is>
-      </c>
+          <t>供应商产品规格编号，标签上常写作 Cat. No.；同一货号可有多个生产批号</t>
+        </is>
+      </c>
+      <c r="K12" s="11" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
@@ -6352,22 +6348,22 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>形态与性状</t>
+          <t>供应商等级</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>试剂外观</t>
+          <t>供应商给出的产品等级或规格名称</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>下拉+其他</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>粉末/颗粒/块/液体/箔/靶/其他</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
@@ -6382,17 +6378,17 @@
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>粉末</t>
+          <t>ACS reagent</t>
         </is>
       </c>
       <c r="I13" s="11" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>2026-07-28深度审查</t>
         </is>
       </c>
       <c r="J13" s="11" t="inlineStr">
         <is>
-          <t>外观=性状；气瓶不使用粉末/箔/靶等物料形态</t>
+          <t>与实测纯度分开</t>
         </is>
       </c>
       <c r="K13" s="11" t="inlineStr"/>
@@ -6405,54 +6401,50 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>粒径D50</t>
+          <t>商业产品规格</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>供应商或CoA报告的来料中位粒径；影响挥发和成核</t>
+          <t>随货号稳定的商业产品规格</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>JSON对象</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>供应商或CoA报告的D50</t>
+          <t>具名规格键值</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>µm</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G14" s="16" t="inlineStr">
         <is>
-          <t>条件选填(粉末或颗粒)</t>
+          <t>选填</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>{"mesh":"100"}</t>
         </is>
       </c>
       <c r="I14" s="11" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>2026-07-28深度审查</t>
         </is>
       </c>
       <c r="J14" s="11" t="inlineStr">
         <is>
-          <t>仅在来料形态为粉末或颗粒且供应商/CoA有报告时填写；无报告留空，不用目数或猜测值代替</t>
-        </is>
-      </c>
-      <c r="K14" s="11" t="inlineStr">
-        <is>
-          <t>{"gt":0}</t>
-        </is>
-      </c>
+          <t>归一化到CommercialProduct实体</t>
+        </is>
+      </c>
+      <c r="K14" s="11" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
@@ -6462,17 +6454,17 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>开封日期</t>
+          <t>生产批号</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>影响吸潮/氧化</t>
+          <t>商业批次：生产批号（同名不同批的区分键）</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>日期</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
@@ -6485,14 +6477,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G15" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
+      <c r="G15" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>B202405</t>
         </is>
       </c>
       <c r="I15" s="11" t="inlineStr">
@@ -6500,7 +6492,11 @@
           <t>review</t>
         </is>
       </c>
-      <c r="J15" s="11" t="inlineStr"/>
+      <c r="J15" s="11" t="inlineStr">
+        <is>
+          <t>GMP法定术语『批号』；标签上常写作 Lot No. 或 Batch No.</t>
+        </is>
+      </c>
       <c r="K15" s="11" t="inlineStr"/>
     </row>
     <row r="16">
@@ -6511,37 +6507,37 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>存储方式</t>
+          <t>纯度</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>存放条件</t>
+          <t>仅存质量百分数；N值由质量百分数派生显示，不作为独立存储值</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>下拉+其他</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>干燥器/手套箱/常温避光/冷藏/其他</t>
+          <t>质量百分数（N值仅派生显示）</t>
         </is>
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="G16" s="14" t="inlineStr">
+        <is>
+          <t>条件必填(化学品或气瓶)</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>干燥器</t>
+          <t>99.995（派生显示4N5）</t>
         </is>
       </c>
       <c r="I16" s="11" t="inlineStr">
@@ -6551,10 +6547,14 @@
       </c>
       <c r="J16" s="11" t="inlineStr">
         <is>
-          <t>desiccator=干燥器</t>
-        </is>
-      </c>
-      <c r="K16" s="11" t="inlineStr"/>
+          <t>原始证书中的N值或其他纯度表述保留在CoA/附件说明中</t>
+        </is>
+      </c>
+      <c r="K16" s="11" t="inlineStr">
+        <is>
+          <t>{"gt":0,"le":100}</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
@@ -6564,22 +6564,22 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>证书附件(CoA)</t>
+          <t>纯度基准</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>质检证书</t>
+          <t>纯度数值所采用的组成基准</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>FileAsset引用</t>
+          <t>下拉</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>{file_asset_id, sha256}</t>
+          <t>质量分数/原子分数/体积分数</t>
         </is>
       </c>
       <c r="F17" s="11" t="inlineStr">
@@ -6587,22 +6587,26 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G17" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>条件必填(填写纯度时)</t>
         </is>
       </c>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>coa.pdf</t>
+          <t>质量分数</t>
         </is>
       </c>
       <c r="I17" s="11" t="inlineStr">
         <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="J17" s="11" t="inlineStr"/>
+          <t>2026-07-28深度审查</t>
+        </is>
+      </c>
+      <c r="J17" s="11" t="inlineStr">
+        <is>
+          <t>禁止只存没有基准的百分数</t>
+        </is>
+      </c>
       <c r="K17" s="11" t="inlineStr"/>
     </row>
     <row r="18">
@@ -6613,22 +6617,22 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>瓶身或包装标签附件</t>
+          <t>纯度来源</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>试剂瓶身、气瓶或衬底包装标签的原始照片，用于追溯批号与规格</t>
+          <t>纯度数值来自供应商声明还是CoA实测</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>FileAsset引用</t>
+          <t>下拉</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>{file_asset_id, sha256}</t>
+          <t>供应商声明/CoA实测</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -6636,24 +6640,24 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G18" s="15" t="inlineStr">
-        <is>
-          <t>推荐</t>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>条件必填(填写纯度时)</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>bottle-label.jpg</t>
+          <t>CoA实测</t>
         </is>
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>2026-07-24导师走查</t>
+          <t>2026-07-28深度审查</t>
         </is>
       </c>
       <c r="J18" s="11" t="inlineStr">
         <is>
-          <t>与CoA分开；同一物料版本至少上传一次并可预览、下载</t>
+          <t>来源文件仍由CoA附件保存</t>
         </is>
       </c>
       <c r="K18" s="11" t="inlineStr"/>
@@ -6666,12 +6670,12 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>▸衬底·材料</t>
+          <t>形态与性状</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>子类(批次类别=衬底)</t>
+          <t>试剂外观</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
@@ -6681,7 +6685,7 @@
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>SiO₂/Si·蓝宝石(Al₂O₃)·石英·云母·Cu箔·Au箔·h-BN·其他</t>
+          <t>粉末/颗粒/块/液体/箔/靶/其他</t>
         </is>
       </c>
       <c r="F19" s="11" t="inlineStr">
@@ -6689,14 +6693,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G19" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(衬底)</t>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
         </is>
       </c>
       <c r="H19" s="11" t="inlineStr">
         <is>
-          <t>SiO₂/Si</t>
+          <t>粉末</t>
         </is>
       </c>
       <c r="I19" s="11" t="inlineStr">
@@ -6706,7 +6710,7 @@
       </c>
       <c r="J19" s="11" t="inlineStr">
         <is>
-          <t>与§4衬底材料词表一致</t>
+          <t>外观=性状；气瓶不使用粉末/箔/靶等物料形态</t>
         </is>
       </c>
       <c r="K19" s="11" t="inlineStr"/>
@@ -6719,12 +6723,12 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>▸衬底·氧化层厚度</t>
+          <t>粒径D50</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>仅SiO₂/Si</t>
+          <t>供应商或CoA报告的来料中位粒径；影响挥发和成核</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -6734,22 +6738,22 @@
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>供应商或CoA报告的D50</t>
         </is>
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
-          <t>nm</t>
-        </is>
-      </c>
-      <c r="G20" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(SiO₂/Si)</t>
+          <t>µm</t>
+        </is>
+      </c>
+      <c r="G20" s="16" t="inlineStr">
+        <is>
+          <t>条件选填(粉末或颗粒)</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>285</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I20" s="11" t="inlineStr">
@@ -6757,7 +6761,11 @@
           <t>review</t>
         </is>
       </c>
-      <c r="J20" s="11" t="inlineStr"/>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>仅在来料形态为粉末或颗粒且供应商/CoA有报告时填写；无报告留空，不用目数或猜测值代替</t>
+        </is>
+      </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
           <t>{"gt":0}</t>
@@ -6772,22 +6780,22 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>▸衬底·晶向与抛光信息</t>
+          <t>D50测量方法</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>供应商是否提供且该衬底是否适用晶面取向与抛光规格</t>
+          <t>得到D50数值所用的方法</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>下拉</t>
+          <t>下拉+其他</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>有规格数值·供应商未提供·不适用</t>
+          <t>激光衍射/筛分/图像分析/其他</t>
         </is>
       </c>
       <c r="F21" s="11" t="inlineStr">
@@ -6795,24 +6803,24 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G21" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(衬底)</t>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>条件选填(填写D50时)</t>
         </is>
       </c>
       <c r="H21" s="11" t="inlineStr">
         <is>
-          <t>有规格数值</t>
+          <t>激光衍射</t>
         </is>
       </c>
       <c r="I21" s="11" t="inlineStr">
         <is>
-          <t>2026-07-25用户复核</t>
+          <t>2026-07-28深度审查</t>
         </is>
       </c>
       <c r="J21" s="11" t="inlineStr">
         <is>
-          <t>Cu/Au箔等不适用时明确选择不适用；禁止伪填晶向或抛光面</t>
+          <t>未报告时留空，不猜测</t>
         </is>
       </c>
       <c r="K21" s="11" t="inlineStr"/>
@@ -6825,22 +6833,22 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>▸衬底·晶向与抛光</t>
+          <t>D50统计基准</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>取向与抛光面</t>
+          <t>粒径分布按体积、数目或质量统计</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>文本+下拉</t>
+          <t>下拉</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>晶向；单面抛/双面抛</t>
+          <t>体积分数/数目基准/质量基准</t>
         </is>
       </c>
       <c r="F22" s="11" t="inlineStr">
@@ -6848,31 +6856,27 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G22" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(有规格数值)</t>
+      <c r="G22" s="16" t="inlineStr">
+        <is>
+          <t>条件选填(填写D50时)</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>Si(100)；单面抛</t>
+          <t>体积分数</t>
         </is>
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>2026-07-28深度审查</t>
         </is>
       </c>
       <c r="J22" s="11" t="inlineStr">
         <is>
-          <t>实验引用批次后只读带出</t>
-        </is>
-      </c>
-      <c r="K22" s="11" t="inlineStr">
-        <is>
-          <t>{"require_option":true,"require_value":true}</t>
-        </is>
-      </c>
+          <t>与测量方法共同决定可比性</t>
+        </is>
+      </c>
+      <c r="K22" s="11" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
@@ -6882,12 +6886,12 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>▸衬底·偏切信息</t>
+          <t>D50来源</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>供应商是否提供且该衬底是否适用相对标称晶面的偏切规格</t>
+          <t>D50数值的来源</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
@@ -6897,7 +6901,7 @@
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>有规格数值·供应商未提供·不适用</t>
+          <t>供应商声明/CoA实测</t>
         </is>
       </c>
       <c r="F23" s="11" t="inlineStr">
@@ -6905,24 +6909,24 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G23" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(衬底)</t>
+      <c r="G23" s="16" t="inlineStr">
+        <is>
+          <t>条件选填(填写D50时)</t>
         </is>
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>供应商未提供</t>
+          <t>CoA实测</t>
         </is>
       </c>
       <c r="I23" s="11" t="inlineStr">
         <is>
-          <t>2026-07-25用户复核</t>
+          <t>2026-07-28深度审查</t>
         </is>
       </c>
       <c r="J23" s="11" t="inlineStr">
         <is>
-          <t>0仅表示供应商明确报告无偏切，不能表示未知或不适用</t>
+          <t>来源文件仍由CoA附件保存</t>
         </is>
       </c>
       <c r="K23" s="11" t="inlineStr"/>
@@ -6935,17 +6939,17 @@
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>▸衬底·偏切角</t>
+          <t>开封日期</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>实际晶面相对标称晶面的偏切角</t>
+          <t>影响吸潮/氧化</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>日期</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
@@ -6955,34 +6959,26 @@
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>°</t>
-        </is>
-      </c>
-      <c r="G24" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(有规格数值)</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G24" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>2026-07-24用户走查</t>
-        </is>
-      </c>
-      <c r="J24" s="11" t="inlineStr">
-        <is>
-          <t>大于0时必须同时填写substrate_miscut_direction</t>
-        </is>
-      </c>
-      <c r="K24" s="11" t="inlineStr">
-        <is>
-          <t>{"ge":0,"lt":90}</t>
-        </is>
-      </c>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="J24" s="11" t="inlineStr"/>
+      <c r="K24" s="11" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
@@ -6992,22 +6988,22 @@
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>▸衬底·偏切方向</t>
+          <t>存储方式</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>偏切角所指的晶轴或晶向</t>
+          <t>存放条件</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>下拉+其他</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>干燥器/手套箱/常温避光/冷藏/其他</t>
         </is>
       </c>
       <c r="F25" s="11" t="inlineStr">
@@ -7015,24 +7011,24 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G25" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(偏切角&gt;0)</t>
+      <c r="G25" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
         </is>
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>c面向a轴</t>
+          <t>干燥器</t>
         </is>
       </c>
       <c r="I25" s="11" t="inlineStr">
         <is>
-          <t>2026-07-24用户走查</t>
+          <t>review</t>
         </is>
       </c>
       <c r="J25" s="11" t="inlineStr">
         <is>
-          <t>substrate_miscut_angle_deg大于0时由跨字段校验强制填写</t>
+          <t>desiccator=干燥器</t>
         </is>
       </c>
       <c r="K25" s="11" t="inlineStr"/>
@@ -7045,49 +7041,45 @@
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>▸衬底·标称表面粗糙度</t>
+          <t>证书附件(CoA)</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>供应商或批次规格中的标称粗糙度</t>
+          <t>质检证书</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>粗糙度对象</t>
+          <t>FileAsset引用</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>{availability: 有规格数值|供应商未提供；有规格数值时 metric: Ra|RMS, value_nm}</t>
+          <t>{file_asset_id, sha256}</t>
         </is>
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>nm</t>
-        </is>
-      </c>
-      <c r="G26" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(衬底)</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G26" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>{availability: not_provided}</t>
+          <t>coa.pdf</t>
         </is>
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>2026-07-25用户复核</t>
-        </is>
-      </c>
-      <c r="J26" s="11" t="inlineStr">
-        <is>
-          <t>reported时metric与value_nm必填；not_provided时二者禁止填写；历史无availability对象按reported兼容；本片AFM实测值属于表征结果</t>
-        </is>
-      </c>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="J26" s="11" t="inlineStr"/>
       <c r="K26" s="11" t="inlineStr"/>
     </row>
     <row r="27">
@@ -7098,47 +7090,47 @@
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>▸衬底·来料尺寸规格</t>
+          <t>瓶身或包装标签附件</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>供应商标称或该批次来料的原始几何；切割后本次实际单片尺寸属于实验记录</t>
+          <t>试剂瓶身、气瓶或衬底包装标签的原始照片，用于追溯批号与规格</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>FileAsset引用</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>长×宽×厚</t>
+          <t>{file_asset_id, sha256}</t>
         </is>
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
-          <t>mm</t>
-        </is>
-      </c>
-      <c r="G27" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G27" s="15" t="inlineStr">
+        <is>
+          <t>推荐</t>
         </is>
       </c>
       <c r="H27" s="11" t="inlineStr">
         <is>
-          <t>10×10×0.5</t>
+          <t>bottle-label.jpg</t>
         </is>
       </c>
       <c r="I27" s="11" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>2026-07-24导师走查</t>
         </is>
       </c>
       <c r="J27" s="11" t="inlineStr">
         <is>
-          <t>不替代每次实验的本片实际尺寸</t>
+          <t>与CoA分开；同一物料版本至少上传一次并可预览、下载</t>
         </is>
       </c>
       <c r="K27" s="11" t="inlineStr"/>
@@ -7151,22 +7143,22 @@
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>▸气瓶·纯度等级</t>
+          <t>▸衬底·材料</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>子类(批次类别=气瓶)；与base『纯度』分工</t>
+          <t>子类(批次类别=衬底)</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>下拉</t>
+          <t>下拉+其他</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>6N/5N/4N/工业级</t>
+          <t>SiO₂/Si·蓝宝石(Al₂O₃)·石英·云母·Cu箔·Au箔·h-BN·其他</t>
         </is>
       </c>
       <c r="F28" s="11" t="inlineStr">
@@ -7174,14 +7166,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G28" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
+      <c r="G28" s="14" t="inlineStr">
+        <is>
+          <t>条件必填(衬底)</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>5N</t>
+          <t>SiO₂/Si</t>
         </is>
       </c>
       <c r="I28" s="11" t="inlineStr">
@@ -7191,7 +7183,7 @@
       </c>
       <c r="J28" s="11" t="inlineStr">
         <is>
-          <t>base纯度的数值百分比为权威值；这里只保留供应商标签</t>
+          <t>与§4衬底材料词表一致</t>
         </is>
       </c>
       <c r="K28" s="11" t="inlineStr"/>
@@ -7204,17 +7196,17 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>▸气瓶·气瓶编号</t>
+          <t>▸衬底·氧化层厚度</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>钢瓶追溯号</t>
+          <t>仅SiO₂/Si</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="E29" s="11" t="inlineStr">
@@ -7224,17 +7216,17 @@
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G29" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
+          <t>nm</t>
+        </is>
+      </c>
+      <c r="G29" s="14" t="inlineStr">
+        <is>
+          <t>条件必填(SiO₂/Si)</t>
         </is>
       </c>
       <c r="H29" s="11" t="inlineStr">
         <is>
-          <t>GC-Ar-07</t>
+          <t>285</t>
         </is>
       </c>
       <c r="I29" s="11" t="inlineStr">
@@ -7243,49 +7235,89 @@
         </is>
       </c>
       <c r="J29" s="11" t="inlineStr"/>
-      <c r="K29" s="11" t="inlineStr"/>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="10" t="inlineStr">
-        <is>
-          <t>实体② 装置库 Setup（一台炉登记一次，实验 §2 引用；坐标系随引用冻结）</t>
-        </is>
-      </c>
-      <c r="B30" s="8" t="n"/>
-      <c r="C30" s="8" t="n"/>
-      <c r="D30" s="8" t="n"/>
-      <c r="E30" s="8" t="n"/>
-      <c r="F30" s="8" t="n"/>
-      <c r="G30" s="8" t="n"/>
-      <c r="H30" s="8" t="n"/>
-      <c r="I30" s="8" t="n"/>
-      <c r="J30" s="8" t="n"/>
-      <c r="K30" s="8" t="n"/>
+      <c r="K29" s="11" t="inlineStr">
+        <is>
+          <t>{"gt":0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>MaterialLot</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>▸衬底·晶向与抛光信息</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>供应商是否提供且该衬底是否适用晶面取向与抛光规格</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>下拉</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>有规格数值·供应商未提供·不适用</t>
+        </is>
+      </c>
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="inlineStr">
+        <is>
+          <t>条件必填(衬底)</t>
+        </is>
+      </c>
+      <c r="H30" s="11" t="inlineStr">
+        <is>
+          <t>有规格数值</t>
+        </is>
+      </c>
+      <c r="I30" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-25用户复核</t>
+        </is>
+      </c>
+      <c r="J30" s="11" t="inlineStr">
+        <is>
+          <t>Cu/Au箔等不适用时明确选择不适用；禁止伪填晶向或抛光面</t>
+        </is>
+      </c>
+      <c r="K30" s="11" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>装置Setup</t>
+          <t>MaterialLot</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>装置名称</t>
+          <t>▸衬底·晶向与抛光</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>人读名</t>
+          <t>取向与抛光面</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>文本+下拉</t>
         </is>
       </c>
       <c r="E31" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>晶向；单面抛/双面抛</t>
         </is>
       </c>
       <c r="F31" s="11" t="inlineStr">
@@ -7293,48 +7325,56 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G31" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
+      <c r="G31" s="14" t="inlineStr">
+        <is>
+          <t>条件必填(有规格数值)</t>
         </is>
       </c>
       <c r="H31" s="11" t="inlineStr">
         <is>
-          <t>1号双温区管式炉</t>
+          <t>Si(100)；单面抛</t>
         </is>
       </c>
       <c r="I31" s="11" t="inlineStr">
         <is>
-          <t>会议</t>
-        </is>
-      </c>
-      <c r="J31" s="11" t="inlineStr"/>
-      <c r="K31" s="11" t="inlineStr"/>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="J31" s="11" t="inlineStr">
+        <is>
+          <t>实验引用批次后只读带出</t>
+        </is>
+      </c>
+      <c r="K31" s="11" t="inlineStr">
+        <is>
+          <t>{"require_option":true,"require_value":true}</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>装置Setup</t>
+          <t>MaterialLot</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>版本号</t>
+          <t>▸衬底·偏切信息</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>每次修改+1；引用时冻结此版本</t>
+          <t>供应商是否提供且该衬底是否适用相对标称晶面的偏切规格</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>下拉</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>有规格数值·供应商未提供·不适用</t>
         </is>
       </c>
       <c r="F32" s="11" t="inlineStr">
@@ -7342,24 +7382,24 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G32" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
+      <c r="G32" s="14" t="inlineStr">
+        <is>
+          <t>条件必填(衬底)</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>供应商未提供</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>★锁版使能(Fable三轮B2)</t>
+          <t>2026-07-25用户复核</t>
         </is>
       </c>
       <c r="J32" s="11" t="inlineStr">
         <is>
-          <t>对标 v1 setup_version_snapshot</t>
+          <t>0仅表示供应商明确报告无偏切，不能表示未知或不适用</t>
         </is>
       </c>
       <c r="K32" s="11" t="inlineStr"/>
@@ -7367,66 +7407,74 @@
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>装置Setup</t>
+          <t>MaterialLot</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>装置来源</t>
+          <t>▸衬底·偏切角</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>装置是商业购买、实验室自制还是在既有设备上改造</t>
+          <t>实际晶面相对标称晶面的偏切角</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>下拉</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>商业设备/实验室自制/改造设备</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F33" s="11" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G33" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
+          <t>°</t>
+        </is>
+      </c>
+      <c r="G33" s="14" t="inlineStr">
+        <is>
+          <t>条件必填(有规格数值)</t>
         </is>
       </c>
       <c r="H33" s="11" t="inlineStr">
         <is>
-          <t>商业设备</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="I33" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28用户逐项复核</t>
-        </is>
-      </c>
-      <c r="J33" s="11" t="inlineStr"/>
-      <c r="K33" s="11" t="inlineStr"/>
+          <t>2026-07-24用户走查</t>
+        </is>
+      </c>
+      <c r="J33" s="11" t="inlineStr">
+        <is>
+          <t>大于0时必须同时填写substrate_miscut_direction</t>
+        </is>
+      </c>
+      <c r="K33" s="11" t="inlineStr">
+        <is>
+          <t>{"ge":0,"lt":90}</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>装置Setup</t>
+          <t>MaterialLot</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>制造商或品牌</t>
+          <t>▸衬底·偏切方向</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>设备制造商或品牌，独立于型号保存以支持筛选和统计</t>
+          <t>偏切角所指的晶轴或晶向</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -7444,87 +7492,95 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G34" s="16" t="inlineStr">
-        <is>
-          <t>条件选填(商业设备或改造设备)</t>
+      <c r="G34" s="14" t="inlineStr">
+        <is>
+          <t>条件必填(偏切角&gt;0)</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>合肥科晶</t>
+          <t>c面向a轴</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28用户逐项复核</t>
-        </is>
-      </c>
-      <c r="J34" s="11" t="inlineStr"/>
+          <t>2026-07-24用户走查</t>
+        </is>
+      </c>
+      <c r="J34" s="11" t="inlineStr">
+        <is>
+          <t>substrate_miscut_angle_deg大于0时由跨字段校验强制填写</t>
+        </is>
+      </c>
       <c r="K34" s="11" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>装置Setup</t>
+          <t>MaterialLot</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>型号</t>
+          <t>▸衬底·标称表面粗糙度</t>
         </is>
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>制造商给出的设备型号</t>
+          <t>供应商或批次规格中的标称粗糙度</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>粗糙度对象</t>
         </is>
       </c>
       <c r="E35" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>{availability: 有规格数值|供应商未提供；有规格数值时 metric: Ra|RMS, value_nm}</t>
         </is>
       </c>
       <c r="F35" s="11" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G35" s="16" t="inlineStr">
-        <is>
-          <t>条件选填(商业设备或改造设备)</t>
+          <t>nm</t>
+        </is>
+      </c>
+      <c r="G35" s="14" t="inlineStr">
+        <is>
+          <t>条件必填(衬底)</t>
         </is>
       </c>
       <c r="H35" s="11" t="inlineStr">
         <is>
-          <t>OTF-1200X</t>
+          <t>{availability: not_provided}</t>
         </is>
       </c>
       <c r="I35" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28用户逐项复核</t>
-        </is>
-      </c>
-      <c r="J35" s="11" t="inlineStr"/>
+          <t>2026-07-25用户复核</t>
+        </is>
+      </c>
+      <c r="J35" s="11" t="inlineStr">
+        <is>
+          <t>reported时metric与value_nm必填；not_provided时二者禁止填写；历史无availability对象按reported兼容；本片AFM实测值属于表征结果</t>
+        </is>
+      </c>
       <c r="K35" s="11" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>装置Setup</t>
+          <t>MaterialLot</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>设计或建造单位</t>
+          <t>▸衬底·来料尺寸规格</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>实验室自制装置的设计或建造单位</t>
+          <t>供应商标称或该批次来料的原始几何；切割后本次实际单片尺寸属于实验记录</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -7534,95 +7590,103 @@
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>长×宽×厚</t>
         </is>
       </c>
       <c r="F36" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="G36" s="16" t="inlineStr">
         <is>
-          <t>条件选填(实验室自制)</t>
+          <t>选填</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>二维材料课题组</t>
+          <t>10×10×0.5</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28用户逐项复核</t>
-        </is>
-      </c>
-      <c r="J36" s="11" t="inlineStr"/>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="J36" s="11" t="inlineStr">
+        <is>
+          <t>不替代每次实验的本片实际尺寸</t>
+        </is>
+      </c>
       <c r="K36" s="11" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>装置Setup</t>
+          <t>MaterialLot</t>
         </is>
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>内部型号</t>
+          <t>▸衬底·层堆栈</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>实验室自制装置使用的内部型号或版本名称</t>
+          <t>从体材料到顶表面逐层记录供应商交付的衬底结构</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>JSON数组</t>
         </is>
       </c>
       <c r="E37" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>[{material_name,chemical_formula?,thickness_nm?,orientation?,supplier_lot_id?}]</t>
         </is>
       </c>
       <c r="F37" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>nm</t>
         </is>
       </c>
       <c r="G37" s="16" t="inlineStr">
         <is>
-          <t>条件选填(实验室自制)</t>
+          <t>条件选填(多层衬底)</t>
         </is>
       </c>
       <c r="H37" s="11" t="inlineStr">
         <is>
-          <t>CVD-LAB-A</t>
+          <t>[{"material_name":"Si"},{"material_name":"SiO2","thickness_nm":285}]</t>
         </is>
       </c>
       <c r="I37" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28用户逐项复核</t>
-        </is>
-      </c>
-      <c r="J37" s="11" t="inlineStr"/>
+          <t>2026-07-28深度审查</t>
+        </is>
+      </c>
+      <c r="J37" s="11" t="inlineStr">
+        <is>
+          <t>按数组顺序生成SubstrateStack；不得用单个字符串拼层</t>
+        </is>
+      </c>
       <c r="K37" s="11" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>装置Setup</t>
+          <t>MaterialLot</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>改造内容</t>
+          <t>▸衬底·顶表面</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>相对原设备发生变化且会影响实验条件或复现的改造</t>
+          <t>实验放样时实际暴露的最上层表面</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -7642,46 +7706,50 @@
       </c>
       <c r="G38" s="16" t="inlineStr">
         <is>
-          <t>条件选填(改造设备)</t>
+          <t>条件选填(多层衬底)</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>更换三温区加热模块并增加独立控温</t>
+          <t>SiO2</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28用户逐项复核</t>
-        </is>
-      </c>
-      <c r="J38" s="11" t="inlineStr"/>
+          <t>2026-07-28深度审查</t>
+        </is>
+      </c>
+      <c r="J38" s="11" t="inlineStr">
+        <is>
+          <t>与层堆栈配套</t>
+        </is>
+      </c>
       <c r="K38" s="11" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="11" t="inlineStr">
         <is>
-          <t>装置Setup</t>
+          <t>MaterialLot</t>
         </is>
       </c>
       <c r="B39" s="11" t="inlineStr">
         <is>
-          <t>实验室装置编号（资产编号）</t>
+          <t>▸气瓶·纯度等级</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>课题组用于识别这台装置的唯一业务编号；系统内部身份使用不可变UUID</t>
+          <t>子类(批次类别=气瓶)；与base『纯度』分工</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>下拉</t>
         </is>
       </c>
       <c r="E39" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6N/5N/4N/工业级</t>
         </is>
       </c>
       <c r="F39" s="11" t="inlineStr">
@@ -7689,24 +7757,24 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G39" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
+      <c r="G39" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
         </is>
       </c>
       <c r="H39" s="11" t="inlineStr">
         <is>
-          <t>CVD-炉1</t>
+          <t>5N</t>
         </is>
       </c>
       <c r="I39" s="11" t="inlineStr">
         <is>
-          <t>review§4.1B·2026-07-27终版整改</t>
+          <t>review</t>
         </is>
       </c>
       <c r="J39" s="11" t="inlineStr">
         <is>
-          <t>要求唯一；仅管理员可通过新版本纠正录入错误，历史版本保留原编号</t>
+          <t>base纯度的数值百分比为权威值；这里只保留供应商标签</t>
         </is>
       </c>
       <c r="K39" s="11" t="inlineStr"/>
@@ -7714,22 +7782,22 @@
     <row r="40">
       <c r="A40" s="11" t="inlineStr">
         <is>
-          <t>装置Setup</t>
+          <t>MaterialLot</t>
         </is>
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>温区数</t>
+          <t>▸气瓶·气瓶编号</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>独立控温区数</t>
+          <t>钢瓶追溯号</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
@@ -7739,83 +7807,43 @@
       </c>
       <c r="F40" s="11" t="inlineStr">
         <is>
-          <t>个</t>
-        </is>
-      </c>
-      <c r="G40" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G40" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>GC-Ar-07</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>会议</t>
+          <t>review</t>
         </is>
       </c>
       <c r="J40" s="11" t="inlineStr"/>
-      <c r="K40" s="11" t="inlineStr">
-        <is>
-          <t>{"ge":1,"type":"integer"}</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="11" t="inlineStr">
-        <is>
-          <t>装置Setup</t>
-        </is>
-      </c>
-      <c r="B41" s="11" t="inlineStr">
-        <is>
-          <t>各温区温度传感器</t>
-        </is>
-      </c>
-      <c r="C41" s="11" t="inlineStr">
-        <is>
-          <t>装置每个温区的传感器类别，以及设备资料明确给出时的标称测温精度</t>
-        </is>
-      </c>
-      <c r="D41" s="11" t="inlineStr">
-        <is>
-          <t>温度传感器数组</t>
-        </is>
-      </c>
-      <c r="E41" s="11" t="inlineStr">
-        <is>
-          <t>{sensor_type: thermocouple|rtd|infrared_thermometer|fiber_optic_temperature_sensor|thermistor|other, sensor_type_other?, zone_index, nominal_accuracy_C?}</t>
-        </is>
-      </c>
-      <c r="F41" s="11" t="inlineStr">
-        <is>
-          <t>℃</t>
-        </is>
-      </c>
-      <c r="G41" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
-        </is>
-      </c>
-      <c r="H41" s="11" t="inlineStr">
-        <is>
-          <t>[{sensor_type: 热电偶, zone_index: 1, nominal_accuracy_C: 1}]</t>
-        </is>
-      </c>
-      <c r="I41" s="11" t="inlineStr">
-        <is>
-          <t>2026-07-24导师走查·2026-07-27终版整改·2026-07-28用户复核</t>
-        </is>
-      </c>
-      <c r="J41" s="11" t="inlineStr">
-        <is>
-          <t>温区数决定卡片数量；传感器类别必填；标称测温精度仅在设备资料明确提供时填写，不要求用户估算</t>
-        </is>
-      </c>
-      <c r="K41" s="11" t="inlineStr"/>
+      <c r="K40" s="11" t="inlineStr"/>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>实体② 装置库 Setup（一台炉登记一次，实验 §2 引用；坐标系随引用冻结）</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="n"/>
+      <c r="C41" s="8" t="n"/>
+      <c r="D41" s="8" t="n"/>
+      <c r="E41" s="8" t="n"/>
+      <c r="F41" s="8" t="n"/>
+      <c r="G41" s="8" t="n"/>
+      <c r="H41" s="8" t="n"/>
+      <c r="I41" s="8" t="n"/>
+      <c r="J41" s="8" t="n"/>
+      <c r="K41" s="8" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="11" t="inlineStr">
@@ -7825,22 +7853,22 @@
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>炉体方向</t>
+          <t>装置名称</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>水平/垂直</t>
+          <t>人读名</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>下拉</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E42" s="11" t="inlineStr">
         <is>
-          <t>水平/垂直</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F42" s="11" t="inlineStr">
@@ -7855,7 +7883,7 @@
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>水平</t>
+          <t>1号双温区管式炉</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
@@ -7874,22 +7902,22 @@
       </c>
       <c r="B43" s="11" t="inlineStr">
         <is>
-          <t>炉管材质与截面</t>
+          <t>版本号</t>
         </is>
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>炉管材料与截面</t>
+          <t>每次修改+1；引用时冻结此版本</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr">
         <is>
-          <t>管材质形状对象</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="E43" s="11" t="inlineStr">
         <is>
-          <t>{material: 石英|刚玉|其他, material_other?, shape: 圆形|方形|矩形|其他, shape_other?}</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F43" s="11" t="inlineStr">
@@ -7904,17 +7932,17 @@
       </c>
       <c r="H43" s="11" t="inlineStr">
         <is>
-          <t>{material: 石英, shape: 圆形}</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I43" s="11" t="inlineStr">
         <is>
-          <t>2026-07-24导师走查</t>
+          <t>★锁版使能(Fable三轮B2)</t>
         </is>
       </c>
       <c r="J43" s="11" t="inlineStr">
         <is>
-          <t>材质与截面形状独立保存，禁止把“刚玉；圆”当作一个选项</t>
+          <t>对标 v1 setup_version_snapshot</t>
         </is>
       </c>
       <c r="K43" s="11" t="inlineStr"/>
@@ -7927,49 +7955,45 @@
       </c>
       <c r="B44" s="11" t="inlineStr">
         <is>
-          <t>炉管尺寸</t>
+          <t>装置来源</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>按截面形状记录外部尺寸和壁厚</t>
+          <t>装置是商业购买、实验室自制还是在既有设备上改造</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>炉管尺寸对象</t>
+          <t>下拉</t>
         </is>
       </c>
       <c r="E44" s="11" t="inlineStr">
         <is>
-          <t>{圆形: outer_diameter_mm+wall_thickness_mm; 方形: outer_side_mm+wall_thickness_mm; 矩形: outer_width_mm+outer_height_mm+wall_thickness_mm; 其他: dimension_description}</t>
+          <t>商业设备/实验室自制/改造设备</t>
         </is>
       </c>
       <c r="F44" s="11" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G44" s="12" t="inlineStr">
         <is>
-          <t>必填；按炉管截面填写</t>
+          <t>必填</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>{outer_width_mm: 50, outer_height_mm: 30, wall_thickness_mm: 2}</t>
+          <t>商业设备</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>会议·用户复核2026-07-24</t>
-        </is>
-      </c>
-      <c r="J44" s="11" t="inlineStr">
-        <is>
-          <t>选择材质与截面后必须按形状完整填写；圆形填外径+壁厚，方形填外边长+壁厚，矩形填外宽+外高+壁厚，其他截面填写具名尺寸说明</t>
-        </is>
-      </c>
+          <t>2026-07-28用户逐项复核</t>
+        </is>
+      </c>
+      <c r="J44" s="11" t="inlineStr"/>
       <c r="K44" s="11" t="inlineStr"/>
     </row>
     <row r="45">
@@ -7980,22 +8004,22 @@
       </c>
       <c r="B45" s="11" t="inlineStr">
         <is>
-          <t>壁型</t>
+          <t>制造商或品牌</t>
         </is>
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>热壁/冷壁</t>
+          <t>设备制造商或品牌，独立于型号保存以支持筛选和统计</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>下拉</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E45" s="11" t="inlineStr">
         <is>
-          <t>热壁/冷壁</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F45" s="11" t="inlineStr">
@@ -8003,26 +8027,22 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G45" s="15" t="inlineStr">
-        <is>
-          <t>推荐</t>
+      <c r="G45" s="16" t="inlineStr">
+        <is>
+          <t>条件选填(商业设备或改造设备)</t>
         </is>
       </c>
       <c r="H45" s="11" t="inlineStr">
         <is>
-          <t>热壁</t>
+          <t>合肥科晶</t>
         </is>
       </c>
       <c r="I45" s="11" t="inlineStr">
         <is>
-          <t>复审</t>
-        </is>
-      </c>
-      <c r="J45" s="11" t="inlineStr">
-        <is>
-          <t>放在装置身份、温区与炉管结构之后，避免打断由粗到细的登记顺序</t>
-        </is>
-      </c>
+          <t>2026-07-28用户逐项复核</t>
+        </is>
+      </c>
+      <c r="J45" s="11" t="inlineStr"/>
       <c r="K45" s="11" t="inlineStr"/>
     </row>
     <row r="46">
@@ -8033,22 +8053,22 @@
       </c>
       <c r="B46" s="11" t="inlineStr">
         <is>
-          <t>坐标系定义</t>
+          <t>型号</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>系统统一采用上游为负、下游为正的固定坐标定义</t>
+          <t>制造商给出的设备型号</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>固定定义</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
         <is>
-          <t>上游为负；下游为正；原点固定</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F46" s="11" t="inlineStr">
@@ -8056,26 +8076,22 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G46" s="17" t="inlineStr">
-        <is>
-          <t>定义项</t>
+      <c r="G46" s="16" t="inlineStr">
+        <is>
+          <t>条件选填(商业设备或改造设备)</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>上游(-)←原点→下游(+)</t>
+          <t>OTF-1200X</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>2026-07-24导师走查</t>
-        </is>
-      </c>
-      <c r="J46" s="11" t="inlineStr">
-        <is>
-          <t>服务端写入固定机器码，管理员和成员均不可编辑</t>
-        </is>
-      </c>
+          <t>2026-07-28用户逐项复核</t>
+        </is>
+      </c>
+      <c r="J46" s="11" t="inlineStr"/>
       <c r="K46" s="11" t="inlineStr"/>
     </row>
     <row r="47">
@@ -8086,22 +8102,22 @@
       </c>
       <c r="B47" s="11" t="inlineStr">
         <is>
-          <t>外场能力</t>
+          <t>设计或建造单位</t>
         </is>
       </c>
       <c r="C47" s="11" t="inlineStr">
         <is>
-          <t>装置具备的光、电或等离子体能力</t>
+          <t>实验室自制装置的设计或建造单位</t>
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr">
         <is>
-          <t>多选</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E47" s="11" t="inlineStr">
         <is>
-          <t>无/光/电/等离子体</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F47" s="11" t="inlineStr">
@@ -8109,26 +8125,22 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G47" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
+      <c r="G47" s="16" t="inlineStr">
+        <is>
+          <t>条件选填(实验室自制)</t>
         </is>
       </c>
       <c r="H47" s="11" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>二维材料课题组</t>
         </is>
       </c>
       <c r="I47" s="11" t="inlineStr">
         <is>
-          <t>2026-07-24导师走查</t>
-        </is>
-      </c>
-      <c r="J47" s="11" t="inlineStr">
-        <is>
-          <t>这里只登记能力；每炉实际使用情况在反应条件中记录</t>
-        </is>
-      </c>
+          <t>2026-07-28用户逐项复核</t>
+        </is>
+      </c>
+      <c r="J47" s="11" t="inlineStr"/>
       <c r="K47" s="11" t="inlineStr"/>
     </row>
     <row r="48">
@@ -8139,22 +8151,22 @@
       </c>
       <c r="B48" s="11" t="inlineStr">
         <is>
-          <t>装置示意图与描述</t>
+          <t>内部型号</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>装置照片或示意图及文字说明</t>
+          <t>实验室自制装置使用的内部型号或版本名称</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>FileAsset引用+自由</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
-          <t>{file_asset_id, sha256, note}</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F48" s="11" t="inlineStr">
@@ -8162,55 +8174,87 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G48" s="15" t="inlineStr">
-        <is>
-          <t>推荐</t>
+      <c r="G48" s="16" t="inlineStr">
+        <is>
+          <t>条件选填(实验室自制)</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>setup.png</t>
+          <t>CVD-LAB-A</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>会议</t>
+          <t>2026-07-28用户逐项复核</t>
         </is>
       </c>
       <c r="J48" s="11" t="inlineStr"/>
       <c r="K48" s="11" t="inlineStr"/>
     </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="10" t="inlineStr">
-        <is>
-          <t>实体③ 表征仪器 Instrument（实验 §7 表征引用；对标 NeXus NXfabrication 仪器溯源）</t>
-        </is>
-      </c>
-      <c r="B49" s="8" t="n"/>
-      <c r="C49" s="8" t="n"/>
-      <c r="D49" s="8" t="n"/>
-      <c r="E49" s="8" t="n"/>
-      <c r="F49" s="8" t="n"/>
-      <c r="G49" s="8" t="n"/>
-      <c r="H49" s="8" t="n"/>
-      <c r="I49" s="8" t="n"/>
-      <c r="J49" s="8" t="n"/>
-      <c r="K49" s="8" t="n"/>
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
+        <is>
+          <t>装置Setup</t>
+        </is>
+      </c>
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>改造内容</t>
+        </is>
+      </c>
+      <c r="C49" s="11" t="inlineStr">
+        <is>
+          <t>相对原设备发生变化且会影响实验条件或复现的改造</t>
+        </is>
+      </c>
+      <c r="D49" s="11" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="E49" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F49" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G49" s="16" t="inlineStr">
+        <is>
+          <t>条件选填(改造设备)</t>
+        </is>
+      </c>
+      <c r="H49" s="11" t="inlineStr">
+        <is>
+          <t>更换三温区加热模块并增加独立控温</t>
+        </is>
+      </c>
+      <c r="I49" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-28用户逐项复核</t>
+        </is>
+      </c>
+      <c r="J49" s="11" t="inlineStr"/>
+      <c r="K49" s="11" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="11" t="inlineStr">
         <is>
-          <t>表征仪器</t>
+          <t>装置Setup</t>
         </is>
       </c>
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>仪器编号</t>
+          <t>实验室装置编号（资产编号）</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>唯一编号</t>
+          <t>课题组用于识别这台装置的唯一业务编号；系统内部身份使用不可变UUID</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -8235,46 +8279,50 @@
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>RAMAN-1</t>
+          <t>CVD-炉1</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>复审</t>
-        </is>
-      </c>
-      <c r="J50" s="11" t="inlineStr"/>
+          <t>review§4.1B·2026-07-27终版整改</t>
+        </is>
+      </c>
+      <c r="J50" s="11" t="inlineStr">
+        <is>
+          <t>要求唯一；仅管理员可通过新版本纠正录入错误，历史版本保留原编号</t>
+        </is>
+      </c>
       <c r="K50" s="11" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="11" t="inlineStr">
         <is>
-          <t>表征仪器</t>
+          <t>装置Setup</t>
         </is>
       </c>
       <c r="B51" s="11" t="inlineStr">
         <is>
-          <t>适用表征方法</t>
+          <t>温区数</t>
         </is>
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t>该仪器适用的表征方法，用于结果录入时筛选仪器</t>
+          <t>独立控温区数</t>
         </is>
       </c>
       <c r="D51" s="11" t="inlineStr">
         <is>
-          <t>下拉+其他</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="E51" s="11" t="inlineStr">
         <is>
-          <t>光镜/SEM/Raman/低波数Raman/PL/AFM/XRD/TEM/其他</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F51" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>个</t>
         </is>
       </c>
       <c r="G51" s="12" t="inlineStr">
@@ -8284,7 +8332,7 @@
       </c>
       <c r="H51" s="11" t="inlineStr">
         <is>
-          <t>Raman</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I51" s="11" t="inlineStr">
@@ -8292,86 +8340,90 @@
           <t>会议</t>
         </is>
       </c>
-      <c r="J51" s="11" t="inlineStr">
-        <is>
-          <t>API key 保持 name_type 以兼容现有数据</t>
-        </is>
-      </c>
-      <c r="K51" s="11" t="inlineStr"/>
+      <c r="J51" s="11" t="inlineStr"/>
+      <c r="K51" s="11" t="inlineStr">
+        <is>
+          <t>{"ge":1,"type":"integer"}</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
         <is>
-          <t>表征仪器</t>
+          <t>装置Setup</t>
         </is>
       </c>
       <c r="B52" s="11" t="inlineStr">
         <is>
-          <t>厂商</t>
+          <t>各温区温度传感器</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>品牌</t>
+          <t>装置每个温区的传感器类别，以及设备资料明确给出时的标称测温精度</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>温度传感器数组</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>{sensor_type: thermocouple|rtd|infrared_thermometer|fiber_optic_temperature_sensor|thermistor|other, sensor_type_other?, zone_index, nominal_accuracy_C?}</t>
         </is>
       </c>
       <c r="F52" s="11" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G52" s="15" t="inlineStr">
-        <is>
-          <t>推荐</t>
+          <t>℃</t>
+        </is>
+      </c>
+      <c r="G52" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>Horiba</t>
+          <t>[{sensor_type: 热电偶, zone_index: 1, nominal_accuracy_C: 1}]</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>★NXfabrication</t>
-        </is>
-      </c>
-      <c r="J52" s="11" t="inlineStr"/>
+          <t>2026-07-24导师走查·2026-07-27终版整改·2026-07-28用户复核</t>
+        </is>
+      </c>
+      <c r="J52" s="11" t="inlineStr">
+        <is>
+          <t>温区数决定卡片数量；传感器类别必填；标称测温精度仅在设备资料明确提供时填写，不要求用户估算</t>
+        </is>
+      </c>
       <c r="K52" s="11" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="11" t="inlineStr">
         <is>
-          <t>表征仪器</t>
+          <t>装置Setup</t>
         </is>
       </c>
       <c r="B53" s="11" t="inlineStr">
         <is>
-          <t>型号</t>
+          <t>炉体方向</t>
         </is>
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>型号</t>
+          <t>水平/垂直</t>
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>下拉</t>
         </is>
       </c>
       <c r="E53" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>水平/垂直</t>
         </is>
       </c>
       <c r="F53" s="11" t="inlineStr">
@@ -8379,19 +8431,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G53" s="15" t="inlineStr">
-        <is>
-          <t>推荐</t>
+      <c r="G53" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
         </is>
       </c>
       <c r="H53" s="11" t="inlineStr">
         <is>
-          <t>LabRAM HR</t>
+          <t>水平</t>
         </is>
       </c>
       <c r="I53" s="11" t="inlineStr">
         <is>
-          <t>★NXfabrication</t>
+          <t>会议</t>
         </is>
       </c>
       <c r="J53" s="11" t="inlineStr"/>
@@ -8400,27 +8452,27 @@
     <row r="54">
       <c r="A54" s="11" t="inlineStr">
         <is>
-          <t>表征仪器</t>
+          <t>装置Setup</t>
         </is>
       </c>
       <c r="B54" s="11" t="inlineStr">
         <is>
-          <t>序列号</t>
+          <t>炉管材质与截面</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>设备序列号</t>
+          <t>炉管材料与截面</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>管材质形状对象</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>{material: 石英|刚玉|其他, material_other?, shape: 圆形|方形|矩形|其他, shape_other?}</t>
         </is>
       </c>
       <c r="F54" s="11" t="inlineStr">
@@ -8428,73 +8480,77 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G54" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
+      <c r="G54" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>{material: 石英, shape: 圆形}</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>★NXfabrication</t>
-        </is>
-      </c>
-      <c r="J54" s="11" t="inlineStr"/>
+          <t>2026-07-24导师走查</t>
+        </is>
+      </c>
+      <c r="J54" s="11" t="inlineStr">
+        <is>
+          <t>材质与截面形状独立保存，禁止把“刚玉；圆”当作一个选项</t>
+        </is>
+      </c>
       <c r="K54" s="11" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="11" t="inlineStr">
         <is>
-          <t>表征仪器</t>
+          <t>装置Setup</t>
         </is>
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
-          <t>仪器持久标识</t>
+          <t>炉管尺寸</t>
         </is>
       </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>可长期稳定指向该仪器的公开或机构标识，不等同于设备序列号</t>
+          <t>按截面形状记录外部尺寸和壁厚</t>
         </is>
       </c>
       <c r="D55" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>炉管尺寸对象</t>
         </is>
       </c>
       <c r="E55" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>{圆形: outer_diameter_mm+wall_thickness_mm; 方形: outer_side_mm+wall_thickness_mm; 矩形: outer_width_mm+outer_height_mm+wall_thickness_mm; 其他: dimension_description}</t>
         </is>
       </c>
       <c r="F55" s="11" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G55" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="G55" s="12" t="inlineStr">
+        <is>
+          <t>必填；按炉管截面填写</t>
         </is>
       </c>
       <c r="H55" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>{outer_width_mm: 50, outer_height_mm: 30, wall_thickness_mm: 2}</t>
         </is>
       </c>
       <c r="I55" s="11" t="inlineStr">
         <is>
-          <t>★NXfabrication/PIDINST</t>
+          <t>会议·用户复核2026-07-24</t>
         </is>
       </c>
       <c r="J55" s="11" t="inlineStr">
         <is>
-          <t>PID 是 Persistent Identifier 的缩写；没有机构标识时可留空</t>
+          <t>选择材质与截面后必须按形状完整填写；圆形填外径+壁厚，方形填外边长+壁厚，矩形填外宽+外高+壁厚，其他截面填写具名尺寸说明</t>
         </is>
       </c>
       <c r="K55" s="11" t="inlineStr"/>
@@ -8502,27 +8558,27 @@
     <row r="56">
       <c r="A56" s="11" t="inlineStr">
         <is>
-          <t>表征仪器</t>
+          <t>装置Setup</t>
         </is>
       </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
-          <t>所在实验室与位置</t>
+          <t>壁型</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>物理位置</t>
+          <t>热壁/冷壁</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>下拉</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>热壁/冷壁</t>
         </is>
       </c>
       <c r="F56" s="11" t="inlineStr">
@@ -8530,48 +8586,52 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G56" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
+      <c r="G56" s="15" t="inlineStr">
+        <is>
+          <t>推荐</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>A305</t>
+          <t>热壁</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>建议</t>
-        </is>
-      </c>
-      <c r="J56" s="11" t="inlineStr"/>
+          <t>复审</t>
+        </is>
+      </c>
+      <c r="J56" s="11" t="inlineStr">
+        <is>
+          <t>放在装置身份、温区与炉管结构之后，避免打断由粗到细的登记顺序</t>
+        </is>
+      </c>
       <c r="K56" s="11" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="inlineStr">
         <is>
-          <t>表征仪器</t>
+          <t>装置Setup</t>
         </is>
       </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
-          <t>关键固定配置</t>
+          <t>坐标系定义</t>
         </is>
       </c>
       <c r="C57" s="11" t="inlineStr">
         <is>
-          <t>随仪器长期固定的硬件或能力；本次实际使用参数在表征结果的测试条件中填写</t>
+          <t>系统统一采用上游为负、下游为正的固定坐标定义</t>
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr">
         <is>
-          <t>自由</t>
+          <t>固定定义</t>
         </is>
       </c>
       <c r="E57" s="11" t="inlineStr">
         <is>
-          <t>如探测器型号、光栅范围、可用激光与物镜范围</t>
+          <t>上游为负；下游为正；原点固定</t>
         </is>
       </c>
       <c r="F57" s="11" t="inlineStr">
@@ -8579,24 +8639,24 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G57" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
+      <c r="G57" s="17" t="inlineStr">
+        <is>
+          <t>定义项</t>
         </is>
       </c>
       <c r="H57" s="11" t="inlineStr">
         <is>
-          <t>CCD探测器；300、600、1800 lines·mm⁻¹光栅</t>
+          <t>上游(-)←原点→下游(+)</t>
         </is>
       </c>
       <c r="I57" s="11" t="inlineStr">
         <is>
-          <t>会议</t>
+          <t>2026-07-24导师走查</t>
         </is>
       </c>
       <c r="J57" s="11" t="inlineStr">
         <is>
-          <t>不在此重复本次实际使用的波长、物镜、功率或积分时间</t>
+          <t>服务端写入固定机器码，管理员和成员均不可编辑</t>
         </is>
       </c>
       <c r="K57" s="11" t="inlineStr"/>
@@ -8604,57 +8664,686 @@
     <row r="58">
       <c r="A58" s="11" t="inlineStr">
         <is>
+          <t>装置Setup</t>
+        </is>
+      </c>
+      <c r="B58" s="11" t="inlineStr">
+        <is>
+          <t>外场能力</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>装置具备的光、电或等离子体能力</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>多选</t>
+        </is>
+      </c>
+      <c r="E58" s="11" t="inlineStr">
+        <is>
+          <t>无/光/电/等离子体</t>
+        </is>
+      </c>
+      <c r="F58" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G58" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
+        </is>
+      </c>
+      <c r="H58" s="11" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="I58" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-24导师走查</t>
+        </is>
+      </c>
+      <c r="J58" s="11" t="inlineStr">
+        <is>
+          <t>这里只登记能力；每炉实际使用情况在反应条件中记录</t>
+        </is>
+      </c>
+      <c r="K58" s="11" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="11" t="inlineStr">
+        <is>
+          <t>装置Setup</t>
+        </is>
+      </c>
+      <c r="B59" s="11" t="inlineStr">
+        <is>
+          <t>装置示意图与描述</t>
+        </is>
+      </c>
+      <c r="C59" s="11" t="inlineStr">
+        <is>
+          <t>装置照片或示意图及文字说明</t>
+        </is>
+      </c>
+      <c r="D59" s="11" t="inlineStr">
+        <is>
+          <t>FileAsset引用+自由</t>
+        </is>
+      </c>
+      <c r="E59" s="11" t="inlineStr">
+        <is>
+          <t>{file_asset_id, sha256, note}</t>
+        </is>
+      </c>
+      <c r="F59" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G59" s="15" t="inlineStr">
+        <is>
+          <t>推荐</t>
+        </is>
+      </c>
+      <c r="H59" s="11" t="inlineStr">
+        <is>
+          <t>setup.png</t>
+        </is>
+      </c>
+      <c r="I59" s="11" t="inlineStr">
+        <is>
+          <t>会议</t>
+        </is>
+      </c>
+      <c r="J59" s="11" t="inlineStr"/>
+      <c r="K59" s="11" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>装置Setup</t>
+        </is>
+      </c>
+      <c r="B60" s="11" t="inlineStr">
+        <is>
+          <t>可更换部件绑定</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>当前Setup版本实际安装的炉管、传感器、MFC、压力计等部件</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
+        <is>
+          <t>JSON数组</t>
+        </is>
+      </c>
+      <c r="E60" s="11" t="inlineStr">
+        <is>
+          <t>[{component_id,role,position?}]</t>
+        </is>
+      </c>
+      <c r="F60" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G60" s="15" t="inlineStr">
+        <is>
+          <t>推荐</t>
+        </is>
+      </c>
+      <c r="H60" s="11" t="inlineStr">
+        <is>
+          <t>[{"component_id":"UUID","role":"furnace_tube"}]</t>
+        </is>
+      </c>
+      <c r="I60" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-28深度审查</t>
+        </is>
+      </c>
+      <c r="J60" s="11" t="inlineStr">
+        <is>
+          <t>部件身份、校准和维护走独立生命周期事件</t>
+        </is>
+      </c>
+      <c r="K60" s="11" t="inlineStr"/>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="10" t="inlineStr">
+        <is>
+          <t>实体③ 表征仪器 Instrument（实验 §7 表征引用；对标 NeXus NXfabrication 仪器溯源）</t>
+        </is>
+      </c>
+      <c r="B61" s="8" t="n"/>
+      <c r="C61" s="8" t="n"/>
+      <c r="D61" s="8" t="n"/>
+      <c r="E61" s="8" t="n"/>
+      <c r="F61" s="8" t="n"/>
+      <c r="G61" s="8" t="n"/>
+      <c r="H61" s="8" t="n"/>
+      <c r="I61" s="8" t="n"/>
+      <c r="J61" s="8" t="n"/>
+      <c r="K61" s="8" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
           <t>表征仪器</t>
         </is>
       </c>
-      <c r="B58" s="11" t="inlineStr">
+      <c r="B62" s="11" t="inlineStr">
+        <is>
+          <t>仪器编号</t>
+        </is>
+      </c>
+      <c r="C62" s="11" t="inlineStr">
+        <is>
+          <t>唯一编号</t>
+        </is>
+      </c>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="E62" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F62" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G62" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
+        </is>
+      </c>
+      <c r="H62" s="11" t="inlineStr">
+        <is>
+          <t>RAMAN-1</t>
+        </is>
+      </c>
+      <c r="I62" s="11" t="inlineStr">
+        <is>
+          <t>复审</t>
+        </is>
+      </c>
+      <c r="J62" s="11" t="inlineStr"/>
+      <c r="K62" s="11" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="11" t="inlineStr">
+        <is>
+          <t>表征仪器</t>
+        </is>
+      </c>
+      <c r="B63" s="11" t="inlineStr">
+        <is>
+          <t>适用表征方法</t>
+        </is>
+      </c>
+      <c r="C63" s="11" t="inlineStr">
+        <is>
+          <t>该仪器适用的表征方法，用于结果录入时筛选仪器</t>
+        </is>
+      </c>
+      <c r="D63" s="11" t="inlineStr">
+        <is>
+          <t>下拉+其他</t>
+        </is>
+      </c>
+      <c r="E63" s="11" t="inlineStr">
+        <is>
+          <t>光镜/SEM/Raman/低波数Raman/PL/AFM/XRD/TEM/其他</t>
+        </is>
+      </c>
+      <c r="F63" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G63" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
+        </is>
+      </c>
+      <c r="H63" s="11" t="inlineStr">
+        <is>
+          <t>Raman</t>
+        </is>
+      </c>
+      <c r="I63" s="11" t="inlineStr">
+        <is>
+          <t>会议</t>
+        </is>
+      </c>
+      <c r="J63" s="11" t="inlineStr">
+        <is>
+          <t>API key 保持 name_type 以兼容现有数据</t>
+        </is>
+      </c>
+      <c r="K63" s="11" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="inlineStr">
+        <is>
+          <t>表征仪器</t>
+        </is>
+      </c>
+      <c r="B64" s="11" t="inlineStr">
+        <is>
+          <t>厂商</t>
+        </is>
+      </c>
+      <c r="C64" s="11" t="inlineStr">
+        <is>
+          <t>品牌</t>
+        </is>
+      </c>
+      <c r="D64" s="11" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="E64" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F64" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G64" s="15" t="inlineStr">
+        <is>
+          <t>推荐</t>
+        </is>
+      </c>
+      <c r="H64" s="11" t="inlineStr">
+        <is>
+          <t>Horiba</t>
+        </is>
+      </c>
+      <c r="I64" s="11" t="inlineStr">
+        <is>
+          <t>★NXfabrication</t>
+        </is>
+      </c>
+      <c r="J64" s="11" t="inlineStr"/>
+      <c r="K64" s="11" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="11" t="inlineStr">
+        <is>
+          <t>表征仪器</t>
+        </is>
+      </c>
+      <c r="B65" s="11" t="inlineStr">
+        <is>
+          <t>型号</t>
+        </is>
+      </c>
+      <c r="C65" s="11" t="inlineStr">
+        <is>
+          <t>型号</t>
+        </is>
+      </c>
+      <c r="D65" s="11" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="E65" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F65" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G65" s="15" t="inlineStr">
+        <is>
+          <t>推荐</t>
+        </is>
+      </c>
+      <c r="H65" s="11" t="inlineStr">
+        <is>
+          <t>LabRAM HR</t>
+        </is>
+      </c>
+      <c r="I65" s="11" t="inlineStr">
+        <is>
+          <t>★NXfabrication</t>
+        </is>
+      </c>
+      <c r="J65" s="11" t="inlineStr"/>
+      <c r="K65" s="11" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t>表征仪器</t>
+        </is>
+      </c>
+      <c r="B66" s="11" t="inlineStr">
+        <is>
+          <t>序列号</t>
+        </is>
+      </c>
+      <c r="C66" s="11" t="inlineStr">
+        <is>
+          <t>设备序列号</t>
+        </is>
+      </c>
+      <c r="D66" s="11" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="E66" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F66" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G66" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
+        </is>
+      </c>
+      <c r="H66" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I66" s="11" t="inlineStr">
+        <is>
+          <t>★NXfabrication</t>
+        </is>
+      </c>
+      <c r="J66" s="11" t="inlineStr"/>
+      <c r="K66" s="11" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="11" t="inlineStr">
+        <is>
+          <t>表征仪器</t>
+        </is>
+      </c>
+      <c r="B67" s="11" t="inlineStr">
+        <is>
+          <t>仪器持久标识</t>
+        </is>
+      </c>
+      <c r="C67" s="11" t="inlineStr">
+        <is>
+          <t>可长期稳定指向该仪器的公开或机构标识，不等同于设备序列号</t>
+        </is>
+      </c>
+      <c r="D67" s="11" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="E67" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F67" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G67" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
+        </is>
+      </c>
+      <c r="H67" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I67" s="11" t="inlineStr">
+        <is>
+          <t>★NXfabrication/PIDINST</t>
+        </is>
+      </c>
+      <c r="J67" s="11" t="inlineStr">
+        <is>
+          <t>PID 是 Persistent Identifier 的缩写；没有机构标识时可留空</t>
+        </is>
+      </c>
+      <c r="K67" s="11" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="inlineStr">
+        <is>
+          <t>表征仪器</t>
+        </is>
+      </c>
+      <c r="B68" s="11" t="inlineStr">
+        <is>
+          <t>所在实验室与位置</t>
+        </is>
+      </c>
+      <c r="C68" s="11" t="inlineStr">
+        <is>
+          <t>物理位置</t>
+        </is>
+      </c>
+      <c r="D68" s="11" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="E68" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F68" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G68" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
+        </is>
+      </c>
+      <c r="H68" s="11" t="inlineStr">
+        <is>
+          <t>A305</t>
+        </is>
+      </c>
+      <c r="I68" s="11" t="inlineStr">
+        <is>
+          <t>建议</t>
+        </is>
+      </c>
+      <c r="J68" s="11" t="inlineStr"/>
+      <c r="K68" s="11" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="11" t="inlineStr">
+        <is>
+          <t>表征仪器</t>
+        </is>
+      </c>
+      <c r="B69" s="11" t="inlineStr">
+        <is>
+          <t>关键固定配置</t>
+        </is>
+      </c>
+      <c r="C69" s="11" t="inlineStr">
+        <is>
+          <t>随仪器长期固定的硬件或能力；本次实际使用参数在表征结果的测试条件中填写</t>
+        </is>
+      </c>
+      <c r="D69" s="11" t="inlineStr">
+        <is>
+          <t>自由</t>
+        </is>
+      </c>
+      <c r="E69" s="11" t="inlineStr">
+        <is>
+          <t>如探测器型号、光栅范围、可用激光与物镜范围</t>
+        </is>
+      </c>
+      <c r="F69" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G69" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
+        </is>
+      </c>
+      <c r="H69" s="11" t="inlineStr">
+        <is>
+          <t>CCD探测器；300、600、1800 lines·mm⁻¹光栅</t>
+        </is>
+      </c>
+      <c r="I69" s="11" t="inlineStr">
+        <is>
+          <t>会议</t>
+        </is>
+      </c>
+      <c r="J69" s="11" t="inlineStr">
+        <is>
+          <t>不在此重复本次实际使用的波长、物镜、功率或积分时间</t>
+        </is>
+      </c>
+      <c r="K69" s="11" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="inlineStr">
+        <is>
+          <t>表征仪器</t>
+        </is>
+      </c>
+      <c r="B70" s="11" t="inlineStr">
+        <is>
+          <t>测量能力配置</t>
+        </is>
+      </c>
+      <c r="C70" s="11" t="inlineStr">
+        <is>
+          <t>仪器版本支持的测量方法及其可选固定配置</t>
+        </is>
+      </c>
+      <c r="D70" s="11" t="inlineStr">
+        <is>
+          <t>JSON数组</t>
+        </is>
+      </c>
+      <c r="E70" s="11" t="inlineStr">
+        <is>
+          <t>[{code,configuration}]</t>
+        </is>
+      </c>
+      <c r="F70" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G70" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
+        </is>
+      </c>
+      <c r="H70" s="11" t="inlineStr">
+        <is>
+          <t>[{"code":"Raman","configuration":{"lasers_nm":[532]}}]</t>
+        </is>
+      </c>
+      <c r="I70" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-28深度审查</t>
+        </is>
+      </c>
+      <c r="J70" s="11" t="inlineStr">
+        <is>
+          <t>本次MeasurementRun只能选择这里声明的能力</t>
+        </is>
+      </c>
+      <c r="K70" s="11" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="11" t="inlineStr">
+        <is>
+          <t>表征仪器</t>
+        </is>
+      </c>
+      <c r="B71" s="11" t="inlineStr">
         <is>
           <t>最近校准或维护日期</t>
         </is>
       </c>
-      <c r="C58" s="11" t="inlineStr">
+      <c r="C71" s="11" t="inlineStr">
         <is>
           <t>校准/维护日期</t>
         </is>
       </c>
-      <c r="D58" s="11" t="inlineStr">
+      <c r="D71" s="11" t="inlineStr">
         <is>
           <t>日期</t>
         </is>
       </c>
-      <c r="E58" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F58" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G58" s="16" t="inlineStr">
+      <c r="E71" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F71" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G71" s="16" t="inlineStr">
         <is>
           <t>选填</t>
         </is>
       </c>
-      <c r="H58" s="11" t="inlineStr">
+      <c r="H71" s="11" t="inlineStr">
         <is>
           <t>2026-06</t>
         </is>
       </c>
-      <c r="I58" s="11" t="inlineStr">
+      <c r="I71" s="11" t="inlineStr">
         <is>
           <t>会议</t>
         </is>
       </c>
-      <c r="J58" s="11" t="inlineStr"/>
-      <c r="K58" s="11" t="inlineStr"/>
+      <c r="J71" s="11" t="inlineStr"/>
+      <c r="K71" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A49:K49"/>
-    <mergeCell ref="A30:K30"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="A61:K61"/>
     <mergeCell ref="A3:K3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8667,7 +9356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -9971,20 +10660,42 @@
     <row r="63">
       <c r="A63" s="11" t="inlineStr">
         <is>
+          <t>v4.0-rc.1</t>
+        </is>
+      </c>
+      <c r="B63" s="11" t="inlineStr">
+        <is>
+          <t>科学对象/实体/结果</t>
+        </is>
+      </c>
+      <c r="C63" s="11" t="inlineStr">
+        <is>
+          <t>引入正交TargetSpec、物理SourceLoad、统一ProcessTimeline、不可变RunRevision、样品转换图及MeasurementRun→AnalysisRun→PropertyValue/MaterialAssertion溯源链；物料、装置部件和仪器能力补齐归一化字段；PVD不进入发布契约</t>
+        </is>
+      </c>
+      <c r="D63" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-28深度审查整改</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="inlineStr">
+        <is>
           <t>R0</t>
         </is>
       </c>
-      <c r="B63" s="11" t="inlineStr">
+      <c r="B64" s="11" t="inlineStr">
         <is>
           <t>硬必填核心(29项，含条件必填)</t>
         </is>
       </c>
-      <c r="C63" s="11" t="inlineStr">
+      <c r="C64" s="11" t="inlineStr">
         <is>
           <t>v3.18删除炉次内重复的前驱体化学式R0；物料身份仍由必填的批次版本快照冻结；其余R0定义不变</t>
         </is>
       </c>
-      <c r="D63" s="11" t="inlineStr">
+      <c r="D64" s="11" t="inlineStr">
         <is>
           <t>必填集</t>
         </is>

</xml_diff>

<commit_message>
fix: close scientific v4 audit blockers
</commit_message>
<xml_diff>
--- a/docs/standard/字段草案-v3.xlsx
+++ b/docs/standard/字段草案-v3.xlsx
@@ -9356,7 +9356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10682,20 +10682,42 @@
     <row r="64">
       <c r="A64" s="11" t="inlineStr">
         <is>
+          <t>v4.0-alpha.2</t>
+        </is>
+      </c>
+      <c r="B64" s="11" t="inlineStr">
+        <is>
+          <t>科学完整性复核</t>
+        </is>
+      </c>
+      <c r="C64" s="11" t="inlineStr">
+        <is>
+          <t>关闭旧结果写入与手工派生入口；收紧审阅和转化权限；修正跨炉次转化溯源、过程单位归一化、不可变修订导出及数据集查询语义；冻结装料容器、测量时校准和样品—修订关联快照；状态降为内部验证</t>
+        </is>
+      </c>
+      <c r="D64" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-29二次复核整改</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="11" t="inlineStr">
+        <is>
           <t>R0</t>
         </is>
       </c>
-      <c r="B64" s="11" t="inlineStr">
+      <c r="B65" s="11" t="inlineStr">
         <is>
           <t>硬必填核心(29项，含条件必填)</t>
         </is>
       </c>
-      <c r="C64" s="11" t="inlineStr">
+      <c r="C65" s="11" t="inlineStr">
         <is>
           <t>v3.18删除炉次内重复的前驱体化学式R0；物料身份仍由必填的批次版本快照冻结；其余R0定义不变</t>
         </is>
       </c>
-      <c r="D64" s="11" t="inlineStr">
+      <c r="D65" s="11" t="inlineStr">
         <is>
           <t>必填集</t>
         </is>

</xml_diff>

<commit_message>
refactor(ui): simplify preparation workflow
</commit_message>
<xml_diff>
--- a/docs/standard/字段草案-v3.xlsx
+++ b/docs/standard/字段草案-v3.xlsx
@@ -550,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K104"/>
+  <dimension ref="A1:K106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3819,47 +3819,83 @@
       </c>
       <c r="K65" s="11" t="inlineStr"/>
     </row>
-    <row r="66" ht="20" customHeight="1">
-      <c r="A66" s="10" t="inlineStr">
-        <is>
-          <t>§5 实验过程（有序记录预处理、反应条件；具名其他记录仅作不丢信息的兜底）</t>
-        </is>
-      </c>
-      <c r="B66" s="8" t="n"/>
-      <c r="C66" s="8" t="n"/>
-      <c r="D66" s="8" t="n"/>
-      <c r="E66" s="8" t="n"/>
-      <c r="F66" s="8" t="n"/>
-      <c r="G66" s="8" t="n"/>
-      <c r="H66" s="8" t="n"/>
-      <c r="I66" s="8" t="n"/>
-      <c r="J66" s="8" t="n"/>
-      <c r="K66" s="8" t="n"/>
+    <row r="66">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t>衬底</t>
+        </is>
+      </c>
+      <c r="B66" s="11" t="inlineStr">
+        <is>
+          <t>轴向位置</t>
+        </is>
+      </c>
+      <c r="C66" s="11" t="inlineStr">
+        <is>
+          <t>本片衬底相对装置轴向原点的位置</t>
+        </is>
+      </c>
+      <c r="D66" s="11" t="inlineStr">
+        <is>
+          <t>数值</t>
+        </is>
+      </c>
+      <c r="E66" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F66" s="11" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="G66" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
+        </is>
+      </c>
+      <c r="H66" s="11" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="I66" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-30产品简化</t>
+        </is>
+      </c>
+      <c r="J66" s="11" t="inlineStr">
+        <is>
+          <t>普通用户只填写装置轴向位置；不暴露三维坐标</t>
+        </is>
+      </c>
+      <c r="K66" s="11" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="11" t="inlineStr">
         <is>
-          <t>过程步</t>
+          <t>衬底</t>
         </is>
       </c>
       <c r="B67" s="11" t="inlineStr">
         <is>
-          <t>记录类型</t>
+          <t>备注</t>
         </is>
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>本条过程记录属于预处理、反应条件或具名其他记录</t>
+          <t>本片衬底摆放或处理的补充说明</t>
         </is>
       </c>
       <c r="D67" s="11" t="inlineStr">
         <is>
-          <t>下拉</t>
+          <t>自由</t>
         </is>
       </c>
       <c r="E67" s="11" t="inlineStr">
         <is>
-          <t>预处理/反应条件/其他记录</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F67" s="11" t="inlineStr">
@@ -3867,120 +3903,80 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G67" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
+      <c r="G67" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
         </is>
       </c>
       <c r="H67" s="11" t="inlineStr">
         <is>
-          <t>反应条件</t>
+          <t>靠近气体入口</t>
         </is>
       </c>
       <c r="I67" s="11" t="inlineStr">
         <is>
-          <t>2026-07-24导师走查</t>
-        </is>
-      </c>
-      <c r="J67" s="11" t="inlineStr">
-        <is>
-          <t>数组顺序即过程顺序；不再重复拆成升温、稳定、生长、退火、降温和卸样</t>
-        </is>
-      </c>
+          <t>2026-07-30产品简化</t>
+        </is>
+      </c>
+      <c r="J67" s="11" t="inlineStr"/>
       <c r="K67" s="11" t="inlineStr"/>
     </row>
-    <row r="68">
-      <c r="A68" s="11" t="inlineStr">
-        <is>
-          <t>过程步</t>
-        </is>
-      </c>
-      <c r="B68" s="11" t="inlineStr">
-        <is>
-          <t>预处理操作</t>
-        </is>
-      </c>
-      <c r="C68" s="11" t="inlineStr">
-        <is>
-          <t>抽气、气路置换等有序可重复的实验前操作</t>
-        </is>
-      </c>
-      <c r="D68" s="11" t="inlineStr">
-        <is>
-          <t>预处理操作数组</t>
-        </is>
-      </c>
-      <c r="E68" s="11" t="inlineStr">
-        <is>
-          <t>{operation_type: 抽气|气路置换|其他, target_absolute_pressure_Pa?, duration_min, cycle_count?, gases?, other_name?, parameters?}</t>
-        </is>
-      </c>
-      <c r="F68" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G68" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(预处理记录)</t>
-        </is>
-      </c>
-      <c r="H68" s="11" t="inlineStr">
-        <is>
-          <t>[{operation_type: 抽气, target_absolute_pressure_Pa: 100, duration_min: 15}]</t>
-        </is>
-      </c>
-      <c r="I68" s="11" t="inlineStr">
-        <is>
-          <t>2026-07-24导师走查</t>
-        </is>
-      </c>
-      <c r="J68" s="11" t="inlineStr">
-        <is>
-          <t>漏率是否逐炉记录待组内确认，本轮不混入抽气字段</t>
-        </is>
-      </c>
-      <c r="K68" s="11" t="inlineStr"/>
+    <row r="68" ht="20" customHeight="1">
+      <c r="A68" s="10" t="inlineStr">
+        <is>
+          <t>§5 实验过程（有序记录预处理、反应条件；具名其他记录仅作不丢信息的兜底）</t>
+        </is>
+      </c>
+      <c r="B68" s="8" t="n"/>
+      <c r="C68" s="8" t="n"/>
+      <c r="D68" s="8" t="n"/>
+      <c r="E68" s="8" t="n"/>
+      <c r="F68" s="8" t="n"/>
+      <c r="G68" s="8" t="n"/>
+      <c r="H68" s="8" t="n"/>
+      <c r="I68" s="8" t="n"/>
+      <c r="J68" s="8" t="n"/>
+      <c r="K68" s="8" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="11" t="inlineStr">
         <is>
-          <t>步·温度</t>
+          <t>过程步</t>
         </is>
       </c>
       <c r="B69" s="11" t="inlineStr">
         <is>
-          <t>设定温度程序</t>
+          <t>记录类型</t>
         </is>
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>各温区按实验起点计时的时间—设定温度点</t>
+          <t>本条过程记录属于预处理、反应条件或具名其他记录</t>
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr">
         <is>
-          <t>分温区温度程序</t>
+          <t>下拉</t>
         </is>
       </c>
       <c r="E69" s="11" t="inlineStr">
         <is>
-          <t>{zones: [{zone_index, points: [{elapsed_min, setpoint_C}]}]}</t>
+          <t>预处理/反应条件/其他记录</t>
         </is>
       </c>
       <c r="F69" s="11" t="inlineStr">
         <is>
-          <t>min·℃</t>
-        </is>
-      </c>
-      <c r="G69" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(反应条件记录)</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G69" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
         </is>
       </c>
       <c r="H69" s="11" t="inlineStr">
         <is>
-          <t>{zones: [{zone_index: 1, points: [{elapsed_min: 0, setpoint_C: 25}, {elapsed_min: 30, setpoint_C: 750}, {elapsed_min: 45, setpoint_C: 750}]}]}</t>
+          <t>反应条件</t>
         </is>
       </c>
       <c r="I69" s="11" t="inlineStr">
@@ -3990,7 +3986,7 @@
       </c>
       <c r="J69" s="11" t="inlineStr">
         <is>
-          <t>每温区时间严格递增且不得超过Setup温区数；相邻同温点表示保温；拒绝任意字符串</t>
+          <t>数组顺序即过程顺序；不再重复拆成升温、稳定、生长、退火、降温和卸样</t>
         </is>
       </c>
       <c r="K69" s="11" t="inlineStr"/>
@@ -3998,42 +3994,42 @@
     <row r="70">
       <c r="A70" s="11" t="inlineStr">
         <is>
-          <t>步·温度</t>
+          <t>过程步</t>
         </is>
       </c>
       <c r="B70" s="11" t="inlineStr">
         <is>
-          <t>实测温度文件与通道</t>
+          <t>预处理操作</t>
         </is>
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>控温实测曲线文件及时间列、温区通道映射；不是估算衬底真温</t>
+          <t>抽气、气路置换等有序可重复的实验前操作</t>
         </is>
       </c>
       <c r="D70" s="11" t="inlineStr">
         <is>
-          <t>温度时序文件引用</t>
+          <t>预处理操作数组</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
         <is>
-          <t>{file_asset_id, time_column, channels: [{zone_index, column_name}]}</t>
+          <t>{operation_type: 抽气|气路置换|其他, target_absolute_pressure_Pa?, duration_min, cycle_count?, gases?, other_name?, parameters?}</t>
         </is>
       </c>
       <c r="F70" s="11" t="inlineStr">
         <is>
-          <t>℃ 随时间</t>
-        </is>
-      </c>
-      <c r="G70" s="15" t="inlineStr">
-        <is>
-          <t>推荐</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G70" s="14" t="inlineStr">
+        <is>
+          <t>条件必填(预处理记录)</t>
         </is>
       </c>
       <c r="H70" s="11" t="inlineStr">
         <is>
-          <t>{file_asset_id: UUID, time_column: elapsed_min, channels: [{zone_index: 1, column_name: zone1_C}]}</t>
+          <t>[{operation_type: 抽气, target_absolute_pressure_Pa: 100, duration_min: 15}]</t>
         </is>
       </c>
       <c r="I70" s="11" t="inlineStr">
@@ -4043,7 +4039,7 @@
       </c>
       <c r="J70" s="11" t="inlineStr">
         <is>
-          <t>文件使用现有FileAsset保存SHA与炉次关联；传感器和不确定度从Setup快照只读带出</t>
+          <t>漏率是否逐炉记录待组内确认，本轮不混入抽气字段</t>
         </is>
       </c>
       <c r="K70" s="11" t="inlineStr"/>
@@ -4051,32 +4047,32 @@
     <row r="71">
       <c r="A71" s="11" t="inlineStr">
         <is>
-          <t>步·气体</t>
+          <t>步·温度</t>
         </is>
       </c>
       <c r="B71" s="11" t="inlineStr">
         <is>
-          <t>逐气体供气程序</t>
+          <t>设定温度程序</t>
         </is>
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>每种气体独立引用气瓶批次并记录一个或多个供气区间</t>
+          <t>各温区按实验起点计时的时间—设定温度点</t>
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr">
         <is>
-          <t>逐气体供气数组</t>
+          <t>分温区温度程序</t>
         </is>
       </c>
       <c r="E71" s="11" t="inlineStr">
         <is>
-          <t>{species, other_name?, lot_ref, measurement_source: MFC|转子|其他, measurement_source_other?, intervals: [{start_min, end_min, flow_sccm}]}</t>
+          <t>{zones: [{zone_index, points: [{elapsed_min, setpoint_C}]}]}</t>
         </is>
       </c>
       <c r="F71" s="11" t="inlineStr">
         <is>
-          <t>min·sccm</t>
+          <t>min·℃</t>
         </is>
       </c>
       <c r="G71" s="14" t="inlineStr">
@@ -4086,7 +4082,7 @@
       </c>
       <c r="H71" s="11" t="inlineStr">
         <is>
-          <t>[{species: Ar, lot_ref: Ar-B01, intervals: [{start_min: 0, end_min: 30, flow_sccm: 80}, {start_min: 45, end_min: 50, flow_sccm: 80}]}]</t>
+          <t>{zones: [{zone_index: 1, points: [{elapsed_min: 0, setpoint_C: 25}, {elapsed_min: 30, setpoint_C: 750}, {elapsed_min: 45, setpoint_C: 750}]}]}</t>
         </is>
       </c>
       <c r="I71" s="11" t="inlineStr">
@@ -4096,7 +4092,7 @@
       </c>
       <c r="J71" s="11" t="inlineStr">
         <is>
-          <t>purity从lot_ref.snapshot带出；区间end_min必须大于start_min；同时间段体积流量占比由各气体流量派生</t>
+          <t>每温区时间严格递增且不得超过Setup温区数；相邻同温点表示保温；拒绝任意字符串</t>
         </is>
       </c>
       <c r="K71" s="11" t="inlineStr"/>
@@ -4104,42 +4100,42 @@
     <row r="72">
       <c r="A72" s="11" t="inlineStr">
         <is>
-          <t>步·压力</t>
+          <t>步·温度</t>
         </is>
       </c>
       <c r="B72" s="11" t="inlineStr">
         <is>
-          <t>压力体系与工作绝对压力</t>
+          <t>实测温度文件与通道</t>
         </is>
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>常压、低压或超高真空类别及工作绝对压力</t>
+          <t>控温实测曲线文件及时间列、温区通道映射；不是估算衬底真温</t>
         </is>
       </c>
       <c r="D72" s="11" t="inlineStr">
         <is>
-          <t>下拉+数值</t>
+          <t>温度时序文件引用</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
         <is>
-          <t>常压(APCVD)/低压(LPCVD)/超高真空</t>
+          <t>{file_asset_id, time_column, channels: [{zone_index, column_name}]}</t>
         </is>
       </c>
       <c r="F72" s="11" t="inlineStr">
         <is>
-          <t>Pa</t>
-        </is>
-      </c>
-      <c r="G72" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(反应条件记录)</t>
+          <t>℃ 随时间</t>
+        </is>
+      </c>
+      <c r="G72" s="15" t="inlineStr">
+        <is>
+          <t>推荐</t>
         </is>
       </c>
       <c r="H72" s="11" t="inlineStr">
         <is>
-          <t>常压；1.01325×10⁵ Pa</t>
+          <t>{file_asset_id: UUID, time_column: elapsed_min, channels: [{zone_index: 1, column_name: zone1_C}]}</t>
         </is>
       </c>
       <c r="I72" s="11" t="inlineStr">
@@ -4149,44 +4145,40 @@
       </c>
       <c r="J72" s="11" t="inlineStr">
         <is>
-          <t>填绝对压力，不填相对大气压的表压</t>
-        </is>
-      </c>
-      <c r="K72" s="11" t="inlineStr">
-        <is>
-          <t>{"gt":0,"option_ranges":{"atmospheric_pressure":{"ge":80000,"le":120000},"low_pressure":{"gt":1e-06,"lt":80000},"ultra_high_vacuum":{"gt":0,"le":1e-06}},"require_option":true,"require_value":true}</t>
-        </is>
-      </c>
+          <t>文件使用现有FileAsset保存SHA与炉次关联；传感器和不确定度从Setup快照只读带出</t>
+        </is>
+      </c>
+      <c r="K72" s="11" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="11" t="inlineStr">
         <is>
-          <t>过程步</t>
+          <t>步·气体</t>
         </is>
       </c>
       <c r="B73" s="11" t="inlineStr">
         <is>
-          <t>反应持续时间</t>
+          <t>逐气体供气程序</t>
         </is>
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>从统一实验时间零点起计的反应条件持续时间</t>
+          <t>每种气体独立引用气瓶批次并记录一个或多个供气区间</t>
         </is>
       </c>
       <c r="D73" s="11" t="inlineStr">
         <is>
-          <t>时长循环对象</t>
+          <t>逐气体供气数组</t>
         </is>
       </c>
       <c r="E73" s="11" t="inlineStr">
         <is>
-          <t>{duration_min；旧记录可含cycle_count}</t>
+          <t>{species, other_name?, lot_ref, measurement_source: MFC|转子|其他, measurement_source_other?, intervals: [{start_min, end_min, flow_sccm}]}</t>
         </is>
       </c>
       <c r="F73" s="11" t="inlineStr">
         <is>
-          <t>min</t>
+          <t>min·sccm</t>
         </is>
       </c>
       <c r="G73" s="14" t="inlineStr">
@@ -4196,17 +4188,17 @@
       </c>
       <c r="H73" s="11" t="inlineStr">
         <is>
-          <t>{duration_min: 45}</t>
+          <t>[{species: Ar, lot_ref: Ar-B01, intervals: [{start_min: 0, end_min: 30, flow_sccm: 80}, {start_min: 45, end_min: 50, flow_sccm: 80}]}]</t>
         </is>
       </c>
       <c r="I73" s="11" t="inlineStr">
         <is>
-          <t>2026-07-24导师走查·2026-07-27终版整改</t>
+          <t>2026-07-24导师走查</t>
         </is>
       </c>
       <c r="J73" s="11" t="inlineStr">
         <is>
-          <t>duration_min&gt;0；历史cycle_count只读兼容，新记录不再把供气区间数解释为反应循环次数</t>
+          <t>purity从lot_ref.snapshot带出；区间end_min必须大于start_min；同时间段体积流量占比由各气体流量派生</t>
         </is>
       </c>
       <c r="K73" s="11" t="inlineStr"/>
@@ -4214,42 +4206,42 @@
     <row r="74">
       <c r="A74" s="11" t="inlineStr">
         <is>
-          <t>步·降温</t>
+          <t>步·压力</t>
         </is>
       </c>
       <c r="B74" s="11" t="inlineStr">
         <is>
-          <t>降温参数</t>
+          <t>压力体系与工作绝对压力</t>
         </is>
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>降温方式以及适用的开盖温度、降温速率</t>
+          <t>常压、低压或超高真空类别及工作绝对压力</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr">
         <is>
-          <t>降温参数对象</t>
+          <t>下拉+数值</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
         <is>
-          <t>{method: 随炉冷却|开盖冷却|移炉快速冷却|其他, lid_open_temperature_C?, cooling_rate_C_per_min?, method_other?}</t>
+          <t>常压(APCVD)/低压(LPCVD)/超高真空</t>
         </is>
       </c>
       <c r="F74" s="11" t="inlineStr">
         <is>
-          <t>℃·℃/min</t>
-        </is>
-      </c>
-      <c r="G74" s="15" t="inlineStr">
-        <is>
-          <t>推荐</t>
+          <t>Pa</t>
+        </is>
+      </c>
+      <c r="G74" s="14" t="inlineStr">
+        <is>
+          <t>条件必填(反应条件记录)</t>
         </is>
       </c>
       <c r="H74" s="11" t="inlineStr">
         <is>
-          <t>{method: 开盖冷却, lid_open_temperature_C: 580, cooling_rate_C_per_min: 20}</t>
+          <t>常压；1.01325×10⁵ Pa</t>
         </is>
       </c>
       <c r="I74" s="11" t="inlineStr">
@@ -4259,60 +4251,64 @@
       </c>
       <c r="J74" s="11" t="inlineStr">
         <is>
-          <t>method=开盖冷却时开盖温度必填；method=其他时method_other必填</t>
-        </is>
-      </c>
-      <c r="K74" s="11" t="inlineStr"/>
+          <t>填绝对压力，不填相对大气压的表压</t>
+        </is>
+      </c>
+      <c r="K74" s="11" t="inlineStr">
+        <is>
+          <t>{"gt":0,"option_ranges":{"atmospheric_pressure":{"ge":80000,"le":120000},"low_pressure":{"gt":1e-06,"lt":80000},"ultra_high_vacuum":{"gt":0,"le":1e-06}},"require_option":true,"require_value":true}</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="11" t="inlineStr">
         <is>
-          <t>步·外场</t>
+          <t>过程步</t>
         </is>
       </c>
       <c r="B75" s="11" t="inlineStr">
         <is>
-          <t>实际外场程序</t>
+          <t>反应持续时间</t>
         </is>
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>本炉实际启用的外场、时间区间与按类型展开的参数</t>
+          <t>从统一实验时间零点起计的反应条件持续时间</t>
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr">
         <is>
-          <t>实际外场数组</t>
+          <t>时长循环对象</t>
         </is>
       </c>
       <c r="E75" s="11" t="inlineStr">
         <is>
-          <t>{field_type: 等离子体|光|电, start_min, end_min, parameters: 等离子体[power_W, gas_species, pressure_Pa]；光[wavelength_nm, power_mW或irradiance_mW_cm2, source_distance_mm]；电[voltage_V或field_strength_V_cm, electrode_gap_mm, direction]；other_parameters?}</t>
+          <t>{duration_min；旧记录可含cycle_count}</t>
         </is>
       </c>
       <c r="F75" s="11" t="inlineStr">
         <is>
-          <t>按参数</t>
-        </is>
-      </c>
-      <c r="G75" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="G75" s="14" t="inlineStr">
+        <is>
+          <t>条件必填(反应条件记录)</t>
         </is>
       </c>
       <c r="H75" s="11" t="inlineStr">
         <is>
-          <t>[{field_type: 等离子体, start_min: 10, end_min: 40, parameters: [{name: power_W, value: 50, unit: W}, {name: gas_species, value: Ar, unit: —}, {name: pressure_Pa, value: 50, unit: Pa}]}]</t>
+          <t>{duration_min: 45}</t>
         </is>
       </c>
       <c r="I75" s="11" t="inlineStr">
         <is>
-          <t>2026-07-24导师走查</t>
+          <t>2026-07-24导师走查·2026-07-27终版整改</t>
         </is>
       </c>
       <c r="J75" s="11" t="inlineStr">
         <is>
-          <t>field_type必须属于Setup能力；界面按类型显示明确字段，其他参数仍使用具名值和单位</t>
+          <t>duration_min&gt;0；历史cycle_count只读兼容，新记录不再把供气区间数解释为反应循环次数</t>
         </is>
       </c>
       <c r="K75" s="11" t="inlineStr"/>
@@ -4320,52 +4316,52 @@
     <row r="76">
       <c r="A76" s="11" t="inlineStr">
         <is>
-          <t>过程步</t>
+          <t>步·降温</t>
         </is>
       </c>
       <c r="B76" s="11" t="inlineStr">
         <is>
-          <t>其他记录名称</t>
+          <t>降温参数</t>
         </is>
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>具名说明未被预处理或反应条件覆盖的过程记录</t>
+          <t>降温方式以及适用的开盖温度、降温速率</t>
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>降温参数对象</t>
         </is>
       </c>
       <c r="E76" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>{method: 随炉冷却|开盖冷却|移炉快速冷却|其他, lid_open_temperature_C?, cooling_rate_C_per_min?, method_other?}</t>
         </is>
       </c>
       <c r="F76" s="11" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G76" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(其他记录)</t>
+          <t>℃·℃/min</t>
+        </is>
+      </c>
+      <c r="G76" s="15" t="inlineStr">
+        <is>
+          <t>推荐</t>
         </is>
       </c>
       <c r="H76" s="11" t="inlineStr">
         <is>
-          <t>临时移动源舟</t>
+          <t>{method: 开盖冷却, lid_open_temperature_C: 580, cooling_rate_C_per_min: 20}</t>
         </is>
       </c>
       <c r="I76" s="11" t="inlineStr">
         <is>
-          <t>2026-07-24整改</t>
+          <t>2026-07-24导师走查</t>
         </is>
       </c>
       <c r="J76" s="11" t="inlineStr">
         <is>
-          <t>禁止仅保存“其他”</t>
+          <t>method=开盖冷却时开盖温度必填；method=其他时method_other必填</t>
         </is>
       </c>
       <c r="K76" s="11" t="inlineStr"/>
@@ -4373,97 +4369,133 @@
     <row r="77">
       <c r="A77" s="11" t="inlineStr">
         <is>
+          <t>步·外场</t>
+        </is>
+      </c>
+      <c r="B77" s="11" t="inlineStr">
+        <is>
+          <t>实际外场程序</t>
+        </is>
+      </c>
+      <c r="C77" s="11" t="inlineStr">
+        <is>
+          <t>本炉实际启用的外场、时间区间与按类型展开的参数</t>
+        </is>
+      </c>
+      <c r="D77" s="11" t="inlineStr">
+        <is>
+          <t>实际外场数组</t>
+        </is>
+      </c>
+      <c r="E77" s="11" t="inlineStr">
+        <is>
+          <t>{field_type: 等离子体|光|电, start_min, end_min, parameters: 等离子体[power_W, gas_species, pressure_Pa]；光[wavelength_nm, power_mW或irradiance_mW_cm2, source_distance_mm]；电[voltage_V或field_strength_V_cm, electrode_gap_mm, direction]；other_parameters?}</t>
+        </is>
+      </c>
+      <c r="F77" s="11" t="inlineStr">
+        <is>
+          <t>按参数</t>
+        </is>
+      </c>
+      <c r="G77" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
+        </is>
+      </c>
+      <c r="H77" s="11" t="inlineStr">
+        <is>
+          <t>[{field_type: 等离子体, start_min: 10, end_min: 40, parameters: [{name: power_W, value: 50, unit: W}, {name: gas_species, value: Ar, unit: —}, {name: pressure_Pa, value: 50, unit: Pa}]}]</t>
+        </is>
+      </c>
+      <c r="I77" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-24导师走查</t>
+        </is>
+      </c>
+      <c r="J77" s="11" t="inlineStr">
+        <is>
+          <t>field_type必须属于Setup能力；界面按类型显示明确字段，其他参数仍使用具名值和单位</t>
+        </is>
+      </c>
+      <c r="K77" s="11" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="11" t="inlineStr">
+        <is>
           <t>过程步</t>
         </is>
       </c>
-      <c r="B77" s="11" t="inlineStr">
-        <is>
-          <t>其他记录说明</t>
-        </is>
-      </c>
-      <c r="C77" s="11" t="inlineStr">
-        <is>
-          <t>说明该记录的时间、操作和必要参数</t>
-        </is>
-      </c>
-      <c r="D77" s="11" t="inlineStr">
-        <is>
-          <t>自由</t>
-        </is>
-      </c>
-      <c r="E77" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F77" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G77" s="14" t="inlineStr">
+      <c r="B78" s="11" t="inlineStr">
+        <is>
+          <t>其他记录名称</t>
+        </is>
+      </c>
+      <c r="C78" s="11" t="inlineStr">
+        <is>
+          <t>具名说明未被预处理或反应条件覆盖的过程记录</t>
+        </is>
+      </c>
+      <c r="D78" s="11" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="E78" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F78" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G78" s="14" t="inlineStr">
         <is>
           <t>条件必填(其他记录)</t>
         </is>
       </c>
-      <c r="H77" s="11" t="inlineStr">
-        <is>
-          <t>第30分钟将源舟向下游移动10 mm</t>
-        </is>
-      </c>
-      <c r="I77" s="11" t="inlineStr">
+      <c r="H78" s="11" t="inlineStr">
+        <is>
+          <t>临时移动源舟</t>
+        </is>
+      </c>
+      <c r="I78" s="11" t="inlineStr">
         <is>
           <t>2026-07-24整改</t>
         </is>
       </c>
-      <c r="J77" s="11" t="inlineStr">
-        <is>
-          <t>必须持久化，绝不静默过滤</t>
-        </is>
-      </c>
-      <c r="K77" s="11" t="inlineStr"/>
-    </row>
-    <row r="78" ht="20" customHeight="1">
-      <c r="A78" s="10" t="inlineStr">
-        <is>
-          <t>§6 过程事件 Process Events（记录异常、中断与人工干预等客观事件；只记客观事实，不判成败）</t>
-        </is>
-      </c>
-      <c r="B78" s="8" t="n"/>
-      <c r="C78" s="8" t="n"/>
-      <c r="D78" s="8" t="n"/>
-      <c r="E78" s="8" t="n"/>
-      <c r="F78" s="8" t="n"/>
-      <c r="G78" s="8" t="n"/>
-      <c r="H78" s="8" t="n"/>
-      <c r="I78" s="8" t="n"/>
-      <c r="J78" s="8" t="n"/>
-      <c r="K78" s="8" t="n"/>
+      <c r="J78" s="11" t="inlineStr">
+        <is>
+          <t>禁止仅保存“其他”</t>
+        </is>
+      </c>
+      <c r="K78" s="11" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="11" t="inlineStr">
         <is>
-          <t>过程事件</t>
+          <t>过程步</t>
         </is>
       </c>
       <c r="B79" s="11" t="inlineStr">
         <is>
-          <t>事件编号</t>
+          <t>其他记录说明</t>
         </is>
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>每条事件稳定且不可重复的标识，用于关联附件</t>
+          <t>说明该记录的时间、操作和必要参数</t>
         </is>
       </c>
       <c r="D79" s="11" t="inlineStr">
         <is>
-          <t>UUID</t>
+          <t>自由</t>
         </is>
       </c>
       <c r="E79" s="11" t="inlineStr">
         <is>
-          <t>系统生成</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F79" s="11" t="inlineStr">
@@ -4471,14 +4503,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G79" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
+      <c r="G79" s="14" t="inlineStr">
+        <is>
+          <t>条件必填(其他记录)</t>
         </is>
       </c>
       <c r="H79" s="11" t="inlineStr">
         <is>
-          <t>550e8400-e29b-41d4-a716-446655440000</t>
+          <t>第30分钟将源舟向下游移动10 mm</t>
         </is>
       </c>
       <c r="I79" s="11" t="inlineStr">
@@ -4488,63 +4520,27 @@
       </c>
       <c r="J79" s="11" t="inlineStr">
         <is>
-          <t>创建事件时生成，排序和编辑不得改变</t>
+          <t>必须持久化，绝不静默过滤</t>
         </is>
       </c>
       <c r="K79" s="11" t="inlineStr"/>
     </row>
-    <row r="80">
-      <c r="A80" s="11" t="inlineStr">
-        <is>
-          <t>过程事件</t>
-        </is>
-      </c>
-      <c r="B80" s="11" t="inlineStr">
-        <is>
-          <t>事件</t>
-        </is>
-      </c>
-      <c r="C80" s="11" t="inlineStr">
-        <is>
-          <t>过程中发生的客观事件类型</t>
-        </is>
-      </c>
-      <c r="D80" s="11" t="inlineStr">
-        <is>
-          <t>下拉+其他</t>
-        </is>
-      </c>
-      <c r="E80" s="11" t="inlineStr">
-        <is>
-          <t>供电中断/供水中断/供气中断/管路堵塞/压力突变/信号异常/人工干预/设备报警/其他</t>
-        </is>
-      </c>
-      <c r="F80" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G80" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
-        </is>
-      </c>
-      <c r="H80" s="11" t="inlineStr">
-        <is>
-          <t>供气中断</t>
-        </is>
-      </c>
-      <c r="I80" s="11" t="inlineStr">
-        <is>
-          <t>2026-07-24导师走查</t>
-        </is>
-      </c>
-      <c r="J80" s="11" t="inlineStr">
-        <is>
-          <t>选择其他时必须填写明确事件名称；不再把事件与部位揉成一个值</t>
-        </is>
-      </c>
-      <c r="K80" s="11" t="inlineStr"/>
+    <row r="80" ht="20" customHeight="1">
+      <c r="A80" s="10" t="inlineStr">
+        <is>
+          <t>§6 过程事件 Process Events（记录异常、中断与人工干预等客观事件；只记客观事实，不判成败）</t>
+        </is>
+      </c>
+      <c r="B80" s="8" t="n"/>
+      <c r="C80" s="8" t="n"/>
+      <c r="D80" s="8" t="n"/>
+      <c r="E80" s="8" t="n"/>
+      <c r="F80" s="8" t="n"/>
+      <c r="G80" s="8" t="n"/>
+      <c r="H80" s="8" t="n"/>
+      <c r="I80" s="8" t="n"/>
+      <c r="J80" s="8" t="n"/>
+      <c r="K80" s="8" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="11" t="inlineStr">
@@ -4554,22 +4550,22 @@
       </c>
       <c r="B81" s="11" t="inlineStr">
         <is>
-          <t>发生时刻</t>
+          <t>事件编号</t>
         </is>
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>何时发生（带 UTC offset 的绝对日期时间，可跨午夜）</t>
+          <t>每条事件稳定且不可重复的标识，用于关联附件</t>
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr">
         <is>
-          <t>日期时间</t>
+          <t>UUID</t>
         </is>
       </c>
       <c r="E81" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>系统生成</t>
         </is>
       </c>
       <c r="F81" s="11" t="inlineStr">
@@ -4584,17 +4580,17 @@
       </c>
       <c r="H81" s="11" t="inlineStr">
         <is>
-          <t>2026-07-24T10:28:00+08:00</t>
+          <t>550e8400-e29b-41d4-a716-446655440000</t>
         </is>
       </c>
       <c r="I81" s="11" t="inlineStr">
         <is>
-          <t>2026-07-24导师走查</t>
+          <t>2026-07-24整改</t>
         </is>
       </c>
       <c r="J81" s="11" t="inlineStr">
         <is>
-          <t>相对时间可由t0算</t>
+          <t>创建事件时生成，排序和编辑不得改变</t>
         </is>
       </c>
       <c r="K81" s="11" t="inlineStr"/>
@@ -4607,22 +4603,22 @@
       </c>
       <c r="B82" s="11" t="inlineStr">
         <is>
-          <t>是否导致实验终止</t>
+          <t>事件</t>
         </is>
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>该事件是否导致本炉实验提前终止</t>
+          <t>过程中发生的客观事件类型</t>
         </is>
       </c>
       <c r="D82" s="11" t="inlineStr">
         <is>
-          <t>复选</t>
+          <t>下拉+其他</t>
         </is>
       </c>
       <c r="E82" s="11" t="inlineStr">
         <is>
-          <t>是/否</t>
+          <t>供电中断/供水中断/供气中断/管路堵塞/压力突变/信号异常/人工干预/设备报警/其他</t>
         </is>
       </c>
       <c r="F82" s="11" t="inlineStr">
@@ -4637,7 +4633,7 @@
       </c>
       <c r="H82" s="11" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>供气中断</t>
         </is>
       </c>
       <c r="I82" s="11" t="inlineStr">
@@ -4647,7 +4643,7 @@
       </c>
       <c r="J82" s="11" t="inlineStr">
         <is>
-          <t>客观记录，不等同于成败判断</t>
+          <t>选择其他时必须填写明确事件名称；不再把事件与部位揉成一个值</t>
         </is>
       </c>
       <c r="K82" s="11" t="inlineStr"/>
@@ -4660,22 +4656,22 @@
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
-          <t>终止原因</t>
+          <t>发生时刻</t>
         </is>
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>事件导致实验终止时的客观原因</t>
+          <t>何时发生（带 UTC offset 的绝对日期时间，可跨午夜）</t>
         </is>
       </c>
       <c r="D83" s="11" t="inlineStr">
         <is>
-          <t>下拉</t>
+          <t>日期时间</t>
         </is>
       </c>
       <c r="E83" s="11" t="inlineStr">
         <is>
-          <t>设备报警/人工停止/计划变更/其他</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F83" s="11" t="inlineStr">
@@ -4683,14 +4679,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G83" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(导致实验终止)</t>
+      <c r="G83" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
         </is>
       </c>
       <c r="H83" s="11" t="inlineStr">
         <is>
-          <t>设备报警</t>
+          <t>2026-07-24T10:28:00+08:00</t>
         </is>
       </c>
       <c r="I83" s="11" t="inlineStr">
@@ -4700,7 +4696,7 @@
       </c>
       <c r="J83" s="11" t="inlineStr">
         <is>
-          <t>正常计划结束不是异常终止原因</t>
+          <t>相对时间可由t0算</t>
         </is>
       </c>
       <c r="K83" s="11" t="inlineStr"/>
@@ -4713,22 +4709,22 @@
       </c>
       <c r="B84" s="11" t="inlineStr">
         <is>
-          <t>事件具体说明</t>
+          <t>是否导致实验终止</t>
         </is>
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>事件现象、涉及对象和上下文</t>
+          <t>该事件是否导致本炉实验提前终止</t>
         </is>
       </c>
       <c r="D84" s="11" t="inlineStr">
         <is>
-          <t>自由</t>
+          <t>复选</t>
         </is>
       </c>
       <c r="E84" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>是/否</t>
         </is>
       </c>
       <c r="F84" s="11" t="inlineStr">
@@ -4736,14 +4732,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G84" s="16" t="inlineStr">
-        <is>
-          <t>选填；终止原因=其他时必填</t>
+      <c r="G84" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
         </is>
       </c>
       <c r="H84" s="11" t="inlineStr">
         <is>
-          <t>Ar气瓶压力不足，供气中断约2分钟</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I84" s="11" t="inlineStr">
@@ -4753,7 +4749,7 @@
       </c>
       <c r="J84" s="11" t="inlineStr">
         <is>
-          <t>始终可选填写事件上下文，不与处理措施或附件拼接；终止原因选择“其他”时必须具名说明</t>
+          <t>客观记录，不等同于成败判断</t>
         </is>
       </c>
       <c r="K84" s="11" t="inlineStr"/>
@@ -4766,22 +4762,22 @@
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>处理措施</t>
+          <t>终止原因</t>
         </is>
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>事件发生后采取的操作</t>
+          <t>事件导致实验终止时的客观原因</t>
         </is>
       </c>
       <c r="D85" s="11" t="inlineStr">
         <is>
-          <t>自由</t>
+          <t>下拉</t>
         </is>
       </c>
       <c r="E85" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>设备报警/人工停止/计划变更/其他</t>
         </is>
       </c>
       <c r="F85" s="11" t="inlineStr">
@@ -4789,14 +4785,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G85" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
+      <c r="G85" s="14" t="inlineStr">
+        <is>
+          <t>条件必填(导致实验终止)</t>
         </is>
       </c>
       <c r="H85" s="11" t="inlineStr">
         <is>
-          <t>更换气瓶后恢复供气</t>
+          <t>设备报警</t>
         </is>
       </c>
       <c r="I85" s="11" t="inlineStr">
@@ -4806,7 +4802,7 @@
       </c>
       <c r="J85" s="11" t="inlineStr">
         <is>
-          <t>与事件说明独立保存</t>
+          <t>正常计划结束不是异常终止原因</t>
         </is>
       </c>
       <c r="K85" s="11" t="inlineStr"/>
@@ -4819,22 +4815,22 @@
       </c>
       <c r="B86" s="11" t="inlineStr">
         <is>
-          <t>事件附件</t>
+          <t>事件具体说明</t>
         </is>
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
-          <t>与本条事件直接关联的图片、日志或其他文件</t>
+          <t>事件现象、涉及对象和上下文</t>
         </is>
       </c>
       <c r="D86" s="11" t="inlineStr">
         <is>
-          <t>FileAsset引用数组</t>
+          <t>自由</t>
         </is>
       </c>
       <c r="E86" s="11" t="inlineStr">
         <is>
-          <t>FileAsset UUID列表</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F86" s="11" t="inlineStr">
@@ -4844,67 +4840,103 @@
       </c>
       <c r="G86" s="16" t="inlineStr">
         <is>
+          <t>选填；终止原因=其他时必填</t>
+        </is>
+      </c>
+      <c r="H86" s="11" t="inlineStr">
+        <is>
+          <t>Ar气瓶压力不足，供气中断约2分钟</t>
+        </is>
+      </c>
+      <c r="I86" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-24导师走查</t>
+        </is>
+      </c>
+      <c r="J86" s="11" t="inlineStr">
+        <is>
+          <t>始终可选填写事件上下文，不与处理措施或附件拼接；终止原因选择“其他”时必须具名说明</t>
+        </is>
+      </c>
+      <c r="K86" s="11" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="11" t="inlineStr">
+        <is>
+          <t>过程事件</t>
+        </is>
+      </c>
+      <c r="B87" s="11" t="inlineStr">
+        <is>
+          <t>处理措施</t>
+        </is>
+      </c>
+      <c r="C87" s="11" t="inlineStr">
+        <is>
+          <t>事件发生后采取的操作</t>
+        </is>
+      </c>
+      <c r="D87" s="11" t="inlineStr">
+        <is>
+          <t>自由</t>
+        </is>
+      </c>
+      <c r="E87" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F87" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G87" s="16" t="inlineStr">
+        <is>
           <t>选填</t>
         </is>
       </c>
-      <c r="H86" s="11" t="inlineStr">
-        <is>
-          <t>[550e8400-e29b-41d4-a716-446655440001]</t>
-        </is>
-      </c>
-      <c r="I86" s="11" t="inlineStr">
+      <c r="H87" s="11" t="inlineStr">
+        <is>
+          <t>更换气瓶后恢复供气</t>
+        </is>
+      </c>
+      <c r="I87" s="11" t="inlineStr">
         <is>
           <t>2026-07-24导师走查</t>
         </is>
       </c>
-      <c r="J86" s="11" t="inlineStr">
-        <is>
-          <t>文件必须属于同一炉次且asset_role=process_event_attachment</t>
-        </is>
-      </c>
-      <c r="K86" s="11" t="inlineStr"/>
-    </row>
-    <row r="87" ht="20" customHeight="1">
-      <c r="A87" s="10" t="inlineStr">
-        <is>
-          <t>§7 旧扁平结果字段（未发布；由 MeasurementRun → AnalysisRun → PropertyValue / MaterialAssertion 替代）</t>
-        </is>
-      </c>
-      <c r="B87" s="8" t="n"/>
-      <c r="C87" s="8" t="n"/>
-      <c r="D87" s="8" t="n"/>
-      <c r="E87" s="8" t="n"/>
-      <c r="F87" s="8" t="n"/>
-      <c r="G87" s="8" t="n"/>
-      <c r="H87" s="8" t="n"/>
-      <c r="I87" s="8" t="n"/>
-      <c r="J87" s="8" t="n"/>
-      <c r="K87" s="8" t="n"/>
+      <c r="J87" s="11" t="inlineStr">
+        <is>
+          <t>与事件说明独立保存</t>
+        </is>
+      </c>
+      <c r="K87" s="11" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="11" t="inlineStr">
         <is>
-          <t>表征</t>
+          <t>过程事件</t>
         </is>
       </c>
       <c r="B88" s="11" t="inlineStr">
         <is>
-          <t>表征方法</t>
+          <t>事件附件</t>
         </is>
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>本次使用的表征手段；仪器通过独立仪器引用选择</t>
+          <t>与本条事件直接关联的图片、日志或其他文件</t>
         </is>
       </c>
       <c r="D88" s="11" t="inlineStr">
         <is>
-          <t>下拉+其他</t>
+          <t>FileAsset引用数组</t>
         </is>
       </c>
       <c r="E88" s="11" t="inlineStr">
         <is>
-          <t>光镜/SEM/Raman/低波数Raman/PL/AFM/XRD/TEM/其他</t>
+          <t>FileAsset UUID列表</t>
         </is>
       </c>
       <c r="F88" s="11" t="inlineStr">
@@ -4914,78 +4946,42 @@
       </c>
       <c r="G88" s="16" t="inlineStr">
         <is>
-          <t>未发布</t>
+          <t>选填</t>
         </is>
       </c>
       <c r="H88" s="11" t="inlineStr">
         <is>
-          <t>Raman</t>
+          <t>[550e8400-e29b-41d4-a716-446655440001]</t>
         </is>
       </c>
       <c r="I88" s="11" t="inlineStr">
         <is>
-          <t>会议</t>
-        </is>
-      </c>
-      <c r="J88" s="13" t="inlineStr">
-        <is>
-          <t>★v3：长一批表征一批，拆成独立表编号关联；不要在此字段重复写仪器</t>
+          <t>2026-07-24导师走查</t>
+        </is>
+      </c>
+      <c r="J88" s="11" t="inlineStr">
+        <is>
+          <t>文件必须属于同一炉次且asset_role=process_event_attachment</t>
         </is>
       </c>
       <c r="K88" s="11" t="inlineStr"/>
     </row>
-    <row r="89">
-      <c r="A89" s="11" t="inlineStr">
-        <is>
-          <t>表征</t>
-        </is>
-      </c>
-      <c r="B89" s="11" t="inlineStr">
-        <is>
-          <t>测试条件</t>
-        </is>
-      </c>
-      <c r="C89" s="11" t="inlineStr">
-        <is>
-          <t>该表征的测试参数</t>
-        </is>
-      </c>
-      <c r="D89" s="11" t="inlineStr">
-        <is>
-          <t>文本/自由</t>
-        </is>
-      </c>
-      <c r="E89" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F89" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G89" s="16" t="inlineStr">
-        <is>
-          <t>未发布</t>
-        </is>
-      </c>
-      <c r="H89" s="11" t="inlineStr">
-        <is>
-          <t>激光532 nm；功率1 mW；物镜100×</t>
-        </is>
-      </c>
-      <c r="I89" s="11" t="inlineStr">
-        <is>
-          <t>会议</t>
-        </is>
-      </c>
-      <c r="J89" s="11" t="inlineStr">
-        <is>
-          <t>随仪器导出</t>
-        </is>
-      </c>
-      <c r="K89" s="11" t="inlineStr"/>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="10" t="inlineStr">
+        <is>
+          <t>§7 旧扁平结果字段（未发布；由 MeasurementRun → AnalysisRun → PropertyValue / MaterialAssertion 替代）</t>
+        </is>
+      </c>
+      <c r="B89" s="8" t="n"/>
+      <c r="C89" s="8" t="n"/>
+      <c r="D89" s="8" t="n"/>
+      <c r="E89" s="8" t="n"/>
+      <c r="F89" s="8" t="n"/>
+      <c r="G89" s="8" t="n"/>
+      <c r="H89" s="8" t="n"/>
+      <c r="I89" s="8" t="n"/>
+      <c r="J89" s="8" t="n"/>
+      <c r="K89" s="8" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="11" t="inlineStr">
@@ -4995,22 +4991,22 @@
       </c>
       <c r="B90" s="11" t="inlineStr">
         <is>
-          <t>原始数据</t>
+          <t>表征方法</t>
         </is>
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>上传原始文件（留校验和）</t>
+          <t>本次使用的表征手段；仪器通过独立仪器引用选择</t>
         </is>
       </c>
       <c r="D90" s="11" t="inlineStr">
         <is>
-          <t>附件</t>
+          <t>下拉+其他</t>
         </is>
       </c>
       <c r="E90" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>光镜/SEM/Raman/低波数Raman/PL/AFM/XRD/TEM/其他</t>
         </is>
       </c>
       <c r="F90" s="11" t="inlineStr">
@@ -5025,41 +5021,45 @@
       </c>
       <c r="H90" s="11" t="inlineStr">
         <is>
-          <t>raman.txt</t>
+          <t>Raman</t>
         </is>
       </c>
       <c r="I90" s="11" t="inlineStr">
         <is>
-          <t>会议/复审</t>
-        </is>
-      </c>
-      <c r="J90" s="11" t="inlineStr"/>
+          <t>会议</t>
+        </is>
+      </c>
+      <c r="J90" s="13" t="inlineStr">
+        <is>
+          <t>★v3：长一批表征一批，拆成独立表编号关联；不要在此字段重复写仪器</t>
+        </is>
+      </c>
       <c r="K90" s="11" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="11" t="inlineStr">
         <is>
-          <t>实测产物</t>
+          <t>表征</t>
         </is>
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
-          <t>观察到的现象</t>
+          <t>测试条件</t>
         </is>
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>光镜可判的客观现象（非成败判断）</t>
+          <t>该表征的测试参数</t>
         </is>
       </c>
       <c r="D91" s="11" t="inlineStr">
         <is>
-          <t>下拉+多选</t>
+          <t>文本/自由</t>
         </is>
       </c>
       <c r="E91" s="11" t="inlineStr">
         <is>
-          <t>无生长/不连续覆盖/厚层区域/可见颗粒沾污/衬底破损/变色/其他</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F91" s="11" t="inlineStr">
@@ -5074,17 +5074,17 @@
       </c>
       <c r="H91" s="11" t="inlineStr">
         <is>
-          <t>不连续覆盖</t>
+          <t>激光532 nm；功率1 mW；物镜100×</t>
         </is>
       </c>
       <c r="I91" s="11" t="inlineStr">
         <is>
-          <t>复审</t>
-        </is>
-      </c>
-      <c r="J91" s="13" t="inlineStr">
-        <is>
-          <t>★失败炉次最小痕迹；终态无任何结果→『结果缺失』待办(标准§7/§10)</t>
+          <t>会议</t>
+        </is>
+      </c>
+      <c r="J91" s="11" t="inlineStr">
+        <is>
+          <t>随仪器导出</t>
         </is>
       </c>
       <c r="K91" s="11" t="inlineStr"/>
@@ -5092,22 +5092,22 @@
     <row r="92">
       <c r="A92" s="11" t="inlineStr">
         <is>
-          <t>实测产物</t>
+          <t>表征</t>
         </is>
       </c>
       <c r="B92" s="11" t="inlineStr">
         <is>
-          <t>检出相、多型与堆垛</t>
+          <t>原始数据</t>
         </is>
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>测到的物相/多型/堆垛类型</t>
+          <t>上传原始文件（留校验和）</t>
         </is>
       </c>
       <c r="D92" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>附件</t>
         </is>
       </c>
       <c r="E92" s="11" t="inlineStr">
@@ -5127,19 +5127,15 @@
       </c>
       <c r="H92" s="11" t="inlineStr">
         <is>
-          <t>2H-MoS₂；AB堆垛</t>
+          <t>raman.txt</t>
         </is>
       </c>
       <c r="I92" s="11" t="inlineStr">
         <is>
-          <t>复审/导师</t>
-        </is>
-      </c>
-      <c r="J92" s="13" t="inlineStr">
-        <is>
-          <t>★v3.4导师评审(B76红字)：增记堆垛类型（可判粒度待与俊杰确认，或改下拉）；最小结构化结果</t>
-        </is>
-      </c>
+          <t>会议/复审</t>
+        </is>
+      </c>
+      <c r="J92" s="11" t="inlineStr"/>
       <c r="K92" s="11" t="inlineStr"/>
     </row>
     <row r="93">
@@ -5150,27 +5146,27 @@
       </c>
       <c r="B93" s="11" t="inlineStr">
         <is>
-          <t>实测层数</t>
+          <t>观察到的现象</t>
         </is>
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>由表征方法判定的层数</t>
+          <t>光镜可判的客观现象（非成败判断）</t>
         </is>
       </c>
       <c r="D93" s="11" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>下拉+多选</t>
         </is>
       </c>
       <c r="E93" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>无生长/不连续覆盖/厚层区域/可见颗粒沾污/衬底破损/变色/其他</t>
         </is>
       </c>
       <c r="F93" s="11" t="inlineStr">
         <is>
-          <t>层</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G93" s="16" t="inlineStr">
@@ -5180,24 +5176,20 @@
       </c>
       <c r="H93" s="11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>不连续覆盖</t>
         </is>
       </c>
       <c r="I93" s="11" t="inlineStr">
         <is>
-          <t>复审/科学契约审查</t>
-        </is>
-      </c>
-      <c r="J93" s="11" t="inlineStr">
-        <is>
-          <t>仅作为 MaterialAssertion.layer_count 录入，不生成 PropertyValue；与覆盖率拆分，0 表示在该测点未检出层状产物</t>
-        </is>
-      </c>
-      <c r="K93" s="11" t="inlineStr">
-        <is>
-          <t>{"ge":0,"type":"integer"}</t>
-        </is>
-      </c>
+          <t>复审</t>
+        </is>
+      </c>
+      <c r="J93" s="13" t="inlineStr">
+        <is>
+          <t>★失败炉次最小痕迹；终态无任何结果→『结果缺失』待办(标准§7/§10)</t>
+        </is>
+      </c>
+      <c r="K93" s="11" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="11" t="inlineStr">
@@ -5207,17 +5199,17 @@
       </c>
       <c r="B94" s="11" t="inlineStr">
         <is>
-          <t>覆盖率</t>
+          <t>检出相、多型与堆垛</t>
         </is>
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
-          <t>明确视场或统计区域内材料面积占比</t>
+          <t>测到的物相/多型/堆垛类型</t>
         </is>
       </c>
       <c r="D94" s="11" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E94" s="11" t="inlineStr">
@@ -5227,7 +5219,7 @@
       </c>
       <c r="F94" s="11" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G94" s="16" t="inlineStr">
@@ -5237,24 +5229,20 @@
       </c>
       <c r="H94" s="11" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>2H-MoS₂；AB堆垛</t>
         </is>
       </c>
       <c r="I94" s="11" t="inlineStr">
         <is>
-          <t>复审/科学契约审查</t>
-        </is>
-      </c>
-      <c r="J94" s="11" t="inlineStr">
-        <is>
-          <t>量化口径仍须随表征条件记录</t>
-        </is>
-      </c>
-      <c r="K94" s="11" t="inlineStr">
-        <is>
-          <t>{"ge":0,"le":100}</t>
-        </is>
-      </c>
+          <t>复审/导师</t>
+        </is>
+      </c>
+      <c r="J94" s="13" t="inlineStr">
+        <is>
+          <t>★v3.4导师评审(B76红字)：增记堆垛类型（可判粒度待与俊杰确认，或改下拉）；最小结构化结果</t>
+        </is>
+      </c>
+      <c r="K94" s="11" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="11" t="inlineStr">
@@ -5264,12 +5252,12 @@
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
-          <t>畴尺寸</t>
+          <t>实测层数</t>
         </is>
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>由指定统计方法得到的代表性畴尺寸</t>
+          <t>由表征方法判定的层数</t>
         </is>
       </c>
       <c r="D95" s="11" t="inlineStr">
@@ -5284,7 +5272,7 @@
       </c>
       <c r="F95" s="11" t="inlineStr">
         <is>
-          <t>μm</t>
+          <t>层</t>
         </is>
       </c>
       <c r="G95" s="16" t="inlineStr">
@@ -5294,7 +5282,7 @@
       </c>
       <c r="H95" s="11" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I95" s="11" t="inlineStr">
@@ -5302,10 +5290,14 @@
           <t>复审/科学契约审查</t>
         </is>
       </c>
-      <c r="J95" s="11" t="inlineStr"/>
+      <c r="J95" s="11" t="inlineStr">
+        <is>
+          <t>仅作为 MaterialAssertion.layer_count 录入，不生成 PropertyValue；与覆盖率拆分，0 表示在该测点未检出层状产物</t>
+        </is>
+      </c>
       <c r="K95" s="11" t="inlineStr">
         <is>
-          <t>{"gt":0}</t>
+          <t>{"ge":0,"type":"integer"}</t>
         </is>
       </c>
     </row>
@@ -5317,12 +5309,12 @@
       </c>
       <c r="B96" s="11" t="inlineStr">
         <is>
-          <t>成核密度</t>
+          <t>覆盖率</t>
         </is>
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
-          <t>指定统计区域内单位面积成核点数量</t>
+          <t>明确视场或统计区域内材料面积占比</t>
         </is>
       </c>
       <c r="D96" s="11" t="inlineStr">
@@ -5337,7 +5329,7 @@
       </c>
       <c r="F96" s="11" t="inlineStr">
         <is>
-          <t>cm⁻²</t>
+          <t>%</t>
         </is>
       </c>
       <c r="G96" s="16" t="inlineStr">
@@ -5347,7 +5339,7 @@
       </c>
       <c r="H96" s="11" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>70</t>
         </is>
       </c>
       <c r="I96" s="11" t="inlineStr">
@@ -5355,10 +5347,14 @@
           <t>复审/科学契约审查</t>
         </is>
       </c>
-      <c r="J96" s="11" t="inlineStr"/>
+      <c r="J96" s="11" t="inlineStr">
+        <is>
+          <t>量化口径仍须随表征条件记录</t>
+        </is>
+      </c>
       <c r="K96" s="11" t="inlineStr">
         <is>
-          <t>{"ge":0}</t>
+          <t>{"ge":0,"le":100}</t>
         </is>
       </c>
     </row>
@@ -5370,27 +5366,27 @@
       </c>
       <c r="B97" s="11" t="inlineStr">
         <is>
-          <t>关键谱学指标</t>
+          <t>畴尺寸</t>
         </is>
       </c>
       <c r="C97" s="11" t="inlineStr">
         <is>
-          <t>Raman峰位/峰宽/峰面积；PL峰位/峰宽；AFM厚度/粗糙度；SEM覆盖率(视场内材料面积占比,%)/尺寸</t>
+          <t>由指定统计方法得到的代表性畴尺寸</t>
         </is>
       </c>
       <c r="D97" s="11" t="inlineStr">
         <is>
-          <t>结构化指标数组</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="E97" s="11" t="inlineStr">
         <is>
-          <t>每条:{metric_code,value,unit}</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F97" s="11" t="inlineStr">
         <is>
-          <t>按指标</t>
+          <t>μm</t>
         </is>
       </c>
       <c r="G97" s="16" t="inlineStr">
@@ -5400,71 +5396,103 @@
       </c>
       <c r="H97" s="11" t="inlineStr">
         <is>
-          <t>[{"metric_code":"raman_e2g_peak","value":384.2,"unit":"cm-1"}]</t>
+          <t>50</t>
         </is>
       </c>
       <c r="I97" s="11" t="inlineStr">
         <is>
-          <t>复审/导师</t>
-        </is>
-      </c>
-      <c r="J97" s="13" t="inlineStr">
-        <is>
-          <t>★v3.4导师评审(C79红字/K79)：PL补峰宽；『SEM占比』改名『SEM覆盖率』并给定义；随技术选填</t>
-        </is>
-      </c>
+          <t>复审/科学契约审查</t>
+        </is>
+      </c>
+      <c r="J97" s="11" t="inlineStr"/>
       <c r="K97" s="11" t="inlineStr">
         <is>
-          <t>{"finite_value":true,"item_required":["metric_code","value","unit"]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="20" customHeight="1">
-      <c r="A98" s="10" t="inlineStr">
-        <is>
-          <t>§8 PVD 专用（若合成方法选 PVD 类才启用；延后实现，先占位）</t>
-        </is>
-      </c>
-      <c r="B98" s="8" t="n"/>
-      <c r="C98" s="8" t="n"/>
-      <c r="D98" s="8" t="n"/>
-      <c r="E98" s="8" t="n"/>
-      <c r="F98" s="8" t="n"/>
-      <c r="G98" s="8" t="n"/>
-      <c r="H98" s="8" t="n"/>
-      <c r="I98" s="8" t="n"/>
-      <c r="J98" s="8" t="n"/>
-      <c r="K98" s="8" t="n"/>
+          <t>{"gt":0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="11" t="inlineStr">
+        <is>
+          <t>实测产物</t>
+        </is>
+      </c>
+      <c r="B98" s="11" t="inlineStr">
+        <is>
+          <t>成核密度</t>
+        </is>
+      </c>
+      <c r="C98" s="11" t="inlineStr">
+        <is>
+          <t>指定统计区域内单位面积成核点数量</t>
+        </is>
+      </c>
+      <c r="D98" s="11" t="inlineStr">
+        <is>
+          <t>数值</t>
+        </is>
+      </c>
+      <c r="E98" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F98" s="11" t="inlineStr">
+        <is>
+          <t>cm⁻²</t>
+        </is>
+      </c>
+      <c r="G98" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
+        </is>
+      </c>
+      <c r="H98" s="11" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="I98" s="11" t="inlineStr">
+        <is>
+          <t>复审/科学契约审查</t>
+        </is>
+      </c>
+      <c r="J98" s="11" t="inlineStr"/>
+      <c r="K98" s="11" t="inlineStr">
+        <is>
+          <t>{"ge":0}</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="11" t="inlineStr">
         <is>
-          <t>PVD</t>
+          <t>实测产物</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>靶材（批次）</t>
+          <t>关键谱学指标</t>
         </is>
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>靶材化学身份 + 批次</t>
+          <t>Raman峰位/峰宽/峰面积；PL峰位/峰宽；AFM厚度/粗糙度；SEM覆盖率(视场内材料面积占比,%)/尺寸</t>
         </is>
       </c>
       <c r="D99" s="11" t="inlineStr">
         <is>
-          <t>引用</t>
+          <t>结构化指标数组</t>
         </is>
       </c>
       <c r="E99" s="11" t="inlineStr">
         <is>
-          <t>批次库</t>
+          <t>每条:{metric_code,value,unit}</t>
         </is>
       </c>
       <c r="F99" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>按指标</t>
         </is>
       </c>
       <c r="G99" s="16" t="inlineStr">
@@ -5474,69 +5502,41 @@
       </c>
       <c r="H99" s="11" t="inlineStr">
         <is>
-          <t>MoS₂ 靶-T01</t>
+          <t>[{"metric_code":"raman_e2g_peak","value":384.2,"unit":"cm-1"}]</t>
         </is>
       </c>
       <c r="I99" s="11" t="inlineStr">
         <is>
-          <t>复审</t>
-        </is>
-      </c>
-      <c r="J99" s="11" t="inlineStr"/>
-      <c r="K99" s="11" t="inlineStr"/>
-    </row>
-    <row r="100">
-      <c r="A100" s="11" t="inlineStr">
-        <is>
-          <t>PVD</t>
-        </is>
-      </c>
-      <c r="B100" s="11" t="inlineStr">
-        <is>
-          <t>靶基距</t>
-        </is>
-      </c>
-      <c r="C100" s="11" t="inlineStr">
-        <is>
-          <t>靶到衬底距离</t>
-        </is>
-      </c>
-      <c r="D100" s="11" t="inlineStr">
-        <is>
-          <t>数值</t>
-        </is>
-      </c>
-      <c r="E100" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F100" s="11" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-      <c r="G100" s="16" t="inlineStr">
-        <is>
-          <t>未发布</t>
-        </is>
-      </c>
-      <c r="H100" s="11" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
-      <c r="I100" s="11" t="inlineStr">
-        <is>
-          <t>复审</t>
-        </is>
-      </c>
-      <c r="J100" s="11" t="inlineStr"/>
-      <c r="K100" s="11" t="inlineStr">
-        <is>
-          <t>{"gt":0}</t>
-        </is>
-      </c>
+          <t>复审/导师</t>
+        </is>
+      </c>
+      <c r="J99" s="13" t="inlineStr">
+        <is>
+          <t>★v3.4导师评审(C79红字/K79)：PL补峰宽；『SEM占比』改名『SEM覆盖率』并给定义；随技术选填</t>
+        </is>
+      </c>
+      <c r="K99" s="11" t="inlineStr">
+        <is>
+          <t>{"finite_value":true,"item_required":["metric_code","value","unit"]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="20" customHeight="1">
+      <c r="A100" s="10" t="inlineStr">
+        <is>
+          <t>§8 PVD 专用（若合成方法选 PVD 类才启用；延后实现，先占位）</t>
+        </is>
+      </c>
+      <c r="B100" s="8" t="n"/>
+      <c r="C100" s="8" t="n"/>
+      <c r="D100" s="8" t="n"/>
+      <c r="E100" s="8" t="n"/>
+      <c r="F100" s="8" t="n"/>
+      <c r="G100" s="8" t="n"/>
+      <c r="H100" s="8" t="n"/>
+      <c r="I100" s="8" t="n"/>
+      <c r="J100" s="8" t="n"/>
+      <c r="K100" s="8" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="11" t="inlineStr">
@@ -5546,27 +5546,27 @@
       </c>
       <c r="B101" s="11" t="inlineStr">
         <is>
-          <t>功率与偏压</t>
+          <t>靶材（批次）</t>
         </is>
       </c>
       <c r="C101" s="11" t="inlineStr">
         <is>
-          <t>DC/RF 功率、基底偏压</t>
+          <t>靶材化学身份 + 批次</t>
         </is>
       </c>
       <c r="D101" s="11" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>引用</t>
         </is>
       </c>
       <c r="E101" s="11" t="inlineStr">
         <is>
-          <t>DC/RF</t>
+          <t>批次库</t>
         </is>
       </c>
       <c r="F101" s="11" t="inlineStr">
         <is>
-          <t>W·V</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G101" s="16" t="inlineStr">
@@ -5576,7 +5576,7 @@
       </c>
       <c r="H101" s="11" t="inlineStr">
         <is>
-          <t>RF 150W；偏压 -50V</t>
+          <t>MoS₂ 靶-T01</t>
         </is>
       </c>
       <c r="I101" s="11" t="inlineStr">
@@ -5595,27 +5595,27 @@
       </c>
       <c r="B102" s="11" t="inlineStr">
         <is>
-          <t>等离子体气氛与工作气压</t>
+          <t>靶基距</t>
         </is>
       </c>
       <c r="C102" s="11" t="inlineStr">
         <is>
-          <t>溅射气体与气压</t>
+          <t>靶到衬底距离</t>
         </is>
       </c>
       <c r="D102" s="11" t="inlineStr">
         <is>
-          <t>下拉+数值</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="E102" s="11" t="inlineStr">
         <is>
-          <t>Ar / Ar+N₂…</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F102" s="11" t="inlineStr">
         <is>
-          <t>Pa</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="G102" s="16" t="inlineStr">
@@ -5625,7 +5625,7 @@
       </c>
       <c r="H102" s="11" t="inlineStr">
         <is>
-          <t>Ar，0.5 Pa</t>
+          <t>80</t>
         </is>
       </c>
       <c r="I102" s="11" t="inlineStr">
@@ -5636,7 +5636,7 @@
       <c r="J102" s="11" t="inlineStr"/>
       <c r="K102" s="11" t="inlineStr">
         <is>
-          <t>{"gt":0,"require_value":true}</t>
+          <t>{"gt":0}</t>
         </is>
       </c>
     </row>
@@ -5648,12 +5648,12 @@
       </c>
       <c r="B103" s="11" t="inlineStr">
         <is>
-          <t>预溅射与挡板时序</t>
+          <t>功率与偏压</t>
         </is>
       </c>
       <c r="C103" s="11" t="inlineStr">
         <is>
-          <t>预溅射时长、挡板开合时序</t>
+          <t>DC/RF 功率、基底偏压</t>
         </is>
       </c>
       <c r="D103" s="11" t="inlineStr">
@@ -5663,12 +5663,12 @@
       </c>
       <c r="E103" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DC/RF</t>
         </is>
       </c>
       <c r="F103" s="11" t="inlineStr">
         <is>
-          <t>min·s</t>
+          <t>W·V</t>
         </is>
       </c>
       <c r="G103" s="16" t="inlineStr">
@@ -5678,7 +5678,7 @@
       </c>
       <c r="H103" s="11" t="inlineStr">
         <is>
-          <t>预溅 5 min</t>
+          <t>RF 150W；偏压 -50V</t>
         </is>
       </c>
       <c r="I103" s="11" t="inlineStr">
@@ -5687,11 +5687,7 @@
         </is>
       </c>
       <c r="J103" s="11" t="inlineStr"/>
-      <c r="K103" s="11" t="inlineStr">
-        <is>
-          <t>{"gt":0}</t>
-        </is>
-      </c>
+      <c r="K103" s="11" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="11" t="inlineStr">
@@ -5701,27 +5697,27 @@
       </c>
       <c r="B104" s="11" t="inlineStr">
         <is>
-          <t>沉积速率</t>
+          <t>等离子体气氛与工作气压</t>
         </is>
       </c>
       <c r="C104" s="11" t="inlineStr">
         <is>
-          <t>速率（QCM 等）</t>
+          <t>溅射气体与气压</t>
         </is>
       </c>
       <c r="D104" s="11" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>下拉+数值</t>
         </is>
       </c>
       <c r="E104" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ar / Ar+N₂…</t>
         </is>
       </c>
       <c r="F104" s="11" t="inlineStr">
         <is>
-          <t>nm/s</t>
+          <t>Pa</t>
         </is>
       </c>
       <c r="G104" s="16" t="inlineStr">
@@ -5731,7 +5727,7 @@
       </c>
       <c r="H104" s="11" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>Ar，0.5 Pa</t>
         </is>
       </c>
       <c r="I104" s="11" t="inlineStr">
@@ -5742,21 +5738,127 @@
       <c r="J104" s="11" t="inlineStr"/>
       <c r="K104" s="11" t="inlineStr">
         <is>
+          <t>{"gt":0,"require_value":true}</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="11" t="inlineStr">
+        <is>
+          <t>PVD</t>
+        </is>
+      </c>
+      <c r="B105" s="11" t="inlineStr">
+        <is>
+          <t>预溅射与挡板时序</t>
+        </is>
+      </c>
+      <c r="C105" s="11" t="inlineStr">
+        <is>
+          <t>预溅射时长、挡板开合时序</t>
+        </is>
+      </c>
+      <c r="D105" s="11" t="inlineStr">
+        <is>
+          <t>数值</t>
+        </is>
+      </c>
+      <c r="E105" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F105" s="11" t="inlineStr">
+        <is>
+          <t>min·s</t>
+        </is>
+      </c>
+      <c r="G105" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
+        </is>
+      </c>
+      <c r="H105" s="11" t="inlineStr">
+        <is>
+          <t>预溅 5 min</t>
+        </is>
+      </c>
+      <c r="I105" s="11" t="inlineStr">
+        <is>
+          <t>复审</t>
+        </is>
+      </c>
+      <c r="J105" s="11" t="inlineStr"/>
+      <c r="K105" s="11" t="inlineStr">
+        <is>
+          <t>{"gt":0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="11" t="inlineStr">
+        <is>
+          <t>PVD</t>
+        </is>
+      </c>
+      <c r="B106" s="11" t="inlineStr">
+        <is>
+          <t>沉积速率</t>
+        </is>
+      </c>
+      <c r="C106" s="11" t="inlineStr">
+        <is>
+          <t>速率（QCM 等）</t>
+        </is>
+      </c>
+      <c r="D106" s="11" t="inlineStr">
+        <is>
+          <t>数值</t>
+        </is>
+      </c>
+      <c r="E106" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F106" s="11" t="inlineStr">
+        <is>
+          <t>nm/s</t>
+        </is>
+      </c>
+      <c r="G106" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
+        </is>
+      </c>
+      <c r="H106" s="11" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="I106" s="11" t="inlineStr">
+        <is>
+          <t>复审</t>
+        </is>
+      </c>
+      <c r="J106" s="11" t="inlineStr"/>
+      <c r="K106" s="11" t="inlineStr">
+        <is>
           <t>{"gt":0}</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="A100:K100"/>
     <mergeCell ref="A20:K20"/>
     <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A78:K78"/>
-    <mergeCell ref="A87:K87"/>
     <mergeCell ref="A38:K38"/>
     <mergeCell ref="A11:K11"/>
     <mergeCell ref="A49:K49"/>
-    <mergeCell ref="A98:K98"/>
-    <mergeCell ref="A66:K66"/>
+    <mergeCell ref="A68:K68"/>
+    <mergeCell ref="A80:K80"/>
+    <mergeCell ref="A89:K89"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9356,7 +9458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D65"/>
+  <dimension ref="A1:D66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10704,20 +10806,42 @@
     <row r="65">
       <c r="A65" s="11" t="inlineStr">
         <is>
+          <t>v4.0-alpha.3</t>
+        </is>
+      </c>
+      <c r="B65" s="11" t="inlineStr">
+        <is>
+          <t>§4 衬底</t>
+        </is>
+      </c>
+      <c r="C65" s="11" t="inlineStr">
+        <is>
+          <t>产品简化界面增加本片轴向位置与备注；轴向位置为普通用户提交前必填，不暴露三维坐标</t>
+        </is>
+      </c>
+      <c r="D65" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-30产品简化</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
           <t>R0</t>
         </is>
       </c>
-      <c r="B65" s="11" t="inlineStr">
+      <c r="B66" s="11" t="inlineStr">
         <is>
           <t>硬必填核心(29项，含条件必填)</t>
         </is>
       </c>
-      <c r="C65" s="11" t="inlineStr">
+      <c r="C66" s="11" t="inlineStr">
         <is>
           <t>v3.18删除炉次内重复的前驱体化学式R0；物料身份仍由必填的批次版本快照冻结；其余R0定义不变</t>
         </is>
       </c>
-      <c r="D65" s="11" t="inlineStr">
+      <c r="D66" s="11" t="inlineStr">
         <is>
           <t>必填集</t>
         </is>

</xml_diff>

<commit_message>
refactor(ui): simplify characterization and samples
</commit_message>
<xml_diff>
--- a/docs/standard/字段草案-v3.xlsx
+++ b/docs/standard/字段草案-v3.xlsx
@@ -9458,7 +9458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D66"/>
+  <dimension ref="A1:D67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10828,20 +10828,42 @@
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
         <is>
+          <t>v4.0-alpha.4</t>
+        </is>
+      </c>
+      <c r="B66" s="11" t="inlineStr">
+        <is>
+          <t>§7 表征</t>
+        </is>
+      </c>
+      <c r="C66" s="11" t="inlineStr">
+        <is>
+          <t>表征方法拆分最小必填与更多测量参数，固定各方法常用结果项，并增加“其他”方法说明；科学对象仍由后端统一落库</t>
+        </is>
+      </c>
+      <c r="D66" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-30产品简化</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="11" t="inlineStr">
+        <is>
           <t>R0</t>
         </is>
       </c>
-      <c r="B66" s="11" t="inlineStr">
+      <c r="B67" s="11" t="inlineStr">
         <is>
           <t>硬必填核心(29项，含条件必填)</t>
         </is>
       </c>
-      <c r="C66" s="11" t="inlineStr">
+      <c r="C67" s="11" t="inlineStr">
         <is>
           <t>v3.18删除炉次内重复的前驱体化学式R0；物料身份仍由必填的批次版本快照冻结；其余R0定义不变</t>
         </is>
       </c>
-      <c r="D66" s="11" t="inlineStr">
+      <c r="D67" s="11" t="inlineStr">
         <is>
           <t>必填集</t>
         </is>

</xml_diff>

<commit_message>
feat: simplify CVD preparation workflow
</commit_message>
<xml_diff>
--- a/docs/standard/字段草案-v3.xlsx
+++ b/docs/standard/字段草案-v3.xlsx
@@ -3206,9 +3206,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G54" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
+      <c r="G54" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
@@ -3259,9 +3259,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G55" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(批次有规格数值)</t>
+      <c r="G55" s="16" t="inlineStr">
+        <is>
+          <t>选填（批次有明确规格时只读带出）</t>
         </is>
       </c>
       <c r="H55" s="11" t="inlineStr">
@@ -3312,9 +3312,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G56" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
+      <c r="G56" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
@@ -3365,9 +3365,9 @@
           <t>°</t>
         </is>
       </c>
-      <c r="G57" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(批次有规格数值)</t>
+      <c r="G57" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H57" s="11" t="inlineStr">
@@ -3422,9 +3422,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G58" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(偏切角&gt;0)</t>
+      <c r="G58" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
@@ -3528,9 +3528,9 @@
           <t>nm</t>
         </is>
       </c>
-      <c r="G60" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
+      <c r="G60" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>本次实验实际放入炉内的这一片衬底尺寸、放置方式及条件角度；批次来料规格另存于MaterialLot</t>
+          <t>本次实验实际放入炉内的这一片衬底尺寸、放置方式及条件角度；长度为沿气流方向的边长，宽度为垂直气流方向的边长</t>
         </is>
       </c>
       <c r="D61" s="11" t="inlineStr">
@@ -3573,7 +3573,7 @@
       </c>
       <c r="E61" s="11" t="inlineStr">
         <is>
-          <t>{length_mm, width_mm, thickness_mm?, placement: 正放|倒扣|倾角|竖放|其他, tilt_angle_deg?, placement_other?}</t>
+          <t>{length_mm, width_mm, thickness_mm?, placement: 正放|倒扣|两片生长面相对|倾角|竖放|其他, tilt_angle_deg?, placement_other?}</t>
         </is>
       </c>
       <c r="F61" s="11" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="J61" s="11" t="inlineStr">
         <is>
-          <t>每片可能经过切割，故不得用批次来料尺寸替代；placement=倾角时tilt_angle_deg条件必填；placement=其他时placement_other条件必填</t>
+          <t>每片可能经过切割，故不得用批次来料尺寸替代；placement=倾角时tilt_angle_deg条件必填且相对水平放置平面大于0°、小于90°；placement=其他时placement_other条件必填</t>
         </is>
       </c>
       <c r="K61" s="11" t="inlineStr"/>
@@ -3797,9 +3797,9 @@
           <t>mm</t>
         </is>
       </c>
-      <c r="G65" s="15" t="inlineStr">
-        <is>
-          <t>推荐</t>
+      <c r="G65" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
         </is>
       </c>
       <c r="H65" s="11" t="inlineStr">
@@ -3850,9 +3850,9 @@
           <t>mm</t>
         </is>
       </c>
-      <c r="G66" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
+      <c r="G66" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H66" s="11" t="inlineStr">
@@ -3867,7 +3867,7 @@
       </c>
       <c r="J66" s="11" t="inlineStr">
         <is>
-          <t>普通用户只填写装置轴向位置；不暴露三维坐标</t>
+          <t>仅兼容旧记录；新记录统一填写所在温区与热电偶距离，不再使用未定义物理原点的全局轴向位置</t>
         </is>
       </c>
       <c r="K66" s="11" t="inlineStr"/>
@@ -4198,7 +4198,7 @@
       </c>
       <c r="J73" s="11" t="inlineStr">
         <is>
-          <t>purity从lot_ref.snapshot带出；区间end_min必须大于start_min；同时间段体积流量占比由各气体流量派生</t>
+          <t>lot_ref与measurement_source必填，purity从lot_ref.snapshot带出；end_min必须大于start_min且flow_sccm&gt;0；同一气体的区间不得重叠；同时间段体积流量占比由各气体流量派生</t>
         </is>
       </c>
       <c r="K73" s="11" t="inlineStr"/>
@@ -4211,7 +4211,7 @@
       </c>
       <c r="B74" s="11" t="inlineStr">
         <is>
-          <t>压力体系与工作绝对压力</t>
+          <t>反应压力条件与工作绝对压力</t>
         </is>
       </c>
       <c r="C74" s="11" t="inlineStr">
@@ -4241,7 +4241,7 @@
       </c>
       <c r="H74" s="11" t="inlineStr">
         <is>
-          <t>常压；1.01325×10⁵ Pa</t>
+          <t>常压；或低压 500 Pa</t>
         </is>
       </c>
       <c r="I74" s="11" t="inlineStr">
@@ -4251,12 +4251,12 @@
       </c>
       <c r="J74" s="11" t="inlineStr">
         <is>
-          <t>填绝对压力，不填相对大气压的表压</t>
+          <t>常压可只记录反应压力条件；低压与超高真空必须填写绝对压力，不填相对大气压的表压</t>
         </is>
       </c>
       <c r="K74" s="11" t="inlineStr">
         <is>
-          <t>{"gt":0,"option_ranges":{"atmospheric_pressure":{"ge":80000,"le":120000},"low_pressure":{"gt":1e-06,"lt":80000},"ultra_high_vacuum":{"gt":0,"le":1e-06}},"require_option":true,"require_value":true}</t>
+          <t>{"gt":0,"option_ranges":{"atmospheric_pressure":{"ge":80000,"le":120000},"low_pressure":{"gt":1e-06,"lt":80000},"ultra_high_vacuum":{"gt":0,"le":1e-06}},"require_option":true,"require_value":false,"require_value_options":["low_pressure","ultra_high_vacuum"]}</t>
         </is>
       </c>
     </row>
@@ -4336,7 +4336,7 @@
       </c>
       <c r="E76" s="11" t="inlineStr">
         <is>
-          <t>{method: 随炉冷却|开盖冷却|移炉快速冷却|其他, lid_open_temperature_C?, cooling_rate_C_per_min?, method_other?}</t>
+          <t>{method: 随炉冷却|开盖冷却|移炉快速冷却|受控降温|其他, lid_open_temperature_C?, cooling_rate_C_per_min?, method_other?}</t>
         </is>
       </c>
       <c r="F76" s="11" t="inlineStr">
@@ -4344,9 +4344,9 @@
           <t>℃·℃/min</t>
         </is>
       </c>
-      <c r="G76" s="15" t="inlineStr">
-        <is>
-          <t>推荐</t>
+      <c r="G76" s="14" t="inlineStr">
+        <is>
+          <t>条件必填(反应条件记录)</t>
         </is>
       </c>
       <c r="H76" s="11" t="inlineStr">
@@ -4361,7 +4361,7 @@
       </c>
       <c r="J76" s="11" t="inlineStr">
         <is>
-          <t>method=开盖冷却时开盖温度必填；method=其他时method_other必填</t>
+          <t>method=开盖冷却时开盖温度必填；method=受控降温时降温速率必填；method=其他时method_other必填</t>
         </is>
       </c>
       <c r="K76" s="11" t="inlineStr"/>
@@ -4414,7 +4414,7 @@
       </c>
       <c r="J77" s="11" t="inlineStr">
         <is>
-          <t>field_type必须属于Setup能力；界面按类型显示明确字段，其他参数仍使用具名值和单位</t>
+          <t>未添加表示本炉未使用外场；添加后field_type必须属于Setup能力，并填写时间区间及对应类型的必要参数</t>
         </is>
       </c>
       <c r="K77" s="11" t="inlineStr"/>
@@ -5870,7 +5870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K71"/>
+  <dimension ref="A1:K62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5963,7 +5963,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>实体① 物料批次库 MaterialLot（统一维护前驱体、衬底与气瓶批次；实验中只引用批次，纯度和粒径自动带出并锁版）</t>
+          <t>实体① 物料批次库 MaterialLot（统一维护前驱体、衬底与气瓶批次；实验中只引用批次并冻结所引用版本）</t>
         </is>
       </c>
       <c r="B3" s="8" t="n"/>
@@ -6091,7 +6091,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>物料名称（按标签）</t>
+          <t>物料名称</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
@@ -6131,7 +6131,7 @@
       </c>
       <c r="J6" s="11" t="inlineStr">
         <is>
-          <t>按标签记录，不要求用户自行翻译；不用化学式代替名称</t>
+          <t>按标签记录，不要求用户自行翻译；不用化学式代替名称；已知类型的衬底由系统根据“衬底材料”生成</t>
         </is>
       </c>
       <c r="K6" s="11" t="inlineStr"/>
@@ -6174,15 +6174,19 @@
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>MoO₃</t>
+          <t>MoO3</t>
         </is>
       </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="J7" s="11" t="inlineStr"/>
+          <t>2026-08-06用户界面复核</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>复用目标产物的化学式输入与即时校验；已知类型的衬底由系统生成生长表面化学式，仅云母或其他衬底需人工填写</t>
+        </is>
+      </c>
       <c r="K7" s="11" t="inlineStr"/>
     </row>
     <row r="8">
@@ -6193,12 +6197,12 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>CAS号</t>
+          <t>CAS 号</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>唯一化学标识</t>
+          <t>标签或CoA明确提供时抄录的CAS登记号</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -6216,9 +6220,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(化学品或气瓶)</t>
+      <c r="G8" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
@@ -6228,10 +6232,14 @@
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="J8" s="11" t="inlineStr"/>
+          <t>2026-08-02供应商标签/CoA公开资料复核</t>
+        </is>
+      </c>
+      <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>自研、复配或供应商资料未提供时留空</t>
+        </is>
+      </c>
       <c r="K8" s="11" t="inlineStr"/>
     </row>
     <row r="9">
@@ -6242,22 +6250,22 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>物质同义名</t>
+          <t>供应商</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>用于检索的稳定同义名，不替代标签名称</t>
+          <t>商业批次：厂商</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>文本数组</t>
+          <t>下拉+其他(可扩展)</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>JSON字符串数组</t>
+          <t>受控+其他</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
@@ -6265,24 +6273,24 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G9" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>推荐</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>["Molybdenum trioxide"]</t>
+          <t>阿拉丁</t>
         </is>
       </c>
       <c r="I9" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28深度审查</t>
+          <t>2026-08-06用户界面复核</t>
         </is>
       </c>
       <c r="J9" s="11" t="inlineStr">
         <is>
-          <t>归一化到Substance实体</t>
+          <t>历史供应商可复用；新增时按包装标签原文填写名称</t>
         </is>
       </c>
       <c r="K9" s="11" t="inlineStr"/>
@@ -6295,22 +6303,22 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>物质标识符</t>
+          <t>货号（Cat. No. / Product No.）</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>CAS、InChIKey等标识符及其类型</t>
+          <t>供应商用于识别产品与规格的编号</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>JSON数组</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>[{type,value}]</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
@@ -6325,17 +6333,17 @@
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>[{"type":"CAS","value":"1313-27-5"}]</t>
+          <t>M112056</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28深度审查</t>
+          <t>2026-08-06用户界面复核</t>
         </is>
       </c>
       <c r="J10" s="11" t="inlineStr">
         <is>
-          <t>归一化到Substance实体</t>
+          <t>同一货号可对应多个批号</t>
         </is>
       </c>
       <c r="K10" s="11" t="inlineStr"/>
@@ -6348,22 +6356,22 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>供应商</t>
+          <t>产品等级（标签原文）</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>商业批次：厂商</t>
+          <t>包装标签、产品页或CoA给出的产品等级原文</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>下拉+其他(可扩展)</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>受控+其他</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F11" s="11" t="inlineStr">
@@ -6371,22 +6379,26 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G11" s="15" t="inlineStr">
-        <is>
-          <t>推荐</t>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>阿拉丁</t>
+          <t>99.98% trace metals basis</t>
         </is>
       </c>
       <c r="I11" s="11" t="inlineStr">
         <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="J11" s="11" t="inlineStr"/>
+          <t>2026-08-02供应商标签/CoA公开资料复核</t>
+        </is>
+      </c>
+      <c r="J11" s="11" t="inlineStr">
+        <is>
+          <t>按供应商资料原文记录；未提供时留空</t>
+        </is>
+      </c>
       <c r="K11" s="11" t="inlineStr"/>
     </row>
     <row r="12">
@@ -6397,12 +6409,12 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>供应商货号</t>
+          <t>批号（Lot No. / Batch No.）</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>商业批次：产品号</t>
+          <t>识别当前这批实物的批次编号</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -6420,24 +6432,24 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G12" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>M112056</t>
+          <t>B202405</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>2026-08-06用户界面复核</t>
         </is>
       </c>
       <c r="J12" s="11" t="inlineStr">
         <is>
-          <t>供应商产品规格编号，标签上常写作 Cat. No.；同一货号可有多个生产批号</t>
+          <t>同一货号下用于区分不同生产批次</t>
         </is>
       </c>
       <c r="K12" s="11" t="inlineStr"/>
@@ -6450,27 +6462,27 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>供应商等级</t>
+          <t>纯度</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>供应商给出的产品等级或规格名称</t>
+          <t>标签或CoA明确给出的数值纯度百分比</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>百分数</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>%</t>
         </is>
       </c>
       <c r="G13" s="16" t="inlineStr">
@@ -6480,20 +6492,24 @@
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>ACS reagent</t>
+          <t>99.995</t>
         </is>
       </c>
       <c r="I13" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28深度审查</t>
+          <t>2026-08-02供应商标签/CoA公开资料复核</t>
         </is>
       </c>
       <c r="J13" s="11" t="inlineStr">
         <is>
-          <t>与实测纯度分开</t>
-        </is>
-      </c>
-      <c r="K13" s="11" t="inlineStr"/>
+          <t>未明确标示百分数时留空；等级原文记录于“产品等级（标签原文）”，原始依据由标签或CoA附件保留</t>
+        </is>
+      </c>
+      <c r="K13" s="11" t="inlineStr">
+        <is>
+          <t>{"gt":0,"le":100}</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
@@ -6503,22 +6519,22 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>商业产品规格</t>
+          <t>物料形态</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>随货号稳定的商业产品规格</t>
+          <t>试剂外观</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>JSON对象</t>
+          <t>下拉+其他</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>具名规格键值</t>
+          <t>粉末/颗粒/块/液体/箔/靶/其他</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
@@ -6533,17 +6549,17 @@
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>{"mesh":"100"}</t>
+          <t>粉末</t>
         </is>
       </c>
       <c r="I14" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28深度审查</t>
+          <t>review</t>
         </is>
       </c>
       <c r="J14" s="11" t="inlineStr">
         <is>
-          <t>归一化到CommercialProduct实体</t>
+          <t>外观=性状；气瓶不使用粉末/箔/靶等物料形态</t>
         </is>
       </c>
       <c r="K14" s="11" t="inlineStr"/>
@@ -6556,17 +6572,17 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>生产批号</t>
+          <t>开封日期</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>商业批次：生产批号（同名不同批的区分键）</t>
+          <t>影响吸潮/氧化</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>日期</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
@@ -6579,14 +6595,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G15" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>B202405</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="I15" s="11" t="inlineStr">
@@ -6594,11 +6610,7 @@
           <t>review</t>
         </is>
       </c>
-      <c r="J15" s="11" t="inlineStr">
-        <is>
-          <t>GMP法定术语『批号』；标签上常写作 Lot No. 或 Batch No.</t>
-        </is>
-      </c>
+      <c r="J15" s="11" t="inlineStr"/>
       <c r="K15" s="11" t="inlineStr"/>
     </row>
     <row r="16">
@@ -6609,37 +6621,37 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>纯度</t>
+          <t>存储方式</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>仅存质量百分数；N值由质量百分数派生显示，不作为独立存储值</t>
+          <t>存放条件</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>下拉+其他</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>质量百分数（N值仅派生显示）</t>
+          <t>干燥器/手套箱/常温避光/冷藏/其他</t>
         </is>
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="G16" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(化学品或气瓶)</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>99.995（派生显示4N5）</t>
+          <t>干燥器</t>
         </is>
       </c>
       <c r="I16" s="11" t="inlineStr">
@@ -6649,14 +6661,10 @@
       </c>
       <c r="J16" s="11" t="inlineStr">
         <is>
-          <t>原始证书中的N值或其他纯度表述保留在CoA/附件说明中</t>
-        </is>
-      </c>
-      <c r="K16" s="11" t="inlineStr">
-        <is>
-          <t>{"gt":0,"le":100}</t>
-        </is>
-      </c>
+          <t>desiccator=干燥器</t>
+        </is>
+      </c>
+      <c r="K16" s="11" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
@@ -6666,22 +6674,22 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>纯度基准</t>
+          <t>分析证书（CoA）</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>纯度数值所采用的组成基准</t>
+          <t>质检证书</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>下拉</t>
+          <t>FileAsset引用</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>质量分数/原子分数/体积分数</t>
+          <t>{file_asset_id, sha256}</t>
         </is>
       </c>
       <c r="F17" s="11" t="inlineStr">
@@ -6689,26 +6697,22 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G17" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(填写纯度时)</t>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
         </is>
       </c>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>质量分数</t>
+          <t>coa.pdf</t>
         </is>
       </c>
       <c r="I17" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28深度审查</t>
-        </is>
-      </c>
-      <c r="J17" s="11" t="inlineStr">
-        <is>
-          <t>禁止只存没有基准的百分数</t>
-        </is>
-      </c>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="J17" s="11" t="inlineStr"/>
       <c r="K17" s="11" t="inlineStr"/>
     </row>
     <row r="18">
@@ -6719,22 +6723,22 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>纯度来源</t>
+          <t>包装标签附件</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>纯度数值来自供应商声明还是CoA实测</t>
+          <t>试剂瓶身、气瓶或衬底包装标签的原始照片，用于追溯批号与规格</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>下拉</t>
+          <t>FileAsset引用</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>供应商声明/CoA实测</t>
+          <t>{file_asset_id, sha256}</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -6742,24 +6746,24 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G18" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(填写纯度时)</t>
+      <c r="G18" s="15" t="inlineStr">
+        <is>
+          <t>推荐</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>CoA实测</t>
+          <t>bottle-label.jpg</t>
         </is>
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28深度审查</t>
+          <t>2026-07-24导师走查</t>
         </is>
       </c>
       <c r="J18" s="11" t="inlineStr">
         <is>
-          <t>来源文件仍由CoA附件保存</t>
+          <t>与CoA分开；同一物料版本至少上传一次并可预览、下载</t>
         </is>
       </c>
       <c r="K18" s="11" t="inlineStr"/>
@@ -6772,12 +6776,12 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>形态与性状</t>
+          <t>▸衬底·材料</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>试剂外观</t>
+          <t>子类(批次类别=衬底)</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
@@ -6787,7 +6791,7 @@
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>粉末/颗粒/块/液体/箔/靶/其他</t>
+          <t>SiO₂/Si·蓝宝石(Al₂O₃)·石英·云母·Cu箔·Au箔·h-BN·其他</t>
         </is>
       </c>
       <c r="F19" s="11" t="inlineStr">
@@ -6795,14 +6799,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G19" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t>条件必填(衬底)</t>
         </is>
       </c>
       <c r="H19" s="11" t="inlineStr">
         <is>
-          <t>粉末</t>
+          <t>SiO₂/Si</t>
         </is>
       </c>
       <c r="I19" s="11" t="inlineStr">
@@ -6812,7 +6816,7 @@
       </c>
       <c r="J19" s="11" t="inlineStr">
         <is>
-          <t>外观=性状；气瓶不使用粉末/箔/靶等物料形态</t>
+          <t>与§4衬底材料词表一致</t>
         </is>
       </c>
       <c r="K19" s="11" t="inlineStr"/>
@@ -6825,12 +6829,12 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>粒径D50</t>
+          <t>▸衬底·氧化层厚度</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>供应商或CoA报告的来料中位粒径；影响挥发和成核</t>
+          <t>仅SiO₂/Si</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -6840,22 +6844,22 @@
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>供应商或CoA报告的D50</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
-          <t>µm</t>
-        </is>
-      </c>
-      <c r="G20" s="16" t="inlineStr">
-        <is>
-          <t>条件选填(粉末或颗粒)</t>
+          <t>nm</t>
+        </is>
+      </c>
+      <c r="G20" s="14" t="inlineStr">
+        <is>
+          <t>条件必填(SiO₂/Si)</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>285</t>
         </is>
       </c>
       <c r="I20" s="11" t="inlineStr">
@@ -6863,11 +6867,7 @@
           <t>review</t>
         </is>
       </c>
-      <c r="J20" s="11" t="inlineStr">
-        <is>
-          <t>仅在来料形态为粉末或颗粒且供应商/CoA有报告时填写；无报告留空，不用目数或猜测值代替</t>
-        </is>
-      </c>
+      <c r="J20" s="11" t="inlineStr"/>
       <c r="K20" s="11" t="inlineStr">
         <is>
           <t>{"gt":0}</t>
@@ -6882,22 +6882,22 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>D50测量方法</t>
+          <t>▸衬底·晶向与抛光信息</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>得到D50数值所用的方法</t>
+          <t>供应商是否提供且该衬底是否适用晶面取向与抛光规格</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>下拉+其他</t>
+          <t>下拉</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>激光衍射/筛分/图像分析/其他</t>
+          <t>有规格数值·供应商未提供·不适用</t>
         </is>
       </c>
       <c r="F21" s="11" t="inlineStr">
@@ -6907,22 +6907,22 @@
       </c>
       <c r="G21" s="16" t="inlineStr">
         <is>
-          <t>条件选填(填写D50时)</t>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H21" s="11" t="inlineStr">
         <is>
-          <t>激光衍射</t>
+          <t>有规格数值</t>
         </is>
       </c>
       <c r="I21" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28深度审查</t>
+          <t>2026-07-25用户复核</t>
         </is>
       </c>
       <c r="J21" s="11" t="inlineStr">
         <is>
-          <t>未报告时留空，不猜测</t>
+          <t>Cu/Au箔等不适用时明确选择不适用；禁止伪填晶向或抛光面</t>
         </is>
       </c>
       <c r="K21" s="11" t="inlineStr"/>
@@ -6935,22 +6935,22 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>D50统计基准</t>
+          <t>▸衬底·晶向与抛光</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>粒径分布按体积、数目或质量统计</t>
+          <t>取向与抛光面</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>下拉</t>
+          <t>文本+下拉</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>体积分数/数目基准/质量基准</t>
+          <t>晶向；单面抛/双面抛</t>
         </is>
       </c>
       <c r="F22" s="11" t="inlineStr">
@@ -6960,25 +6960,29 @@
       </c>
       <c r="G22" s="16" t="inlineStr">
         <is>
-          <t>条件选填(填写D50时)</t>
+          <t>选填(仅供应商明确提供时)</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>体积分数</t>
+          <t>Si(100)；单面抛</t>
         </is>
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28深度审查</t>
+          <t>review</t>
         </is>
       </c>
       <c r="J22" s="11" t="inlineStr">
         <is>
-          <t>与测量方法共同决定可比性</t>
-        </is>
-      </c>
-      <c r="K22" s="11" t="inlineStr"/>
+          <t>供应商资料明确给出且实验需要区分时填写；实验引用批次后只读带出</t>
+        </is>
+      </c>
+      <c r="K22" s="11" t="inlineStr">
+        <is>
+          <t>{"require_option":true,"require_value":true}</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
@@ -6988,12 +6992,12 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>D50来源</t>
+          <t>▸衬底·偏切信息</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>D50数值的来源</t>
+          <t>供应商是否提供且该衬底是否适用相对标称晶面的偏切规格</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
@@ -7003,7 +7007,7 @@
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>供应商声明/CoA实测</t>
+          <t>有规格数值·供应商未提供·不适用</t>
         </is>
       </c>
       <c r="F23" s="11" t="inlineStr">
@@ -7013,22 +7017,22 @@
       </c>
       <c r="G23" s="16" t="inlineStr">
         <is>
-          <t>条件选填(填写D50时)</t>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>CoA实测</t>
+          <t>供应商未提供</t>
         </is>
       </c>
       <c r="I23" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28深度审查</t>
+          <t>2026-07-25用户复核</t>
         </is>
       </c>
       <c r="J23" s="11" t="inlineStr">
         <is>
-          <t>来源文件仍由CoA附件保存</t>
+          <t>0仅表示供应商明确报告无偏切，不能表示未知或不适用</t>
         </is>
       </c>
       <c r="K23" s="11" t="inlineStr"/>
@@ -7041,17 +7045,17 @@
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>开封日期</t>
+          <t>▸衬底·偏切角</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>影响吸潮/氧化</t>
+          <t>实际晶面相对标称晶面的偏切角</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>日期</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
@@ -7061,26 +7065,34 @@
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>°</t>
         </is>
       </c>
       <c r="G24" s="16" t="inlineStr">
         <is>
-          <t>选填</t>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="J24" s="11" t="inlineStr"/>
-      <c r="K24" s="11" t="inlineStr"/>
+          <t>2026-07-24用户走查</t>
+        </is>
+      </c>
+      <c r="J24" s="11" t="inlineStr">
+        <is>
+          <t>大于0时必须同时填写substrate_miscut_direction</t>
+        </is>
+      </c>
+      <c r="K24" s="11" t="inlineStr">
+        <is>
+          <t>{"ge":0,"lt":90}</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
@@ -7090,22 +7102,22 @@
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>存储方式</t>
+          <t>▸衬底·偏切方向</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>存放条件</t>
+          <t>偏切角所指的晶轴或晶向</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>下拉+其他</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>干燥器/手套箱/常温避光/冷藏/其他</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F25" s="11" t="inlineStr">
@@ -7115,22 +7127,22 @@
       </c>
       <c r="G25" s="16" t="inlineStr">
         <is>
-          <t>选填</t>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>干燥器</t>
+          <t>c面向a轴</t>
         </is>
       </c>
       <c r="I25" s="11" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>2026-07-24用户走查</t>
         </is>
       </c>
       <c r="J25" s="11" t="inlineStr">
         <is>
-          <t>desiccator=干燥器</t>
+          <t>substrate_miscut_angle_deg大于0时由跨字段校验强制填写</t>
         </is>
       </c>
       <c r="K25" s="11" t="inlineStr"/>
@@ -7143,45 +7155,49 @@
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>证书附件(CoA)</t>
+          <t>▸衬底·标称表面粗糙度</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>质检证书</t>
+          <t>供应商或批次规格中的标称粗糙度</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>FileAsset引用</t>
+          <t>粗糙度对象</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>{file_asset_id, sha256}</t>
+          <t>{availability: 有规格数值|供应商未提供；有规格数值时 metric: Ra|RMS, value_nm}</t>
         </is>
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>nm</t>
         </is>
       </c>
       <c r="G26" s="16" t="inlineStr">
         <is>
-          <t>选填</t>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>coa.pdf</t>
+          <t>{availability: not_provided}</t>
         </is>
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="J26" s="11" t="inlineStr"/>
+          <t>2026-07-25用户复核</t>
+        </is>
+      </c>
+      <c r="J26" s="11" t="inlineStr">
+        <is>
+          <t>reported时metric与value_nm必填；not_provided时二者禁止填写；历史无availability对象按reported兼容；本片AFM实测值属于表征结果</t>
+        </is>
+      </c>
       <c r="K26" s="11" t="inlineStr"/>
     </row>
     <row r="27">
@@ -7192,47 +7208,47 @@
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>瓶身或包装标签附件</t>
+          <t>▸衬底·来料尺寸规格</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>试剂瓶身、气瓶或衬底包装标签的原始照片，用于追溯批号与规格</t>
+          <t>供应商标称或该批次来料的原始几何；切割后本次实际单片尺寸属于实验记录</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>FileAsset引用</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>{file_asset_id, sha256}</t>
+          <t>长×宽×厚</t>
         </is>
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G27" s="15" t="inlineStr">
-        <is>
-          <t>推荐</t>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="G27" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H27" s="11" t="inlineStr">
         <is>
-          <t>bottle-label.jpg</t>
+          <t>10×10×0.5</t>
         </is>
       </c>
       <c r="I27" s="11" t="inlineStr">
         <is>
-          <t>2026-07-24导师走查</t>
+          <t>review</t>
         </is>
       </c>
       <c r="J27" s="11" t="inlineStr">
         <is>
-          <t>与CoA分开；同一物料版本至少上传一次并可预览、下载</t>
+          <t>不替代每次实验的本片实际尺寸</t>
         </is>
       </c>
       <c r="K27" s="11" t="inlineStr"/>
@@ -7245,47 +7261,47 @@
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>▸衬底·材料</t>
+          <t>▸衬底·层堆栈</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>子类(批次类别=衬底)</t>
+          <t>从体材料到顶表面逐层记录供应商交付的衬底结构</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>下拉+其他</t>
+          <t>JSON数组</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>SiO₂/Si·蓝宝石(Al₂O₃)·石英·云母·Cu箔·Au箔·h-BN·其他</t>
+          <t>[{material_name,chemical_formula?,thickness_nm?,orientation?,supplier_lot_id?}]</t>
         </is>
       </c>
       <c r="F28" s="11" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G28" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(衬底)</t>
+          <t>nm</t>
+        </is>
+      </c>
+      <c r="G28" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>SiO₂/Si</t>
+          <t>[{"material_name":"Si"},{"material_name":"SiO2","thickness_nm":285}]</t>
         </is>
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>2026-07-28深度审查</t>
         </is>
       </c>
       <c r="J28" s="11" t="inlineStr">
         <is>
-          <t>与§4衬底材料词表一致</t>
+          <t>按数组顺序生成SubstrateStack；不得用单个字符串拼层</t>
         </is>
       </c>
       <c r="K28" s="11" t="inlineStr"/>
@@ -7298,17 +7314,17 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>▸衬底·氧化层厚度</t>
+          <t>▸衬底·顶表面</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>仅SiO₂/Si</t>
+          <t>实验放样时实际暴露的最上层表面</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E29" s="11" t="inlineStr">
@@ -7318,30 +7334,30 @@
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>nm</t>
-        </is>
-      </c>
-      <c r="G29" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(SiO₂/Si)</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G29" s="16" t="inlineStr">
+        <is>
+          <t>未发布</t>
         </is>
       </c>
       <c r="H29" s="11" t="inlineStr">
         <is>
-          <t>285</t>
+          <t>SiO2</t>
         </is>
       </c>
       <c r="I29" s="11" t="inlineStr">
         <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="J29" s="11" t="inlineStr"/>
-      <c r="K29" s="11" t="inlineStr">
-        <is>
-          <t>{"gt":0}</t>
-        </is>
-      </c>
+          <t>2026-07-28深度审查</t>
+        </is>
+      </c>
+      <c r="J29" s="11" t="inlineStr">
+        <is>
+          <t>与层堆栈配套</t>
+        </is>
+      </c>
+      <c r="K29" s="11" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
@@ -7351,12 +7367,12 @@
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>▸衬底·晶向与抛光信息</t>
+          <t>▸气瓶·纯度等级</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>供应商是否提供且该衬底是否适用晶面取向与抛光规格</t>
+          <t>子类(批次类别=气瓶)；与base『纯度』分工</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -7366,7 +7382,7 @@
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>有规格数值·供应商未提供·不适用</t>
+          <t>6N/5N/4N/工业级</t>
         </is>
       </c>
       <c r="F30" s="11" t="inlineStr">
@@ -7374,24 +7390,24 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G30" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(衬底)</t>
+      <c r="G30" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>有规格数值</t>
+          <t>5N</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>2026-07-25用户复核</t>
+          <t>review</t>
         </is>
       </c>
       <c r="J30" s="11" t="inlineStr">
         <is>
-          <t>Cu/Au箔等不适用时明确选择不适用；禁止伪填晶向或抛光面</t>
+          <t>有供应商等级标签可照录；没有则留空</t>
         </is>
       </c>
       <c r="K30" s="11" t="inlineStr"/>
@@ -7404,22 +7420,22 @@
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>▸衬底·晶向与抛光</t>
+          <t>▸气瓶·气瓶编号</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>取向与抛光面</t>
+          <t>钢瓶追溯号</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>文本+下拉</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E31" s="11" t="inlineStr">
         <is>
-          <t>晶向；单面抛/双面抛</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F31" s="11" t="inlineStr">
@@ -7427,14 +7443,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G31" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(有规格数值)</t>
+      <c r="G31" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
         </is>
       </c>
       <c r="H31" s="11" t="inlineStr">
         <is>
-          <t>Si(100)；单面抛</t>
+          <t>GC-Ar-07</t>
         </is>
       </c>
       <c r="I31" s="11" t="inlineStr">
@@ -7442,89 +7458,45 @@
           <t>review</t>
         </is>
       </c>
-      <c r="J31" s="11" t="inlineStr">
-        <is>
-          <t>实验引用批次后只读带出</t>
-        </is>
-      </c>
-      <c r="K31" s="11" t="inlineStr">
-        <is>
-          <t>{"require_option":true,"require_value":true}</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="11" t="inlineStr">
-        <is>
-          <t>MaterialLot</t>
-        </is>
-      </c>
-      <c r="B32" s="11" t="inlineStr">
-        <is>
-          <t>▸衬底·偏切信息</t>
-        </is>
-      </c>
-      <c r="C32" s="11" t="inlineStr">
-        <is>
-          <t>供应商是否提供且该衬底是否适用相对标称晶面的偏切规格</t>
-        </is>
-      </c>
-      <c r="D32" s="11" t="inlineStr">
-        <is>
-          <t>下拉</t>
-        </is>
-      </c>
-      <c r="E32" s="11" t="inlineStr">
-        <is>
-          <t>有规格数值·供应商未提供·不适用</t>
-        </is>
-      </c>
-      <c r="F32" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G32" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(衬底)</t>
-        </is>
-      </c>
-      <c r="H32" s="11" t="inlineStr">
-        <is>
-          <t>供应商未提供</t>
-        </is>
-      </c>
-      <c r="I32" s="11" t="inlineStr">
-        <is>
-          <t>2026-07-25用户复核</t>
-        </is>
-      </c>
-      <c r="J32" s="11" t="inlineStr">
-        <is>
-          <t>0仅表示供应商明确报告无偏切，不能表示未知或不适用</t>
-        </is>
-      </c>
-      <c r="K32" s="11" t="inlineStr"/>
+      <c r="J31" s="11" t="inlineStr"/>
+      <c r="K31" s="11" t="inlineStr"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>实体② 装置库 Setup（一台炉登记一次，实验 §2 引用；坐标系随引用冻结）</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="n"/>
+      <c r="C32" s="8" t="n"/>
+      <c r="D32" s="8" t="n"/>
+      <c r="E32" s="8" t="n"/>
+      <c r="F32" s="8" t="n"/>
+      <c r="G32" s="8" t="n"/>
+      <c r="H32" s="8" t="n"/>
+      <c r="I32" s="8" t="n"/>
+      <c r="J32" s="8" t="n"/>
+      <c r="K32" s="8" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>MaterialLot</t>
+          <t>装置Setup</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>▸衬底·偏切角</t>
+          <t>装置名称</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>实际晶面相对标称晶面的偏切角</t>
+          <t>人读名</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E33" s="11" t="inlineStr">
@@ -7534,54 +7506,46 @@
       </c>
       <c r="F33" s="11" t="inlineStr">
         <is>
-          <t>°</t>
-        </is>
-      </c>
-      <c r="G33" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(有规格数值)</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G33" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
         </is>
       </c>
       <c r="H33" s="11" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>1号双温区管式炉</t>
         </is>
       </c>
       <c r="I33" s="11" t="inlineStr">
         <is>
-          <t>2026-07-24用户走查</t>
-        </is>
-      </c>
-      <c r="J33" s="11" t="inlineStr">
-        <is>
-          <t>大于0时必须同时填写substrate_miscut_direction</t>
-        </is>
-      </c>
-      <c r="K33" s="11" t="inlineStr">
-        <is>
-          <t>{"ge":0,"lt":90}</t>
-        </is>
-      </c>
+          <t>会议</t>
+        </is>
+      </c>
+      <c r="J33" s="11" t="inlineStr"/>
+      <c r="K33" s="11" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>MaterialLot</t>
+          <t>装置Setup</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>▸衬底·偏切方向</t>
+          <t>版本号</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>偏切角所指的晶轴或晶向</t>
+          <t>每次修改+1；引用时冻结此版本</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
@@ -7594,24 +7558,24 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G34" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(偏切角&gt;0)</t>
+      <c r="G34" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>c面向a轴</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>2026-07-24用户走查</t>
+          <t>★锁版使能(Fable三轮B2)</t>
         </is>
       </c>
       <c r="J34" s="11" t="inlineStr">
         <is>
-          <t>substrate_miscut_angle_deg大于0时由跨字段校验强制填写</t>
+          <t>对标 v1 setup_version_snapshot</t>
         </is>
       </c>
       <c r="K34" s="11" t="inlineStr"/>
@@ -7619,70 +7583,66 @@
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>MaterialLot</t>
+          <t>装置Setup</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>▸衬底·标称表面粗糙度</t>
+          <t>装置来源</t>
         </is>
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>供应商或批次规格中的标称粗糙度</t>
+          <t>装置是商业购买、实验室自制还是在既有设备上改造</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>粗糙度对象</t>
+          <t>下拉</t>
         </is>
       </c>
       <c r="E35" s="11" t="inlineStr">
         <is>
-          <t>{availability: 有规格数值|供应商未提供；有规格数值时 metric: Ra|RMS, value_nm}</t>
+          <t>商业设备/实验室自制/改造设备</t>
         </is>
       </c>
       <c r="F35" s="11" t="inlineStr">
         <is>
-          <t>nm</t>
-        </is>
-      </c>
-      <c r="G35" s="14" t="inlineStr">
-        <is>
-          <t>条件必填(衬底)</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
         </is>
       </c>
       <c r="H35" s="11" t="inlineStr">
         <is>
-          <t>{availability: not_provided}</t>
+          <t>商业设备</t>
         </is>
       </c>
       <c r="I35" s="11" t="inlineStr">
         <is>
-          <t>2026-07-25用户复核</t>
-        </is>
-      </c>
-      <c r="J35" s="11" t="inlineStr">
-        <is>
-          <t>reported时metric与value_nm必填；not_provided时二者禁止填写；历史无availability对象按reported兼容；本片AFM实测值属于表征结果</t>
-        </is>
-      </c>
+          <t>2026-07-28用户逐项复核</t>
+        </is>
+      </c>
+      <c r="J35" s="11" t="inlineStr"/>
       <c r="K35" s="11" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>MaterialLot</t>
+          <t>装置Setup</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>▸衬底·来料尺寸规格</t>
+          <t>制造商或品牌</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>供应商标称或该批次来料的原始几何；切割后本次实际单片尺寸属于实验记录</t>
+          <t>设备制造商或品牌，独立于型号保存以支持筛选和统计</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -7692,103 +7652,95 @@
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>长×宽×厚</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F36" s="11" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G36" s="16" t="inlineStr">
         <is>
-          <t>选填</t>
+          <t>条件选填(商业设备或改造设备)</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>10×10×0.5</t>
+          <t>合肥科晶</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="J36" s="11" t="inlineStr">
-        <is>
-          <t>不替代每次实验的本片实际尺寸</t>
-        </is>
-      </c>
+          <t>2026-07-28用户逐项复核</t>
+        </is>
+      </c>
+      <c r="J36" s="11" t="inlineStr"/>
       <c r="K36" s="11" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>MaterialLot</t>
+          <t>装置Setup</t>
         </is>
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>▸衬底·层堆栈</t>
+          <t>型号</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>从体材料到顶表面逐层记录供应商交付的衬底结构</t>
+          <t>制造商给出的设备型号</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>JSON数组</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E37" s="11" t="inlineStr">
         <is>
-          <t>[{material_name,chemical_formula?,thickness_nm?,orientation?,supplier_lot_id?}]</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F37" s="11" t="inlineStr">
         <is>
-          <t>nm</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G37" s="16" t="inlineStr">
         <is>
-          <t>条件选填(多层衬底)</t>
+          <t>条件选填(商业设备或改造设备)</t>
         </is>
       </c>
       <c r="H37" s="11" t="inlineStr">
         <is>
-          <t>[{"material_name":"Si"},{"material_name":"SiO2","thickness_nm":285}]</t>
+          <t>OTF-1200X</t>
         </is>
       </c>
       <c r="I37" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28深度审查</t>
-        </is>
-      </c>
-      <c r="J37" s="11" t="inlineStr">
-        <is>
-          <t>按数组顺序生成SubstrateStack；不得用单个字符串拼层</t>
-        </is>
-      </c>
+          <t>2026-07-28用户逐项复核</t>
+        </is>
+      </c>
+      <c r="J37" s="11" t="inlineStr"/>
       <c r="K37" s="11" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>MaterialLot</t>
+          <t>装置Setup</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>▸衬底·顶表面</t>
+          <t>设计或建造单位</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>实验放样时实际暴露的最上层表面</t>
+          <t>实验室自制装置的设计或建造单位</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -7808,50 +7760,46 @@
       </c>
       <c r="G38" s="16" t="inlineStr">
         <is>
-          <t>条件选填(多层衬底)</t>
+          <t>条件选填(实验室自制)</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>SiO2</t>
+          <t>二维材料课题组</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28深度审查</t>
-        </is>
-      </c>
-      <c r="J38" s="11" t="inlineStr">
-        <is>
-          <t>与层堆栈配套</t>
-        </is>
-      </c>
+          <t>2026-07-28用户逐项复核</t>
+        </is>
+      </c>
+      <c r="J38" s="11" t="inlineStr"/>
       <c r="K38" s="11" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="11" t="inlineStr">
         <is>
-          <t>MaterialLot</t>
+          <t>装置Setup</t>
         </is>
       </c>
       <c r="B39" s="11" t="inlineStr">
         <is>
-          <t>▸气瓶·纯度等级</t>
+          <t>内部型号</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>子类(批次类别=气瓶)；与base『纯度』分工</t>
+          <t>实验室自制装置使用的内部型号或版本名称</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>下拉</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E39" s="11" t="inlineStr">
         <is>
-          <t>6N/5N/4N/工业级</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F39" s="11" t="inlineStr">
@@ -7861,40 +7809,36 @@
       </c>
       <c r="G39" s="16" t="inlineStr">
         <is>
-          <t>选填</t>
+          <t>条件选填(实验室自制)</t>
         </is>
       </c>
       <c r="H39" s="11" t="inlineStr">
         <is>
-          <t>5N</t>
+          <t>CVD-LAB-A</t>
         </is>
       </c>
       <c r="I39" s="11" t="inlineStr">
         <is>
-          <t>review</t>
-        </is>
-      </c>
-      <c r="J39" s="11" t="inlineStr">
-        <is>
-          <t>base纯度的数值百分比为权威值；这里只保留供应商标签</t>
-        </is>
-      </c>
+          <t>2026-07-28用户逐项复核</t>
+        </is>
+      </c>
+      <c r="J39" s="11" t="inlineStr"/>
       <c r="K39" s="11" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="11" t="inlineStr">
         <is>
-          <t>MaterialLot</t>
+          <t>装置Setup</t>
         </is>
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>▸气瓶·气瓶编号</t>
+          <t>改造内容</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>钢瓶追溯号</t>
+          <t>相对原设备发生变化且会影响实验条件或复现的改造</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -7914,38 +7858,74 @@
       </c>
       <c r="G40" s="16" t="inlineStr">
         <is>
-          <t>选填</t>
+          <t>条件选填(改造设备)</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>GC-Ar-07</t>
+          <t>更换三温区加热模块并增加独立控温</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>2026-07-28用户逐项复核</t>
         </is>
       </c>
       <c r="J40" s="11" t="inlineStr"/>
       <c r="K40" s="11" t="inlineStr"/>
     </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="10" t="inlineStr">
-        <is>
-          <t>实体② 装置库 Setup（一台炉登记一次，实验 §2 引用；坐标系随引用冻结）</t>
-        </is>
-      </c>
-      <c r="B41" s="8" t="n"/>
-      <c r="C41" s="8" t="n"/>
-      <c r="D41" s="8" t="n"/>
-      <c r="E41" s="8" t="n"/>
-      <c r="F41" s="8" t="n"/>
-      <c r="G41" s="8" t="n"/>
-      <c r="H41" s="8" t="n"/>
-      <c r="I41" s="8" t="n"/>
-      <c r="J41" s="8" t="n"/>
-      <c r="K41" s="8" t="n"/>
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>装置Setup</t>
+        </is>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>实验室装置编号（资产编号）</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>课题组用于识别这台装置的唯一业务编号；系统内部身份使用不可变UUID</t>
+        </is>
+      </c>
+      <c r="D41" s="11" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="E41" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F41" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G41" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
+        </is>
+      </c>
+      <c r="H41" s="11" t="inlineStr">
+        <is>
+          <t>CVD-炉1</t>
+        </is>
+      </c>
+      <c r="I41" s="11" t="inlineStr">
+        <is>
+          <t>review§4.1B·2026-07-27终版整改</t>
+        </is>
+      </c>
+      <c r="J41" s="11" t="inlineStr">
+        <is>
+          <t>要求唯一；仅管理员可通过新版本纠正录入错误，历史版本保留原编号</t>
+        </is>
+      </c>
+      <c r="K41" s="11" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="11" t="inlineStr">
@@ -7955,17 +7935,17 @@
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>装置名称</t>
+          <t>温区数</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>人读名</t>
+          <t>独立控温区数</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="E42" s="11" t="inlineStr">
@@ -7975,7 +7955,7 @@
       </c>
       <c r="F42" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>个</t>
         </is>
       </c>
       <c r="G42" s="12" t="inlineStr">
@@ -7985,7 +7965,7 @@
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>1号双温区管式炉</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
@@ -7994,7 +7974,11 @@
         </is>
       </c>
       <c r="J42" s="11" t="inlineStr"/>
-      <c r="K42" s="11" t="inlineStr"/>
+      <c r="K42" s="11" t="inlineStr">
+        <is>
+          <t>{"ge":1,"type":"integer"}</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="11" t="inlineStr">
@@ -8004,27 +7988,27 @@
       </c>
       <c r="B43" s="11" t="inlineStr">
         <is>
-          <t>版本号</t>
+          <t>各温区温度传感器</t>
         </is>
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>每次修改+1；引用时冻结此版本</t>
+          <t>装置每个温区的传感器类别，以及设备资料明确给出时的标称测温精度</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>温度传感器数组</t>
         </is>
       </c>
       <c r="E43" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>{sensor_type: thermocouple|rtd|infrared_thermometer|fiber_optic_temperature_sensor|thermistor|other, sensor_type_other?, zone_index, nominal_accuracy_C?}</t>
         </is>
       </c>
       <c r="F43" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>℃</t>
         </is>
       </c>
       <c r="G43" s="12" t="inlineStr">
@@ -8034,17 +8018,17 @@
       </c>
       <c r="H43" s="11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>[{sensor_type: 热电偶, zone_index: 1, nominal_accuracy_C: 1}]</t>
         </is>
       </c>
       <c r="I43" s="11" t="inlineStr">
         <is>
-          <t>★锁版使能(Fable三轮B2)</t>
+          <t>2026-07-24导师走查·2026-07-27终版整改·2026-07-28用户复核</t>
         </is>
       </c>
       <c r="J43" s="11" t="inlineStr">
         <is>
-          <t>对标 v1 setup_version_snapshot</t>
+          <t>温区数决定卡片数量；传感器类别必填；标称测温精度仅在设备资料明确提供时填写，不要求用户估算</t>
         </is>
       </c>
       <c r="K43" s="11" t="inlineStr"/>
@@ -8057,12 +8041,12 @@
       </c>
       <c r="B44" s="11" t="inlineStr">
         <is>
-          <t>装置来源</t>
+          <t>炉体方向</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>装置是商业购买、实验室自制还是在既有设备上改造</t>
+          <t>水平/垂直</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -8072,7 +8056,7 @@
       </c>
       <c r="E44" s="11" t="inlineStr">
         <is>
-          <t>商业设备/实验室自制/改造设备</t>
+          <t>水平/垂直</t>
         </is>
       </c>
       <c r="F44" s="11" t="inlineStr">
@@ -8087,12 +8071,12 @@
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>商业设备</t>
+          <t>水平</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28用户逐项复核</t>
+          <t>会议</t>
         </is>
       </c>
       <c r="J44" s="11" t="inlineStr"/>
@@ -8106,22 +8090,22 @@
       </c>
       <c r="B45" s="11" t="inlineStr">
         <is>
-          <t>制造商或品牌</t>
+          <t>炉管材质与截面</t>
         </is>
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>设备制造商或品牌，独立于型号保存以支持筛选和统计</t>
+          <t>炉管材料与截面</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>管材质形状对象</t>
         </is>
       </c>
       <c r="E45" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>{material: 石英|刚玉|其他, material_other?, shape: 圆形|方形|矩形|其他, shape_other?}</t>
         </is>
       </c>
       <c r="F45" s="11" t="inlineStr">
@@ -8129,22 +8113,26 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G45" s="16" t="inlineStr">
-        <is>
-          <t>条件选填(商业设备或改造设备)</t>
+      <c r="G45" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
         </is>
       </c>
       <c r="H45" s="11" t="inlineStr">
         <is>
-          <t>合肥科晶</t>
+          <t>{material: 石英, shape: 圆形}</t>
         </is>
       </c>
       <c r="I45" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28用户逐项复核</t>
-        </is>
-      </c>
-      <c r="J45" s="11" t="inlineStr"/>
+          <t>2026-07-24导师走查</t>
+        </is>
+      </c>
+      <c r="J45" s="11" t="inlineStr">
+        <is>
+          <t>材质与截面形状独立保存，禁止把“刚玉；圆”当作一个选项</t>
+        </is>
+      </c>
       <c r="K45" s="11" t="inlineStr"/>
     </row>
     <row r="46">
@@ -8155,45 +8143,49 @@
       </c>
       <c r="B46" s="11" t="inlineStr">
         <is>
-          <t>型号</t>
+          <t>炉管尺寸</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>制造商给出的设备型号</t>
+          <t>按截面形状记录外部尺寸和壁厚</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>炉管尺寸对象</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>{圆形: outer_diameter_mm+wall_thickness_mm; 方形: outer_side_mm+wall_thickness_mm; 矩形: outer_width_mm+outer_height_mm+wall_thickness_mm; 其他: dimension_description}</t>
         </is>
       </c>
       <c r="F46" s="11" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G46" s="16" t="inlineStr">
-        <is>
-          <t>条件选填(商业设备或改造设备)</t>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="G46" s="12" t="inlineStr">
+        <is>
+          <t>必填；按炉管截面填写</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>OTF-1200X</t>
+          <t>{outer_width_mm: 50, outer_height_mm: 30, wall_thickness_mm: 2}</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28用户逐项复核</t>
-        </is>
-      </c>
-      <c r="J46" s="11" t="inlineStr"/>
+          <t>会议·用户复核2026-07-24</t>
+        </is>
+      </c>
+      <c r="J46" s="11" t="inlineStr">
+        <is>
+          <t>选择材质与截面后必须按形状完整填写；圆形填外径+壁厚，方形填外边长+壁厚，矩形填外宽+外高+壁厚，其他截面填写具名尺寸说明</t>
+        </is>
+      </c>
       <c r="K46" s="11" t="inlineStr"/>
     </row>
     <row r="47">
@@ -8204,22 +8196,22 @@
       </c>
       <c r="B47" s="11" t="inlineStr">
         <is>
-          <t>设计或建造单位</t>
+          <t>壁型</t>
         </is>
       </c>
       <c r="C47" s="11" t="inlineStr">
         <is>
-          <t>实验室自制装置的设计或建造单位</t>
+          <t>热壁/冷壁</t>
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>下拉</t>
         </is>
       </c>
       <c r="E47" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>热壁/冷壁</t>
         </is>
       </c>
       <c r="F47" s="11" t="inlineStr">
@@ -8227,22 +8219,26 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G47" s="16" t="inlineStr">
-        <is>
-          <t>条件选填(实验室自制)</t>
+      <c r="G47" s="15" t="inlineStr">
+        <is>
+          <t>推荐</t>
         </is>
       </c>
       <c r="H47" s="11" t="inlineStr">
         <is>
-          <t>二维材料课题组</t>
+          <t>热壁</t>
         </is>
       </c>
       <c r="I47" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28用户逐项复核</t>
-        </is>
-      </c>
-      <c r="J47" s="11" t="inlineStr"/>
+          <t>复审</t>
+        </is>
+      </c>
+      <c r="J47" s="11" t="inlineStr">
+        <is>
+          <t>放在装置身份、温区与炉管结构之后，避免打断由粗到细的登记顺序</t>
+        </is>
+      </c>
       <c r="K47" s="11" t="inlineStr"/>
     </row>
     <row r="48">
@@ -8253,22 +8249,22 @@
       </c>
       <c r="B48" s="11" t="inlineStr">
         <is>
-          <t>内部型号</t>
+          <t>坐标系定义</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>实验室自制装置使用的内部型号或版本名称</t>
+          <t>系统统一采用上游为负、下游为正的固定坐标定义</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>固定定义</t>
         </is>
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>上游为负；下游为正；原点固定</t>
         </is>
       </c>
       <c r="F48" s="11" t="inlineStr">
@@ -8276,22 +8272,26 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G48" s="16" t="inlineStr">
-        <is>
-          <t>条件选填(实验室自制)</t>
+      <c r="G48" s="17" t="inlineStr">
+        <is>
+          <t>定义项</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>CVD-LAB-A</t>
+          <t>上游(-)←原点→下游(+)</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28用户逐项复核</t>
-        </is>
-      </c>
-      <c r="J48" s="11" t="inlineStr"/>
+          <t>2026-07-24导师走查</t>
+        </is>
+      </c>
+      <c r="J48" s="11" t="inlineStr">
+        <is>
+          <t>服务端写入固定机器码，管理员和成员均不可编辑</t>
+        </is>
+      </c>
       <c r="K48" s="11" t="inlineStr"/>
     </row>
     <row r="49">
@@ -8302,22 +8302,22 @@
       </c>
       <c r="B49" s="11" t="inlineStr">
         <is>
-          <t>改造内容</t>
+          <t>外场能力</t>
         </is>
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>相对原设备发生变化且会影响实验条件或复现的改造</t>
+          <t>装置具备的光、电或等离子体能力</t>
         </is>
       </c>
       <c r="D49" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>多选</t>
         </is>
       </c>
       <c r="E49" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>无/光/电/等离子体</t>
         </is>
       </c>
       <c r="F49" s="11" t="inlineStr">
@@ -8325,22 +8325,26 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G49" s="16" t="inlineStr">
-        <is>
-          <t>条件选填(改造设备)</t>
+      <c r="G49" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
         </is>
       </c>
       <c r="H49" s="11" t="inlineStr">
         <is>
-          <t>更换三温区加热模块并增加独立控温</t>
+          <t>无</t>
         </is>
       </c>
       <c r="I49" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28用户逐项复核</t>
-        </is>
-      </c>
-      <c r="J49" s="11" t="inlineStr"/>
+          <t>2026-07-24导师走查</t>
+        </is>
+      </c>
+      <c r="J49" s="11" t="inlineStr">
+        <is>
+          <t>这里只登记能力；每炉实际使用情况在反应条件中记录</t>
+        </is>
+      </c>
       <c r="K49" s="11" t="inlineStr"/>
     </row>
     <row r="50">
@@ -8351,22 +8355,22 @@
       </c>
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>实验室装置编号（资产编号）</t>
+          <t>装置示意图与描述</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>课题组用于识别这台装置的唯一业务编号；系统内部身份使用不可变UUID</t>
+          <t>装置照片或示意图及文字说明</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>FileAsset引用+自由</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>{file_asset_id, sha256, note}</t>
         </is>
       </c>
       <c r="F50" s="11" t="inlineStr">
@@ -8374,26 +8378,22 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G50" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
+      <c r="G50" s="15" t="inlineStr">
+        <is>
+          <t>推荐</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>CVD-炉1</t>
+          <t>setup.png</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>review§4.1B·2026-07-27终版整改</t>
-        </is>
-      </c>
-      <c r="J50" s="11" t="inlineStr">
-        <is>
-          <t>要求唯一；仅管理员可通过新版本纠正录入错误，历史版本保留原编号</t>
-        </is>
-      </c>
+          <t>会议</t>
+        </is>
+      </c>
+      <c r="J50" s="11" t="inlineStr"/>
       <c r="K50" s="11" t="inlineStr"/>
     </row>
     <row r="51">
@@ -8404,128 +8404,92 @@
       </c>
       <c r="B51" s="11" t="inlineStr">
         <is>
-          <t>温区数</t>
+          <t>可更换部件绑定</t>
         </is>
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t>独立控温区数</t>
+          <t>当前Setup版本实际安装的炉管、传感器、MFC、压力计等部件</t>
         </is>
       </c>
       <c r="D51" s="11" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>JSON数组</t>
         </is>
       </c>
       <c r="E51" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>[{component_id,role,position?}]</t>
         </is>
       </c>
       <c r="F51" s="11" t="inlineStr">
         <is>
-          <t>个</t>
-        </is>
-      </c>
-      <c r="G51" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G51" s="15" t="inlineStr">
+        <is>
+          <t>推荐</t>
         </is>
       </c>
       <c r="H51" s="11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>[{"component_id":"UUID","role":"furnace_tube"}]</t>
         </is>
       </c>
       <c r="I51" s="11" t="inlineStr">
         <is>
-          <t>会议</t>
-        </is>
-      </c>
-      <c r="J51" s="11" t="inlineStr"/>
-      <c r="K51" s="11" t="inlineStr">
-        <is>
-          <t>{"ge":1,"type":"integer"}</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="11" t="inlineStr">
-        <is>
-          <t>装置Setup</t>
-        </is>
-      </c>
-      <c r="B52" s="11" t="inlineStr">
-        <is>
-          <t>各温区温度传感器</t>
-        </is>
-      </c>
-      <c r="C52" s="11" t="inlineStr">
-        <is>
-          <t>装置每个温区的传感器类别，以及设备资料明确给出时的标称测温精度</t>
-        </is>
-      </c>
-      <c r="D52" s="11" t="inlineStr">
-        <is>
-          <t>温度传感器数组</t>
-        </is>
-      </c>
-      <c r="E52" s="11" t="inlineStr">
-        <is>
-          <t>{sensor_type: thermocouple|rtd|infrared_thermometer|fiber_optic_temperature_sensor|thermistor|other, sensor_type_other?, zone_index, nominal_accuracy_C?}</t>
-        </is>
-      </c>
-      <c r="F52" s="11" t="inlineStr">
-        <is>
-          <t>℃</t>
-        </is>
-      </c>
-      <c r="G52" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
-        </is>
-      </c>
-      <c r="H52" s="11" t="inlineStr">
-        <is>
-          <t>[{sensor_type: 热电偶, zone_index: 1, nominal_accuracy_C: 1}]</t>
-        </is>
-      </c>
-      <c r="I52" s="11" t="inlineStr">
-        <is>
-          <t>2026-07-24导师走查·2026-07-27终版整改·2026-07-28用户复核</t>
-        </is>
-      </c>
-      <c r="J52" s="11" t="inlineStr">
-        <is>
-          <t>温区数决定卡片数量；传感器类别必填；标称测温精度仅在设备资料明确提供时填写，不要求用户估算</t>
-        </is>
-      </c>
-      <c r="K52" s="11" t="inlineStr"/>
+          <t>2026-07-28深度审查</t>
+        </is>
+      </c>
+      <c r="J51" s="11" t="inlineStr">
+        <is>
+          <t>部件身份、校准和维护走独立生命周期事件</t>
+        </is>
+      </c>
+      <c r="K51" s="11" t="inlineStr"/>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>实体③ 表征仪器 Instrument（实验 §7 表征引用；对标 NeXus NXfabrication 仪器溯源）</t>
+        </is>
+      </c>
+      <c r="B52" s="8" t="n"/>
+      <c r="C52" s="8" t="n"/>
+      <c r="D52" s="8" t="n"/>
+      <c r="E52" s="8" t="n"/>
+      <c r="F52" s="8" t="n"/>
+      <c r="G52" s="8" t="n"/>
+      <c r="H52" s="8" t="n"/>
+      <c r="I52" s="8" t="n"/>
+      <c r="J52" s="8" t="n"/>
+      <c r="K52" s="8" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="11" t="inlineStr">
         <is>
-          <t>装置Setup</t>
+          <t>表征仪器</t>
         </is>
       </c>
       <c r="B53" s="11" t="inlineStr">
         <is>
-          <t>炉体方向</t>
+          <t>仪器编号</t>
         </is>
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>水平/垂直</t>
+          <t>唯一编号</t>
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr">
         <is>
-          <t>下拉</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E53" s="11" t="inlineStr">
         <is>
-          <t>水平/垂直</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F53" s="11" t="inlineStr">
@@ -8540,12 +8504,12 @@
       </c>
       <c r="H53" s="11" t="inlineStr">
         <is>
-          <t>水平</t>
+          <t>RAMAN-1</t>
         </is>
       </c>
       <c r="I53" s="11" t="inlineStr">
         <is>
-          <t>会议</t>
+          <t>复审</t>
         </is>
       </c>
       <c r="J53" s="11" t="inlineStr"/>
@@ -8554,27 +8518,27 @@
     <row r="54">
       <c r="A54" s="11" t="inlineStr">
         <is>
-          <t>装置Setup</t>
+          <t>表征仪器</t>
         </is>
       </c>
       <c r="B54" s="11" t="inlineStr">
         <is>
-          <t>炉管材质与截面</t>
+          <t>适用表征方法</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>炉管材料与截面</t>
+          <t>该仪器适用的表征方法，用于结果录入时筛选仪器</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>管材质形状对象</t>
+          <t>下拉+其他</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
-          <t>{material: 石英|刚玉|其他, material_other?, shape: 圆形|方形|矩形|其他, shape_other?}</t>
+          <t>光镜/SEM/Raman/低波数Raman/PL/AFM/XRD/TEM/其他</t>
         </is>
       </c>
       <c r="F54" s="11" t="inlineStr">
@@ -8589,17 +8553,17 @@
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>{material: 石英, shape: 圆形}</t>
+          <t>Raman</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>2026-07-24导师走查</t>
+          <t>会议</t>
         </is>
       </c>
       <c r="J54" s="11" t="inlineStr">
         <is>
-          <t>材质与截面形状独立保存，禁止把“刚玉；圆”当作一个选项</t>
+          <t>API key 保持 name_type 以兼容现有数据</t>
         </is>
       </c>
       <c r="K54" s="11" t="inlineStr"/>
@@ -8607,80 +8571,76 @@
     <row r="55">
       <c r="A55" s="11" t="inlineStr">
         <is>
-          <t>装置Setup</t>
+          <t>表征仪器</t>
         </is>
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
-          <t>炉管尺寸</t>
+          <t>厂商</t>
         </is>
       </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>按截面形状记录外部尺寸和壁厚</t>
+          <t>品牌</t>
         </is>
       </c>
       <c r="D55" s="11" t="inlineStr">
         <is>
-          <t>炉管尺寸对象</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E55" s="11" t="inlineStr">
         <is>
-          <t>{圆形: outer_diameter_mm+wall_thickness_mm; 方形: outer_side_mm+wall_thickness_mm; 矩形: outer_width_mm+outer_height_mm+wall_thickness_mm; 其他: dimension_description}</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F55" s="11" t="inlineStr">
         <is>
-          <t>mm</t>
-        </is>
-      </c>
-      <c r="G55" s="12" t="inlineStr">
-        <is>
-          <t>必填；按炉管截面填写</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G55" s="15" t="inlineStr">
+        <is>
+          <t>推荐</t>
         </is>
       </c>
       <c r="H55" s="11" t="inlineStr">
         <is>
-          <t>{outer_width_mm: 50, outer_height_mm: 30, wall_thickness_mm: 2}</t>
+          <t>Horiba</t>
         </is>
       </c>
       <c r="I55" s="11" t="inlineStr">
         <is>
-          <t>会议·用户复核2026-07-24</t>
-        </is>
-      </c>
-      <c r="J55" s="11" t="inlineStr">
-        <is>
-          <t>选择材质与截面后必须按形状完整填写；圆形填外径+壁厚，方形填外边长+壁厚，矩形填外宽+外高+壁厚，其他截面填写具名尺寸说明</t>
-        </is>
-      </c>
+          <t>★NXfabrication</t>
+        </is>
+      </c>
+      <c r="J55" s="11" t="inlineStr"/>
       <c r="K55" s="11" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="inlineStr">
         <is>
-          <t>装置Setup</t>
+          <t>表征仪器</t>
         </is>
       </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
-          <t>壁型</t>
+          <t>型号</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>热壁/冷壁</t>
+          <t>型号</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>下拉</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>热壁/冷壁</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F56" s="11" t="inlineStr">
@@ -8695,45 +8655,41 @@
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>热壁</t>
+          <t>LabRAM HR</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>复审</t>
-        </is>
-      </c>
-      <c r="J56" s="11" t="inlineStr">
-        <is>
-          <t>放在装置身份、温区与炉管结构之后，避免打断由粗到细的登记顺序</t>
-        </is>
-      </c>
+          <t>★NXfabrication</t>
+        </is>
+      </c>
+      <c r="J56" s="11" t="inlineStr"/>
       <c r="K56" s="11" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="inlineStr">
         <is>
-          <t>装置Setup</t>
+          <t>表征仪器</t>
         </is>
       </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
-          <t>坐标系定义</t>
+          <t>序列号</t>
         </is>
       </c>
       <c r="C57" s="11" t="inlineStr">
         <is>
-          <t>系统统一采用上游为负、下游为正的固定坐标定义</t>
+          <t>设备序列号</t>
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr">
         <is>
-          <t>固定定义</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E57" s="11" t="inlineStr">
         <is>
-          <t>上游为负；下游为正；原点固定</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F57" s="11" t="inlineStr">
@@ -8741,52 +8697,48 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G57" s="17" t="inlineStr">
-        <is>
-          <t>定义项</t>
+      <c r="G57" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
         </is>
       </c>
       <c r="H57" s="11" t="inlineStr">
         <is>
-          <t>上游(-)←原点→下游(+)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I57" s="11" t="inlineStr">
         <is>
-          <t>2026-07-24导师走查</t>
-        </is>
-      </c>
-      <c r="J57" s="11" t="inlineStr">
-        <is>
-          <t>服务端写入固定机器码，管理员和成员均不可编辑</t>
-        </is>
-      </c>
+          <t>★NXfabrication</t>
+        </is>
+      </c>
+      <c r="J57" s="11" t="inlineStr"/>
       <c r="K57" s="11" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="11" t="inlineStr">
         <is>
-          <t>装置Setup</t>
+          <t>表征仪器</t>
         </is>
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
-          <t>外场能力</t>
+          <t>仪器持久标识</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>装置具备的光、电或等离子体能力</t>
+          <t>可长期稳定指向该仪器的公开或机构标识，不等同于设备序列号</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>多选</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E58" s="11" t="inlineStr">
         <is>
-          <t>无/光/电/等离子体</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F58" s="11" t="inlineStr">
@@ -8794,24 +8746,24 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G58" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
+      <c r="G58" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>2026-07-24导师走查</t>
+          <t>★NXfabrication/PIDINST</t>
         </is>
       </c>
       <c r="J58" s="11" t="inlineStr">
         <is>
-          <t>这里只登记能力；每炉实际使用情况在反应条件中记录</t>
+          <t>PID 是 Persistent Identifier 的缩写；没有机构标识时可留空</t>
         </is>
       </c>
       <c r="K58" s="11" t="inlineStr"/>
@@ -8819,27 +8771,27 @@
     <row r="59">
       <c r="A59" s="11" t="inlineStr">
         <is>
-          <t>装置Setup</t>
+          <t>表征仪器</t>
         </is>
       </c>
       <c r="B59" s="11" t="inlineStr">
         <is>
-          <t>装置示意图与描述</t>
+          <t>所在实验室与位置</t>
         </is>
       </c>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>装置照片或示意图及文字说明</t>
+          <t>物理位置</t>
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr">
         <is>
-          <t>FileAsset引用+自由</t>
+          <t>文本</t>
         </is>
       </c>
       <c r="E59" s="11" t="inlineStr">
         <is>
-          <t>{file_asset_id, sha256, note}</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F59" s="11" t="inlineStr">
@@ -8847,19 +8799,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G59" s="15" t="inlineStr">
-        <is>
-          <t>推荐</t>
+      <c r="G59" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
         </is>
       </c>
       <c r="H59" s="11" t="inlineStr">
         <is>
-          <t>setup.png</t>
+          <t>A305</t>
         </is>
       </c>
       <c r="I59" s="11" t="inlineStr">
         <is>
-          <t>会议</t>
+          <t>建议</t>
         </is>
       </c>
       <c r="J59" s="11" t="inlineStr"/>
@@ -8868,72 +8820,108 @@
     <row r="60">
       <c r="A60" s="11" t="inlineStr">
         <is>
-          <t>装置Setup</t>
+          <t>表征仪器</t>
         </is>
       </c>
       <c r="B60" s="11" t="inlineStr">
         <is>
-          <t>可更换部件绑定</t>
+          <t>关键固定配置</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>当前Setup版本实际安装的炉管、传感器、MFC、压力计等部件</t>
+          <t>随仪器长期固定的硬件或能力；本次实际使用参数在表征结果的测试条件中填写</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
+          <t>自由</t>
+        </is>
+      </c>
+      <c r="E60" s="11" t="inlineStr">
+        <is>
+          <t>如探测器型号、光栅范围、可用激光与物镜范围</t>
+        </is>
+      </c>
+      <c r="F60" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G60" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
+        </is>
+      </c>
+      <c r="H60" s="11" t="inlineStr">
+        <is>
+          <t>CCD探测器；300、600、1800 lines·mm⁻¹光栅</t>
+        </is>
+      </c>
+      <c r="I60" s="11" t="inlineStr">
+        <is>
+          <t>会议</t>
+        </is>
+      </c>
+      <c r="J60" s="11" t="inlineStr">
+        <is>
+          <t>不在此重复本次实际使用的波长、物镜、功率或积分时间</t>
+        </is>
+      </c>
+      <c r="K60" s="11" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="11" t="inlineStr">
+        <is>
+          <t>表征仪器</t>
+        </is>
+      </c>
+      <c r="B61" s="11" t="inlineStr">
+        <is>
+          <t>测量能力配置</t>
+        </is>
+      </c>
+      <c r="C61" s="11" t="inlineStr">
+        <is>
+          <t>仪器版本支持的测量方法及其可选固定配置</t>
+        </is>
+      </c>
+      <c r="D61" s="11" t="inlineStr">
+        <is>
           <t>JSON数组</t>
         </is>
       </c>
-      <c r="E60" s="11" t="inlineStr">
-        <is>
-          <t>[{component_id,role,position?}]</t>
-        </is>
-      </c>
-      <c r="F60" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G60" s="15" t="inlineStr">
-        <is>
-          <t>推荐</t>
-        </is>
-      </c>
-      <c r="H60" s="11" t="inlineStr">
-        <is>
-          <t>[{"component_id":"UUID","role":"furnace_tube"}]</t>
-        </is>
-      </c>
-      <c r="I60" s="11" t="inlineStr">
+      <c r="E61" s="11" t="inlineStr">
+        <is>
+          <t>[{code,configuration}]</t>
+        </is>
+      </c>
+      <c r="F61" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G61" s="12" t="inlineStr">
+        <is>
+          <t>必填</t>
+        </is>
+      </c>
+      <c r="H61" s="11" t="inlineStr">
+        <is>
+          <t>[{"code":"Raman","configuration":{"lasers_nm":[532]}}]</t>
+        </is>
+      </c>
+      <c r="I61" s="11" t="inlineStr">
         <is>
           <t>2026-07-28深度审查</t>
         </is>
       </c>
-      <c r="J60" s="11" t="inlineStr">
-        <is>
-          <t>部件身份、校准和维护走独立生命周期事件</t>
-        </is>
-      </c>
-      <c r="K60" s="11" t="inlineStr"/>
-    </row>
-    <row r="61" ht="20" customHeight="1">
-      <c r="A61" s="10" t="inlineStr">
-        <is>
-          <t>实体③ 表征仪器 Instrument（实验 §7 表征引用；对标 NeXus NXfabrication 仪器溯源）</t>
-        </is>
-      </c>
-      <c r="B61" s="8" t="n"/>
-      <c r="C61" s="8" t="n"/>
-      <c r="D61" s="8" t="n"/>
-      <c r="E61" s="8" t="n"/>
-      <c r="F61" s="8" t="n"/>
-      <c r="G61" s="8" t="n"/>
-      <c r="H61" s="8" t="n"/>
-      <c r="I61" s="8" t="n"/>
-      <c r="J61" s="8" t="n"/>
-      <c r="K61" s="8" t="n"/>
+      <c r="J61" s="11" t="inlineStr">
+        <is>
+          <t>本次MeasurementRun只能选择这里声明的能力</t>
+        </is>
+      </c>
+      <c r="K61" s="11" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
@@ -8943,17 +8931,17 @@
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>仪器编号</t>
+          <t>最近校准或维护日期</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>唯一编号</t>
+          <t>校准/维护日期</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>日期</t>
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr">
@@ -8966,486 +8954,29 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G62" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
+      <c r="G62" s="16" t="inlineStr">
+        <is>
+          <t>选填</t>
         </is>
       </c>
       <c r="H62" s="11" t="inlineStr">
         <is>
-          <t>RAMAN-1</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="I62" s="11" t="inlineStr">
         <is>
-          <t>复审</t>
+          <t>会议</t>
         </is>
       </c>
       <c r="J62" s="11" t="inlineStr"/>
       <c r="K62" s="11" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="11" t="inlineStr">
-        <is>
-          <t>表征仪器</t>
-        </is>
-      </c>
-      <c r="B63" s="11" t="inlineStr">
-        <is>
-          <t>适用表征方法</t>
-        </is>
-      </c>
-      <c r="C63" s="11" t="inlineStr">
-        <is>
-          <t>该仪器适用的表征方法，用于结果录入时筛选仪器</t>
-        </is>
-      </c>
-      <c r="D63" s="11" t="inlineStr">
-        <is>
-          <t>下拉+其他</t>
-        </is>
-      </c>
-      <c r="E63" s="11" t="inlineStr">
-        <is>
-          <t>光镜/SEM/Raman/低波数Raman/PL/AFM/XRD/TEM/其他</t>
-        </is>
-      </c>
-      <c r="F63" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G63" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
-        </is>
-      </c>
-      <c r="H63" s="11" t="inlineStr">
-        <is>
-          <t>Raman</t>
-        </is>
-      </c>
-      <c r="I63" s="11" t="inlineStr">
-        <is>
-          <t>会议</t>
-        </is>
-      </c>
-      <c r="J63" s="11" t="inlineStr">
-        <is>
-          <t>API key 保持 name_type 以兼容现有数据</t>
-        </is>
-      </c>
-      <c r="K63" s="11" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="11" t="inlineStr">
-        <is>
-          <t>表征仪器</t>
-        </is>
-      </c>
-      <c r="B64" s="11" t="inlineStr">
-        <is>
-          <t>厂商</t>
-        </is>
-      </c>
-      <c r="C64" s="11" t="inlineStr">
-        <is>
-          <t>品牌</t>
-        </is>
-      </c>
-      <c r="D64" s="11" t="inlineStr">
-        <is>
-          <t>文本</t>
-        </is>
-      </c>
-      <c r="E64" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F64" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G64" s="15" t="inlineStr">
-        <is>
-          <t>推荐</t>
-        </is>
-      </c>
-      <c r="H64" s="11" t="inlineStr">
-        <is>
-          <t>Horiba</t>
-        </is>
-      </c>
-      <c r="I64" s="11" t="inlineStr">
-        <is>
-          <t>★NXfabrication</t>
-        </is>
-      </c>
-      <c r="J64" s="11" t="inlineStr"/>
-      <c r="K64" s="11" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="11" t="inlineStr">
-        <is>
-          <t>表征仪器</t>
-        </is>
-      </c>
-      <c r="B65" s="11" t="inlineStr">
-        <is>
-          <t>型号</t>
-        </is>
-      </c>
-      <c r="C65" s="11" t="inlineStr">
-        <is>
-          <t>型号</t>
-        </is>
-      </c>
-      <c r="D65" s="11" t="inlineStr">
-        <is>
-          <t>文本</t>
-        </is>
-      </c>
-      <c r="E65" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F65" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G65" s="15" t="inlineStr">
-        <is>
-          <t>推荐</t>
-        </is>
-      </c>
-      <c r="H65" s="11" t="inlineStr">
-        <is>
-          <t>LabRAM HR</t>
-        </is>
-      </c>
-      <c r="I65" s="11" t="inlineStr">
-        <is>
-          <t>★NXfabrication</t>
-        </is>
-      </c>
-      <c r="J65" s="11" t="inlineStr"/>
-      <c r="K65" s="11" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="11" t="inlineStr">
-        <is>
-          <t>表征仪器</t>
-        </is>
-      </c>
-      <c r="B66" s="11" t="inlineStr">
-        <is>
-          <t>序列号</t>
-        </is>
-      </c>
-      <c r="C66" s="11" t="inlineStr">
-        <is>
-          <t>设备序列号</t>
-        </is>
-      </c>
-      <c r="D66" s="11" t="inlineStr">
-        <is>
-          <t>文本</t>
-        </is>
-      </c>
-      <c r="E66" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F66" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G66" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
-        </is>
-      </c>
-      <c r="H66" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I66" s="11" t="inlineStr">
-        <is>
-          <t>★NXfabrication</t>
-        </is>
-      </c>
-      <c r="J66" s="11" t="inlineStr"/>
-      <c r="K66" s="11" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="11" t="inlineStr">
-        <is>
-          <t>表征仪器</t>
-        </is>
-      </c>
-      <c r="B67" s="11" t="inlineStr">
-        <is>
-          <t>仪器持久标识</t>
-        </is>
-      </c>
-      <c r="C67" s="11" t="inlineStr">
-        <is>
-          <t>可长期稳定指向该仪器的公开或机构标识，不等同于设备序列号</t>
-        </is>
-      </c>
-      <c r="D67" s="11" t="inlineStr">
-        <is>
-          <t>文本</t>
-        </is>
-      </c>
-      <c r="E67" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F67" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G67" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
-        </is>
-      </c>
-      <c r="H67" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I67" s="11" t="inlineStr">
-        <is>
-          <t>★NXfabrication/PIDINST</t>
-        </is>
-      </c>
-      <c r="J67" s="11" t="inlineStr">
-        <is>
-          <t>PID 是 Persistent Identifier 的缩写；没有机构标识时可留空</t>
-        </is>
-      </c>
-      <c r="K67" s="11" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="11" t="inlineStr">
-        <is>
-          <t>表征仪器</t>
-        </is>
-      </c>
-      <c r="B68" s="11" t="inlineStr">
-        <is>
-          <t>所在实验室与位置</t>
-        </is>
-      </c>
-      <c r="C68" s="11" t="inlineStr">
-        <is>
-          <t>物理位置</t>
-        </is>
-      </c>
-      <c r="D68" s="11" t="inlineStr">
-        <is>
-          <t>文本</t>
-        </is>
-      </c>
-      <c r="E68" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F68" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G68" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
-        </is>
-      </c>
-      <c r="H68" s="11" t="inlineStr">
-        <is>
-          <t>A305</t>
-        </is>
-      </c>
-      <c r="I68" s="11" t="inlineStr">
-        <is>
-          <t>建议</t>
-        </is>
-      </c>
-      <c r="J68" s="11" t="inlineStr"/>
-      <c r="K68" s="11" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="11" t="inlineStr">
-        <is>
-          <t>表征仪器</t>
-        </is>
-      </c>
-      <c r="B69" s="11" t="inlineStr">
-        <is>
-          <t>关键固定配置</t>
-        </is>
-      </c>
-      <c r="C69" s="11" t="inlineStr">
-        <is>
-          <t>随仪器长期固定的硬件或能力；本次实际使用参数在表征结果的测试条件中填写</t>
-        </is>
-      </c>
-      <c r="D69" s="11" t="inlineStr">
-        <is>
-          <t>自由</t>
-        </is>
-      </c>
-      <c r="E69" s="11" t="inlineStr">
-        <is>
-          <t>如探测器型号、光栅范围、可用激光与物镜范围</t>
-        </is>
-      </c>
-      <c r="F69" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G69" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
-        </is>
-      </c>
-      <c r="H69" s="11" t="inlineStr">
-        <is>
-          <t>CCD探测器；300、600、1800 lines·mm⁻¹光栅</t>
-        </is>
-      </c>
-      <c r="I69" s="11" t="inlineStr">
-        <is>
-          <t>会议</t>
-        </is>
-      </c>
-      <c r="J69" s="11" t="inlineStr">
-        <is>
-          <t>不在此重复本次实际使用的波长、物镜、功率或积分时间</t>
-        </is>
-      </c>
-      <c r="K69" s="11" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="11" t="inlineStr">
-        <is>
-          <t>表征仪器</t>
-        </is>
-      </c>
-      <c r="B70" s="11" t="inlineStr">
-        <is>
-          <t>测量能力配置</t>
-        </is>
-      </c>
-      <c r="C70" s="11" t="inlineStr">
-        <is>
-          <t>仪器版本支持的测量方法及其可选固定配置</t>
-        </is>
-      </c>
-      <c r="D70" s="11" t="inlineStr">
-        <is>
-          <t>JSON数组</t>
-        </is>
-      </c>
-      <c r="E70" s="11" t="inlineStr">
-        <is>
-          <t>[{code,configuration}]</t>
-        </is>
-      </c>
-      <c r="F70" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G70" s="12" t="inlineStr">
-        <is>
-          <t>必填</t>
-        </is>
-      </c>
-      <c r="H70" s="11" t="inlineStr">
-        <is>
-          <t>[{"code":"Raman","configuration":{"lasers_nm":[532]}}]</t>
-        </is>
-      </c>
-      <c r="I70" s="11" t="inlineStr">
-        <is>
-          <t>2026-07-28深度审查</t>
-        </is>
-      </c>
-      <c r="J70" s="11" t="inlineStr">
-        <is>
-          <t>本次MeasurementRun只能选择这里声明的能力</t>
-        </is>
-      </c>
-      <c r="K70" s="11" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="11" t="inlineStr">
-        <is>
-          <t>表征仪器</t>
-        </is>
-      </c>
-      <c r="B71" s="11" t="inlineStr">
-        <is>
-          <t>最近校准或维护日期</t>
-        </is>
-      </c>
-      <c r="C71" s="11" t="inlineStr">
-        <is>
-          <t>校准/维护日期</t>
-        </is>
-      </c>
-      <c r="D71" s="11" t="inlineStr">
-        <is>
-          <t>日期</t>
-        </is>
-      </c>
-      <c r="E71" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F71" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G71" s="16" t="inlineStr">
-        <is>
-          <t>选填</t>
-        </is>
-      </c>
-      <c r="H71" s="11" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="I71" s="11" t="inlineStr">
-        <is>
-          <t>会议</t>
-        </is>
-      </c>
-      <c r="J71" s="11" t="inlineStr"/>
-      <c r="K71" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A41:K41"/>
-    <mergeCell ref="A61:K61"/>
+    <mergeCell ref="A52:K52"/>
+    <mergeCell ref="A32:K32"/>
     <mergeCell ref="A3:K3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9458,7 +8989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D67"/>
+  <dimension ref="A1:D76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10070,7 +9601,7 @@
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>AP/LP 冗余二选一敲定：保留合成方法 AP/LP，以校验规则强制与压力体系一致（不再悬置）</t>
+          <t>AP/LP 冗余二选一敲定：保留合成方法 AP/LP，以校验规则强制与反应压力条件一致（不再悬置）</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -10850,20 +10381,218 @@
     <row r="67">
       <c r="A67" s="11" t="inlineStr">
         <is>
+          <t>v4.0-alpha.5</t>
+        </is>
+      </c>
+      <c r="B67" s="11" t="inlineStr">
+        <is>
+          <t>实体/物料批次</t>
+        </is>
+      </c>
+      <c r="C67" s="11" t="inlineStr">
+        <is>
+          <t>CAS号与数值纯度改为有来源才选填；删除同义名、标识符、商业规格JSON、纯度基准/来源及D50四字段；供应商规格或等级按标签原文照录</t>
+        </is>
+      </c>
+      <c r="D67" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-02供应商资料复核与减负</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="inlineStr">
+        <is>
+          <t>v4.0-alpha.6</t>
+        </is>
+      </c>
+      <c r="B68" s="11" t="inlineStr">
+        <is>
+          <t>实体/物料批次</t>
+        </is>
+      </c>
+      <c r="C68" s="11" t="inlineStr">
+        <is>
+          <t>物料表单文案正式化：常规字段说明改为简短占位示例，仅为纯度及衬底规格等易误录字段保留必要说明；统一字段名称、中文标点和中英文术语</t>
+        </is>
+      </c>
+      <c r="D68" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-02用户界面复核</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="11" t="inlineStr">
+        <is>
+          <t>v4.0-alpha.7</t>
+        </is>
+      </c>
+      <c r="B69" s="11" t="inlineStr">
+        <is>
+          <t>实体/物料批次</t>
+        </is>
+      </c>
+      <c r="C69" s="11" t="inlineStr">
+        <is>
+          <t>化学式复用目标产物输入控件并提示元素与语法；货号与批号直接对应包装上的 Cat./Product No. 和 Lot/Batch No.，说明两者的产品与实物批次分工</t>
+        </is>
+      </c>
+      <c r="D69" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-06用户界面复核</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="inlineStr">
+        <is>
+          <t>v4.0-alpha.8</t>
+        </is>
+      </c>
+      <c r="B70" s="11" t="inlineStr">
+        <is>
+          <t>实体/物料批次</t>
+        </is>
+      </c>
+      <c r="C70" s="11" t="inlineStr">
+        <is>
+          <t>删除化学式格式说明，只保留示例与即时元素/语法反馈</t>
+        </is>
+      </c>
+      <c r="D70" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-06用户界面复核</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="11" t="inlineStr">
+        <is>
+          <t>v4.0-alpha.9</t>
+        </is>
+      </c>
+      <c r="B71" s="11" t="inlineStr">
+        <is>
+          <t>实体/物料批次</t>
+        </is>
+      </c>
+      <c r="C71" s="11" t="inlineStr">
+        <is>
+          <t>供应商“其他”改为明确的新增供应商与名称输入；供应商规格或等级改为产品等级（标签原文），说明资料未标注时留空</t>
+        </is>
+      </c>
+      <c r="D71" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-06用户界面复核</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="inlineStr">
+        <is>
+          <t>v4.0-alpha.12</t>
+        </is>
+      </c>
+      <c r="B72" s="11" t="inlineStr">
+        <is>
+          <t>§5 生长条件</t>
+        </is>
+      </c>
+      <c r="C72" s="11" t="inlineStr">
+        <is>
+          <t>统一实验时间零点与有效生长窗口；补齐气体批次、流量来源、绝对压力、受控降温速率、实际外场参数和多条异常事件，并自动覆盖生长后的实验过程</t>
+        </is>
+      </c>
+      <c r="D72" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-06用户界面复核</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="11" t="inlineStr">
+        <is>
+          <t>v4.0-alpha.13</t>
+        </is>
+      </c>
+      <c r="B73" s="11" t="inlineStr">
+        <is>
+          <t>§5 生长条件</t>
+        </is>
+      </c>
+      <c r="C73" s="11" t="inlineStr">
+        <is>
+          <t>将容易误解为管理制度的“压力制度/压力体系”统一改为“反应压力条件”，数据字段与校验规则不变</t>
+        </is>
+      </c>
+      <c r="D73" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-07用户界面复核</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="11" t="inlineStr">
+        <is>
+          <t>v4.0-alpha.14</t>
+        </is>
+      </c>
+      <c r="B74" s="11" t="inlineStr">
+        <is>
+          <t>§5 生长条件</t>
+        </is>
+      </c>
+      <c r="C74" s="11" t="inlineStr">
+        <is>
+          <t>改为按实际操作和持续时间录入，系统自动生成系统准备、升温与预处理、反应、反应后处理和降温时间轴；气体优先选择使用阶段，仅自定义时填写起止时间</t>
+        </is>
+      </c>
+      <c r="D74" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-07用户界面复核</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="11" t="inlineStr">
+        <is>
+          <t>v4.0-alpha.15</t>
+        </is>
+      </c>
+      <c r="B75" s="11" t="inlineStr">
+        <is>
+          <t>§5 生长条件</t>
+        </is>
+      </c>
+      <c r="C75" s="11" t="inlineStr">
+        <is>
+          <t>删除缺乏统一文献定义且无法直接观测的反应计时起点、反应开始前用时、反应时长及重复的反应后处理；实际过程由温度步骤、气体时段、系统准备、压力与降温记录</t>
+        </is>
+      </c>
+      <c r="D75" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-07用户界面复核与原始论文核对</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="inlineStr">
+        <is>
           <t>R0</t>
         </is>
       </c>
-      <c r="B67" s="11" t="inlineStr">
+      <c r="B76" s="11" t="inlineStr">
         <is>
           <t>硬必填核心(29项，含条件必填)</t>
         </is>
       </c>
-      <c r="C67" s="11" t="inlineStr">
+      <c r="C76" s="11" t="inlineStr">
         <is>
           <t>v3.18删除炉次内重复的前驱体化学式R0；物料身份仍由必填的批次版本快照冻结；其余R0定义不变</t>
         </is>
       </c>
-      <c r="D67" s="11" t="inlineStr">
+      <c r="D76" s="11" t="inlineStr">
         <is>
           <t>必填集</t>
         </is>

</xml_diff>

<commit_message>
fix: harden characterization traceability
</commit_message>
<xml_diff>
--- a/docs/standard/字段草案-v3.xlsx
+++ b/docs/standard/字段草案-v3.xlsx
@@ -10330,7 +10330,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D79"/>
+  <dimension ref="A1:D80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11986,20 +11986,42 @@
     <row r="79">
       <c r="A79" s="11" t="inlineStr">
         <is>
+          <t>v4.0-alpha.19</t>
+        </is>
+      </c>
+      <c r="B79" s="11" t="inlineStr">
+        <is>
+          <t>表征科学属性</t>
+        </is>
+      </c>
+      <c r="C79" s="11" t="inlineStr">
+        <is>
+          <t>PropertyValue 补齐数值/文本表示类型与物理范围，并统一后端和前端的单一源校验</t>
+        </is>
+      </c>
+      <c r="D79" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-31表征全链路独立审查</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="inlineStr">
+        <is>
           <t>R0</t>
         </is>
       </c>
-      <c r="B79" s="11" t="inlineStr">
+      <c r="B80" s="11" t="inlineStr">
         <is>
           <t>最小可复现核心(27项，含条件必填)</t>
         </is>
       </c>
-      <c r="C79" s="11" t="inlineStr">
+      <c r="C80" s="11" t="inlineStr">
         <is>
           <t>过程R0以温度/气体/压力通道和降温条件为准；不再要求人工划分反应阶段或反应时长</t>
         </is>
       </c>
-      <c r="D79" s="11" t="inlineStr">
+      <c r="D80" s="11" t="inlineStr">
         <is>
           <t>必填集</t>
         </is>

</xml_diff>

<commit_message>
fix: improve preparation form usability
</commit_message>
<xml_diff>
--- a/docs/standard/字段草案-v3.xlsx
+++ b/docs/standard/字段草案-v3.xlsx
@@ -1668,12 +1668,12 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>目标性能</t>
+          <t>实验目标</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>应用导向的目标性能（写清想要什么性能 + 打算用什么方法/判据衡量）</t>
+          <t>本炉希望获得的目标性能或需要验证的研究目标</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
@@ -2624,7 +2624,7 @@
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>当前炉管的累计清洗或更换次数，以及本次实验是最近一次清洗或更换后的第几次使用</t>
+          <t>当前炉管的清洗或更换累计次数，以及本次是最近一次清洗或更换后的第几炉</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -2659,7 +2659,7 @@
       </c>
       <c r="J42" s="11" t="inlineStr">
         <is>
-          <t>每炉手填；清洗或更换炉管后累计次数加1，本次使用序号从1重新累计</t>
+          <t>界面分为“清洗或更换累计次数”和“清洗或更换后第几炉”；清洗或更换炉管后累计次数加1，本次使用序号从1重新累计</t>
         </is>
       </c>
       <c r="K42" s="11" t="inlineStr"/>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
-          <t>处理方式</t>
+          <t>使用前处理</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
@@ -3549,7 +3549,7 @@
       </c>
       <c r="B60" s="11" t="inlineStr">
         <is>
-          <t>前驱体放置位置</t>
+          <t>热电偶相对位置</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="B61" s="11" t="inlineStr">
         <is>
-          <t>前驱体加热温区</t>
+          <t>前驱体所在温区</t>
         </is>
       </c>
       <c r="C61" s="11" t="inlineStr">
@@ -4308,7 +4308,7 @@
       </c>
       <c r="B75" s="11" t="inlineStr">
         <is>
-          <t>预处理（有序步骤）</t>
+          <t>衬底处理（有序步骤）</t>
         </is>
       </c>
       <c r="C75" s="11" t="inlineStr">
@@ -4471,7 +4471,7 @@
       </c>
       <c r="B78" s="11" t="inlineStr">
         <is>
-          <t>所在温区与热电偶距离</t>
+          <t>所在温区与热电偶相对位置</t>
         </is>
       </c>
       <c r="C78" s="11" t="inlineStr">
@@ -4749,22 +4749,22 @@
       </c>
       <c r="B84" s="11" t="inlineStr">
         <is>
-          <t>异常情况确认</t>
+          <t>本炉发生过异常</t>
         </is>
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>明确确认本炉是否发生异常，避免将未填写误判为无异常</t>
+          <t>勾选表示本炉发生过异常，未勾选表示本炉无异常</t>
         </is>
       </c>
       <c r="D84" s="11" t="inlineStr">
         <is>
-          <t>下拉</t>
+          <t>勾选框</t>
         </is>
       </c>
       <c r="E84" s="11" t="inlineStr">
         <is>
-          <t>是/否</t>
+          <t>勾选=是；未勾选=否</t>
         </is>
       </c>
       <c r="F84" s="11" t="inlineStr">
@@ -4779,17 +4779,17 @@
       </c>
       <c r="H84" s="11" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>未勾选</t>
         </is>
       </c>
       <c r="I84" s="11" t="inlineStr">
         <is>
-          <t>2026-09-01用户试填反馈</t>
+          <t>2026-09-01用户试填反馈·2026-09-02交互复核</t>
         </is>
       </c>
       <c r="J84" s="11" t="inlineStr">
         <is>
-          <t>选择是时至少填写一条过程异常事件</t>
+          <t>勾选时至少填写一条过程异常事件</t>
         </is>
       </c>
       <c r="K84" s="11" t="inlineStr"/>
@@ -4802,7 +4802,7 @@
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>反应压力类别</t>
+          <t>反应压力条件</t>
         </is>
       </c>
       <c r="C85" s="11" t="inlineStr">
@@ -5124,7 +5124,7 @@
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
-          <t>预处理操作</t>
+          <t>实验前准备操作</t>
         </is>
       </c>
       <c r="C91" s="11" t="inlineStr">
@@ -10436,7 +10436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D82"/>
+  <dimension ref="A1:D84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -12158,20 +12158,64 @@
     <row r="82">
       <c r="A82" s="11" t="inlineStr">
         <is>
+          <t>v4.0-alpha.22</t>
+        </is>
+      </c>
+      <c r="B82" s="11" t="inlineStr">
+        <is>
+          <t>§3/§5 生长条件与装置履历</t>
+        </is>
+      </c>
+      <c r="C82" s="11" t="inlineStr">
+        <is>
+          <t>生长条件按实验前准备、温度、气体、反应压力、降温和异常分区；温度步骤移除待判断与初始温度伪时长；异常改为勾选框，并缩短温区和炉管履历文案</t>
+        </is>
+      </c>
+      <c r="D82" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-02用户界面复核</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="11" t="inlineStr">
+        <is>
+          <t>v4.0-alpha.23</t>
+        </is>
+      </c>
+      <c r="B83" s="11" t="inlineStr">
+        <is>
+          <t>§1b/§3/§4/§5 制备记录填写体验</t>
+        </is>
+      </c>
+      <c r="C83" s="11" t="inlineStr">
+        <is>
+          <t>缩短晶体结构、实验目标、热电偶相对位置、使用前处理、衬底处理和压力条件文案；明确必填空状态与提交检查，并减少气体首段录入步骤</t>
+        </is>
+      </c>
+      <c r="D83" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-02用户全流程复核</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="11" t="inlineStr">
+        <is>
           <t>R0</t>
         </is>
       </c>
-      <c r="B82" s="11" t="inlineStr">
+      <c r="B84" s="11" t="inlineStr">
         <is>
           <t>最小可复现核心(27项，含条件必填)</t>
         </is>
       </c>
-      <c r="C82" s="11" t="inlineStr">
+      <c r="C84" s="11" t="inlineStr">
         <is>
           <t>过程R0以温度/气体/压力通道和降温条件为准；不再要求人工划分反应阶段或反应时长</t>
         </is>
       </c>
-      <c r="D82" s="11" t="inlineStr">
+      <c r="D84" s="11" t="inlineStr">
         <is>
           <t>必填集</t>
         </is>

</xml_diff>

<commit_message>
fix: refine preparation and characterization records
</commit_message>
<xml_diff>
--- a/docs/standard/字段草案-v3.xlsx
+++ b/docs/standard/字段草案-v3.xlsx
@@ -5129,7 +5129,7 @@
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>选填的实验前操作；每项记录实际持续时间，气路置换引用实际气瓶版本</t>
+          <t>选填的实验前操作；抽真空优先记录终点绝对压力，无压力读数时记录持续时间，气路置换引用实际气瓶版本</t>
         </is>
       </c>
       <c r="D91" s="11" t="inlineStr">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="E91" s="11" t="inlineStr">
         <is>
-          <t>{operation_type: pump_down|gas_exchange|leak_check|other, duration_min, cycle_count?, gas_sources?: [{material_lot_id, material_lot_version, snapshot?}], other_name?}</t>
+          <t>{operation_type: pump_down|gas_exchange|leak_check|other, duration_min?, target_absolute_pressure_Pa?, cycle_count?, gas_sources?: [{material_lot_id, material_lot_version, snapshot?}], other_name?}</t>
         </is>
       </c>
       <c r="F91" s="11" t="inlineStr">
@@ -5154,7 +5154,7 @@
       </c>
       <c r="H91" s="11" t="inlineStr">
         <is>
-          <t>[{operation_type: gas_exchange, duration_min: 10, cycle_count: 3, gas_sources: [{material_lot_id: UUID, material_lot_version: 2}]}]</t>
+          <t>[{operation_type: pump_down, target_absolute_pressure_Pa: 10}, {operation_type: gas_exchange, duration_min: 10, cycle_count: 3, gas_sources: [{material_lot_id: UUID, material_lot_version: 2}]}]</t>
         </is>
       </c>
       <c r="I91" s="11" t="inlineStr">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="J91" s="11" t="inlineStr">
         <is>
-          <t>置换可引用一瓶预混气或多瓶现场混合气；固定组成仅在气瓶版本登记</t>
+          <t>抽真空的 target_absolute_pressure_Pa 与 duration_min 至少填一项，已填项必须大于 0；置换可引用一瓶预混气或多瓶现场混合气，固定组成仅在气瓶版本登记</t>
         </is>
       </c>
       <c r="K91" s="11" t="inlineStr"/>
@@ -10436,7 +10436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D84"/>
+  <dimension ref="A1:D85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -12202,20 +12202,42 @@
     <row r="84">
       <c r="A84" s="11" t="inlineStr">
         <is>
+          <t>v4.0-alpha.24</t>
+        </is>
+      </c>
+      <c r="B84" s="11" t="inlineStr">
+        <is>
+          <t>§5 实验前准备</t>
+        </is>
+      </c>
+      <c r="C84" s="11" t="inlineStr">
+        <is>
+          <t>抽真空优先记录终点绝对压力；有压力读数时持续时间改为选填，无压力读数时持续时间必填</t>
+        </is>
+      </c>
+      <c r="D84" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-02用户实验前准备复核</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="11" t="inlineStr">
+        <is>
           <t>R0</t>
         </is>
       </c>
-      <c r="B84" s="11" t="inlineStr">
+      <c r="B85" s="11" t="inlineStr">
         <is>
           <t>最小可复现核心(27项，含条件必填)</t>
         </is>
       </c>
-      <c r="C84" s="11" t="inlineStr">
+      <c r="C85" s="11" t="inlineStr">
         <is>
           <t>过程R0以温度/气体/压力通道和降温条件为准；不再要求人工划分反应阶段或反应时长</t>
         </is>
       </c>
-      <c r="D84" s="11" t="inlineStr">
+      <c r="D85" s="11" t="inlineStr">
         <is>
           <t>必填集</t>
         </is>

</xml_diff>

<commit_message>
[frontend] fix audit findings and integrate instrument presets
Refresh dependent caches after writes, preserve failed upload cleanup for safe
retry, fix static asset caching and 404 responses, and follow the active toast
theme. Remove unused workspaces and the target editor import cycle.

Include the alpha.44 instrument preset and shared field changes required by
this implementation. Generate a lazy payload validator from the field-source
schema and pin the existing dependency versions.

Validation: frontend 426 tests, typecheck, lint, format and build passed;
backend full suite 498 passed and 4 PostgreSQL-only checks skipped;
PostgreSQL scientific API regression 122 passed; field-source/xlsx checks,
nginx responses and Chromium/FastAPI/PostgreSQL integration passed.
</commit_message>
<xml_diff>
--- a/docs/standard/字段草案-v3.xlsx
+++ b/docs/standard/字段草案-v3.xlsx
@@ -11018,7 +11018,7 @@
       </c>
       <c r="B70" s="11" t="inlineStr">
         <is>
-          <t>关键固定配置</t>
+          <t>其他固定配置说明</t>
         </is>
       </c>
       <c r="C70" s="11" t="inlineStr">
@@ -11086,7 +11086,7 @@
       </c>
       <c r="E71" s="11" t="inlineStr">
         <is>
-          <t>[{code,configuration}]；code=other 时 configuration.method_names 为方法名称列表</t>
+          <t>[{code,configuration}]；configuration.presets=[{name,conditions}]；code=other 时另有 method_names</t>
         </is>
       </c>
       <c r="F71" s="11" t="inlineStr">
@@ -11111,7 +11111,7 @@
       </c>
       <c r="J71" s="11" t="inlineStr">
         <is>
-          <t>UI 使用多选；其他展开方法名称列表，可逐项添加/删除，名称非空且去首尾空白后长度 1–128、忽略大小写不重复；仍以一个 other 能力行保存多个名称，不改变仪器版本和能力代码唯一约束。</t>
+          <t>每种方法可维护最多50套命名预设；名称去空白后1–128字符，同方法内忽略大小写唯一。conditions复用该方法结构化采集字段、单位及校验，至少一项，不要求整套测试必填参数齐全。表征主动选用后复制为本次实际条件，可调整；预设修改产生新仪器版本，不改历史记录。其他方法继续通过method_names具名；保留历史configuration内容。</t>
         </is>
       </c>
       <c r="K71" s="11" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: complete PL characterization metadata workflow
</commit_message>
<xml_diff>
--- a/docs/standard/字段草案-v3.xlsx
+++ b/docs/standard/字段草案-v3.xlsx
@@ -4535,7 +4535,7 @@
       </c>
       <c r="E79" s="11" t="inlineStr">
         <is>
-          <t>{type: 溶剂清洗|氮气吹干|退火|等离子体|紫外臭氧联合处理|其他, other_name?, parameters: 溶剂清洗[solvent: 丙酮|异丙醇|乙醇|甲醇|去离子水|其他, solvent_other?, cleaning_method: 超声|浸泡|冲洗|擦拭|其他, cleaning_method_other?, duration_min?, temperature_C?, wiping_material?, equipment_name?, ultrasonic_frequency_kHz?, ultrasonic_power_W?]；紫外臭氧联合处理[duration_min, mode?, equipment_name?, source_distance_mm?, atmosphere?, temperature_C?, wavelength_nm?, irradiance_mW_cm2?, ozone_concentration_ppm?, gas_flow_sccm?]；其余为对应参数对象}</t>
+          <t>{type: 溶剂清洗|氮气吹干|退火|等离子体|紫外/臭氧表面处理|其他, other_name?, parameters: 溶剂清洗[solvent: 丙酮|异丙醇|乙醇|甲醇|去离子水|其他, solvent_other?, cleaning_method: 超声|浸泡|冲洗|擦拭|其他, cleaning_method_other?, duration_min?, temperature_C?, wiping_material?, equipment_name?, ultrasonic_frequency_kHz?, ultrasonic_power_W?]；紫外/臭氧表面处理[duration_min, mode?, equipment_name?, source_distance_mm?, atmosphere?, temperature_C?, wavelength_nm?, irradiance_mW_cm2?, ozone_concentration_ppm?, gas_flow_sccm?]；其余为对应参数对象}</t>
         </is>
       </c>
       <c r="F79" s="11" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J79" s="11" t="inlineStr">
         <is>
-          <t>有序可重复且每步只记录一种溶剂；连续使用多种溶剂应拆成多步。溶剂清洗选择超声或浸泡时duration_min必填，冲洗或擦拭时选填；紫外臭氧联合处理duration_min必填，模式可明确为联合/仅紫外/仅臭氧；其余参数按实际设置或资料选填，擦拭材料仅擦拭适用，超声频率/功率仅超声适用；等离子体展开power_W、gas_species、pressure_Pa和duration_min；其他步骤必须具名并至少填写一个参数</t>
+          <t>有序可重复且每步只记录一种溶剂；连续使用多种溶剂应拆成多步。溶剂清洗选择超声或浸泡时duration_min必填，冲洗或擦拭时选填；紫外/臭氧表面处理duration_min必填，模式可明确为联合/仅紫外/仅臭氧；其余参数按实际设置或资料选填，擦拭材料仅擦拭适用，超声频率/功率仅超声适用；等离子体展开power_W、gas_species、pressure_Pa和duration_min；其他步骤必须具名并至少填写一个参数</t>
         </is>
       </c>
       <c r="K79" s="11" t="inlineStr"/>

</xml_diff>